<commit_message>
Upload security config, function: register/login/logout
</commit_message>
<xml_diff>
--- a/document/02_c_LAB301x_VN_v0.01_OPPM.xlsx
+++ b/document/02_c_LAB301x_VN_v0.01_OPPM.xlsx
@@ -5,10 +5,10 @@
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thanh\Downloads\FU\LAB\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thanh\Downloads\FU\LAB\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80B07904-DB50-45DA-B960-E390D9D15ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06FE7CA6-4E23-453E-B5DC-EBB3217AD792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="69">
   <si>
     <t>Sub-Objectives</t>
   </si>
@@ -227,60 +227,6 @@
     <t>Requirement Analysis &amp; SRS</t>
   </si>
   <si>
-    <t>User Registration Function (UI + Backend + Integration + Testing)</t>
-  </si>
-  <si>
-    <t>User Authentication (Login/Logout) Function</t>
-  </si>
-  <si>
-    <t>User Profile Management Function</t>
-  </si>
-  <si>
-    <t>Password Recovery Function</t>
-  </si>
-  <si>
-    <t>Job Listing Function (View Job List)</t>
-  </si>
-  <si>
-    <t>Job Search Function</t>
-  </si>
-  <si>
-    <t>Job Detail Viewing Function</t>
-  </si>
-  <si>
-    <t>Job Application Function (Core Feature)</t>
-  </si>
-  <si>
-    <t>Applied Jobs Management Function</t>
-  </si>
-  <si>
-    <t>Company Listing Function</t>
-  </si>
-  <si>
-    <t>Company Detail Viewing Function</t>
-  </si>
-  <si>
-    <t>Admin User Management Function</t>
-  </si>
-  <si>
-    <t>Admin Job Management Function</t>
-  </si>
-  <si>
-    <t>Admin Company Management Function</t>
-  </si>
-  <si>
-    <t>Admin Application Management Function</t>
-  </si>
-  <si>
-    <t>16. UI Development &amp; Integration (Bootstrap + Thymeleaf)</t>
-  </si>
-  <si>
-    <t>17. System Testing &amp; Bug Fixing</t>
-  </si>
-  <si>
-    <t>18. Deployment &amp; Documentation</t>
-  </si>
-  <si>
     <t>Project Manager: Nguyen Van Hau</t>
   </si>
   <si>
@@ -325,6 +271,66 @@
   <si>
     <t>3. UI không đồng nhất → Dùng Bootstrap template</t>
   </si>
+  <si>
+    <t>Spring Security config</t>
+  </si>
+  <si>
+    <t>UC1: Register</t>
+  </si>
+  <si>
+    <t>UC2: Login</t>
+  </si>
+  <si>
+    <t>UC3: Logout</t>
+  </si>
+  <si>
+    <t>UC4: Update Profile</t>
+  </si>
+  <si>
+    <t>UC5: Manager Skills of User</t>
+  </si>
+  <si>
+    <t>UC6: Show job list</t>
+  </si>
+  <si>
+    <t>UC7: Search Job</t>
+  </si>
+  <si>
+    <t>UC8: Filter Job</t>
+  </si>
+  <si>
+    <t>UC9: CUD Job</t>
+  </si>
+  <si>
+    <t>UC10: Create Skill of Job</t>
+  </si>
+  <si>
+    <t>UC11: CU Company</t>
+  </si>
+  <si>
+    <t>UC12: Apply Job (upload CV)</t>
+  </si>
+  <si>
+    <t>UC13: Create cover letter</t>
+  </si>
+  <si>
+    <t>UC14: Show list of applied</t>
+  </si>
+  <si>
+    <t>UC15: Show status applied</t>
+  </si>
+  <si>
+    <t>UC16: Show Applied of Job</t>
+  </si>
+  <si>
+    <t>UC17: Update status of applied</t>
+  </si>
+  <si>
+    <t>File upload config</t>
+  </si>
+  <si>
+    <t>Unit test</t>
+  </si>
 </sst>
 </file>
 
@@ -338,7 +344,7 @@
     <numFmt numFmtId="168" formatCode="_(&quot;$&quot;* #"/>
     <numFmt numFmtId="169" formatCode="dd\-mm\-yyyy;@"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -514,6 +520,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="163"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -1500,7 +1512,7 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="226">
+  <cellXfs count="227">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyProtection="1"/>
@@ -2266,6 +2278,10 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="51" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -3687,6 +3703,182 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>36</xdr:col>
+      <xdr:colOff>676373</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>68106</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2A002ECD-0479-B4CD-00A5-18A1C0820234}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12586447" y="1165412"/>
+          <a:ext cx="8735644" cy="2219635"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>39339</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>156629</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Picture 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{42D3CD07-53A1-35CE-0168-B42389AD838C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12586447" y="3532094"/>
+          <a:ext cx="8878539" cy="2200582"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>191760</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>62511</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="Picture 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E84B7B78-96A5-1423-9B59-DAC4ACCBFAD2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12586447" y="5844988"/>
+          <a:ext cx="9030960" cy="2276793"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>36</xdr:col>
+      <xdr:colOff>733531</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>20495</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="Picture 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3EB83D02-AAB0-0C3F-63C6-C3D3FBBB5DAE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12586447" y="8229600"/>
+          <a:ext cx="8792802" cy="2324424"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -4046,12 +4238,12 @@
       <c r="H2" s="7"/>
       <c r="I2" s="8"/>
       <c r="J2" s="150" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="K2" s="8"/>
       <c r="L2" s="8"/>
       <c r="M2" s="149" t="s">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="N2" s="149"/>
       <c r="O2" s="9"/>
@@ -4065,7 +4257,7 @@
       <c r="W2" s="11"/>
       <c r="X2" s="12"/>
       <c r="Y2" s="137" t="s">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="AA2" s="13"/>
       <c r="AB2" s="14"/>
@@ -4081,7 +4273,7 @@
       <c r="H3" s="16"/>
       <c r="I3" s="17"/>
       <c r="J3" s="190" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="K3" s="191"/>
       <c r="L3" s="191"/>
@@ -4200,7 +4392,7 @@
       <c r="L6" s="29"/>
       <c r="M6" s="29"/>
       <c r="N6" s="161" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="O6" s="30"/>
       <c r="P6" s="30"/>
@@ -4237,7 +4429,7 @@
       <c r="L7" s="140"/>
       <c r="M7" s="140"/>
       <c r="N7" s="162" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="O7" s="41"/>
       <c r="P7" s="41"/>
@@ -4278,7 +4470,9 @@
       <c r="P8" s="37"/>
       <c r="Q8" s="41"/>
       <c r="R8" s="37"/>
-      <c r="S8" s="37"/>
+      <c r="S8" s="124" t="s">
+        <v>10</v>
+      </c>
       <c r="T8" s="37"/>
       <c r="U8" s="37"/>
       <c r="V8" s="37"/>
@@ -4313,7 +4507,9 @@
       <c r="P9" s="39"/>
       <c r="Q9" s="41"/>
       <c r="R9" s="40"/>
-      <c r="S9" s="37"/>
+      <c r="S9" s="124" t="s">
+        <v>10</v>
+      </c>
       <c r="T9" s="37"/>
       <c r="U9" s="37"/>
       <c r="V9" s="37"/>
@@ -4326,7 +4522,7 @@
       <c r="AB9" s="32"/>
       <c r="AC9" s="32"/>
     </row>
-    <row r="10" spans="1:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B10" s="26" t="s">
         <v>11</v>
       </c>
@@ -4342,8 +4538,8 @@
       <c r="J10" s="127">
         <v>5</v>
       </c>
-      <c r="K10" t="s">
-        <v>34</v>
+      <c r="K10" s="35" t="s">
+        <v>49</v>
       </c>
       <c r="L10" s="35"/>
       <c r="M10" s="35"/>
@@ -4352,7 +4548,9 @@
       <c r="P10" s="39"/>
       <c r="Q10" s="41"/>
       <c r="R10" s="40"/>
-      <c r="S10" s="37"/>
+      <c r="S10" s="124" t="s">
+        <v>10</v>
+      </c>
       <c r="T10" s="37"/>
       <c r="U10" s="37"/>
       <c r="V10" s="37"/>
@@ -4367,7 +4565,7 @@
       <c r="AB10" s="32"/>
       <c r="AC10" s="32"/>
     </row>
-    <row r="11" spans="1:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B11" s="26" t="s">
         <v>11</v>
       </c>
@@ -4383,8 +4581,8 @@
       <c r="J11" s="127">
         <v>6</v>
       </c>
-      <c r="K11" t="s">
-        <v>35</v>
+      <c r="K11" s="35" t="s">
+        <v>50</v>
       </c>
       <c r="L11" s="35"/>
       <c r="M11" s="35"/>
@@ -4393,7 +4591,9 @@
       <c r="P11" s="41"/>
       <c r="Q11" s="41"/>
       <c r="R11" s="41"/>
-      <c r="S11" s="37"/>
+      <c r="S11" s="124" t="s">
+        <v>10</v>
+      </c>
       <c r="T11" s="37"/>
       <c r="U11" s="37"/>
       <c r="V11" s="37"/>
@@ -4408,7 +4608,7 @@
       <c r="AB11" s="32"/>
       <c r="AC11" s="32"/>
     </row>
-    <row r="12" spans="1:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B12" s="26" t="s">
         <v>11</v>
       </c>
@@ -4422,8 +4622,8 @@
       <c r="J12" s="127">
         <v>7</v>
       </c>
-      <c r="K12" t="s">
-        <v>36</v>
+      <c r="K12" s="35" t="s">
+        <v>51</v>
       </c>
       <c r="L12" s="35"/>
       <c r="M12" s="35"/>
@@ -4432,7 +4632,9 @@
       <c r="P12" s="37"/>
       <c r="Q12" s="41"/>
       <c r="R12" s="37"/>
-      <c r="S12" s="37"/>
+      <c r="S12" s="124" t="s">
+        <v>10</v>
+      </c>
       <c r="T12" s="37"/>
       <c r="U12" s="37"/>
       <c r="V12" s="37"/>
@@ -4447,7 +4649,7 @@
       <c r="AB12" s="32"/>
       <c r="AC12" s="32"/>
     </row>
-    <row r="13" spans="1:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B13" s="26" t="s">
         <v>11</v>
       </c>
@@ -4461,8 +4663,8 @@
       <c r="J13" s="127">
         <v>8</v>
       </c>
-      <c r="K13" t="s">
-        <v>37</v>
+      <c r="K13" s="35" t="s">
+        <v>52</v>
       </c>
       <c r="L13" s="35"/>
       <c r="M13" s="35"/>
@@ -4471,7 +4673,9 @@
       <c r="P13" s="37"/>
       <c r="Q13" s="41"/>
       <c r="R13" s="37"/>
-      <c r="S13" s="37"/>
+      <c r="S13" s="124" t="s">
+        <v>10</v>
+      </c>
       <c r="T13" s="37"/>
       <c r="U13" s="37"/>
       <c r="V13" s="37"/>
@@ -4482,7 +4686,7 @@
       <c r="AB13" s="32"/>
       <c r="AC13" s="32"/>
     </row>
-    <row r="14" spans="1:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B14" s="26"/>
       <c r="C14" s="33"/>
       <c r="D14" s="173" t="s">
@@ -4496,8 +4700,8 @@
       <c r="J14" s="127">
         <v>9</v>
       </c>
-      <c r="K14" t="s">
-        <v>38</v>
+      <c r="K14" s="35" t="s">
+        <v>53</v>
       </c>
       <c r="L14" s="35"/>
       <c r="M14" s="35"/>
@@ -4517,7 +4721,7 @@
       <c r="AB14" s="32"/>
       <c r="AC14" s="32"/>
     </row>
-    <row r="15" spans="1:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B15" s="26"/>
       <c r="C15" s="33"/>
       <c r="D15" s="173" t="s">
@@ -4531,8 +4735,8 @@
       <c r="J15" s="127">
         <v>10</v>
       </c>
-      <c r="K15" t="s">
-        <v>39</v>
+      <c r="K15" s="35" t="s">
+        <v>54</v>
       </c>
       <c r="L15" s="35"/>
       <c r="M15" s="35"/>
@@ -4552,7 +4756,7 @@
       <c r="AB15" s="32"/>
       <c r="AC15" s="32"/>
     </row>
-    <row r="16" spans="1:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B16" s="26"/>
       <c r="C16" s="33"/>
       <c r="D16" s="173" t="s">
@@ -4566,8 +4770,8 @@
       <c r="J16" s="127">
         <v>11</v>
       </c>
-      <c r="K16" t="s">
-        <v>40</v>
+      <c r="K16" s="35" t="s">
+        <v>55</v>
       </c>
       <c r="L16" s="35"/>
       <c r="M16" s="35"/>
@@ -4587,7 +4791,7 @@
       <c r="AB16" s="32"/>
       <c r="AC16" s="32"/>
     </row>
-    <row r="17" spans="2:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B17" s="26"/>
       <c r="C17" s="33"/>
       <c r="D17" s="173" t="s">
@@ -4601,8 +4805,8 @@
       <c r="J17" s="127">
         <v>12</v>
       </c>
-      <c r="K17" t="s">
-        <v>41</v>
+      <c r="K17" s="35" t="s">
+        <v>56</v>
       </c>
       <c r="L17" s="35"/>
       <c r="M17" s="35"/>
@@ -4622,7 +4826,7 @@
       <c r="AB17" s="32"/>
       <c r="AC17" s="32"/>
     </row>
-    <row r="18" spans="2:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B18" s="26" t="s">
         <v>11</v>
       </c>
@@ -4638,8 +4842,8 @@
       <c r="J18" s="127">
         <v>13</v>
       </c>
-      <c r="K18" t="s">
-        <v>42</v>
+      <c r="K18" s="35" t="s">
+        <v>57</v>
       </c>
       <c r="L18" s="35"/>
       <c r="M18" s="35"/>
@@ -4659,7 +4863,7 @@
       <c r="AB18" s="32"/>
       <c r="AC18" s="32"/>
     </row>
-    <row r="19" spans="2:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B19" s="26"/>
       <c r="C19" s="33"/>
       <c r="D19" s="173"/>
@@ -4673,8 +4877,8 @@
       <c r="J19" s="127">
         <v>14</v>
       </c>
-      <c r="K19" t="s">
-        <v>43</v>
+      <c r="K19" s="35" t="s">
+        <v>58</v>
       </c>
       <c r="L19" s="35"/>
       <c r="M19" s="35"/>
@@ -4694,7 +4898,7 @@
       <c r="AB19" s="32"/>
       <c r="AC19" s="32"/>
     </row>
-    <row r="20" spans="2:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B20" s="26"/>
       <c r="C20" s="33"/>
       <c r="D20" s="173"/>
@@ -4708,8 +4912,8 @@
       <c r="J20" s="127">
         <v>15</v>
       </c>
-      <c r="K20" t="s">
-        <v>44</v>
+      <c r="K20" s="35" t="s">
+        <v>59</v>
       </c>
       <c r="L20" s="35"/>
       <c r="M20" s="35"/>
@@ -4729,7 +4933,7 @@
       <c r="AB20" s="32"/>
       <c r="AC20" s="32"/>
     </row>
-    <row r="21" spans="2:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B21" s="26"/>
       <c r="C21" s="33"/>
       <c r="D21" s="173"/>
@@ -4743,8 +4947,8 @@
       <c r="J21" s="127">
         <v>16</v>
       </c>
-      <c r="K21" t="s">
-        <v>45</v>
+      <c r="K21" s="35" t="s">
+        <v>60</v>
       </c>
       <c r="L21" s="35"/>
       <c r="M21" s="35"/>
@@ -4764,7 +4968,7 @@
       <c r="AB21" s="32"/>
       <c r="AC21" s="32"/>
     </row>
-    <row r="22" spans="2:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B22" s="26"/>
       <c r="C22" s="33"/>
       <c r="D22" s="173"/>
@@ -4778,8 +4982,8 @@
       <c r="J22" s="127">
         <v>17</v>
       </c>
-      <c r="K22" t="s">
-        <v>46</v>
+      <c r="K22" s="35" t="s">
+        <v>61</v>
       </c>
       <c r="L22" s="35"/>
       <c r="M22" s="35"/>
@@ -4799,7 +5003,7 @@
       <c r="AB22" s="32"/>
       <c r="AC22" s="32"/>
     </row>
-    <row r="23" spans="2:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B23" s="26"/>
       <c r="C23" s="33"/>
       <c r="D23" s="173"/>
@@ -4813,8 +5017,8 @@
       <c r="J23" s="127">
         <v>18</v>
       </c>
-      <c r="K23" t="s">
-        <v>47</v>
+      <c r="K23" s="35" t="s">
+        <v>62</v>
       </c>
       <c r="L23" s="35"/>
       <c r="M23" s="35"/>
@@ -4834,7 +5038,7 @@
       <c r="AB23" s="32"/>
       <c r="AC23" s="32"/>
     </row>
-    <row r="24" spans="2:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B24" s="26"/>
       <c r="C24" s="33"/>
       <c r="D24" s="173"/>
@@ -4848,8 +5052,8 @@
       <c r="J24" s="127">
         <v>19</v>
       </c>
-      <c r="K24" t="s">
-        <v>48</v>
+      <c r="K24" s="35" t="s">
+        <v>63</v>
       </c>
       <c r="L24" s="35"/>
       <c r="M24" s="35"/>
@@ -4869,7 +5073,7 @@
       <c r="AB24" s="32"/>
       <c r="AC24" s="32"/>
     </row>
-    <row r="25" spans="2:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B25" s="26"/>
       <c r="C25" s="33"/>
       <c r="D25" s="173"/>
@@ -4881,8 +5085,8 @@
       <c r="J25" s="127">
         <v>20</v>
       </c>
-      <c r="K25" t="s">
-        <v>49</v>
+      <c r="K25" s="35" t="s">
+        <v>64</v>
       </c>
       <c r="L25" s="35"/>
       <c r="M25" s="35"/>
@@ -4902,7 +5106,7 @@
       <c r="AB25" s="32"/>
       <c r="AC25" s="32"/>
     </row>
-    <row r="26" spans="2:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B26" s="26"/>
       <c r="C26" s="33"/>
       <c r="D26" s="173"/>
@@ -4914,8 +5118,8 @@
       <c r="J26" s="127">
         <v>21</v>
       </c>
-      <c r="K26" t="s">
-        <v>50</v>
+      <c r="K26" s="35" t="s">
+        <v>65</v>
       </c>
       <c r="L26" s="35"/>
       <c r="M26" s="42"/>
@@ -4935,7 +5139,7 @@
       <c r="AB26" s="32"/>
       <c r="AC26" s="32"/>
     </row>
-    <row r="27" spans="2:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B27" s="26"/>
       <c r="C27" s="33"/>
       <c r="D27" s="173"/>
@@ -4947,8 +5151,8 @@
       <c r="J27" s="127">
         <v>22</v>
       </c>
-      <c r="K27" t="s">
-        <v>51</v>
+      <c r="K27" s="35" t="s">
+        <v>66</v>
       </c>
       <c r="L27" s="35"/>
       <c r="M27" s="42"/>
@@ -4980,7 +5184,9 @@
       <c r="J28" s="127">
         <v>23</v>
       </c>
-      <c r="K28" s="128"/>
+      <c r="K28" s="226" t="s">
+        <v>67</v>
+      </c>
       <c r="L28" s="42"/>
       <c r="M28" s="42"/>
       <c r="N28" s="36"/>
@@ -5010,7 +5216,9 @@
       <c r="J29" s="143">
         <v>24</v>
       </c>
-      <c r="K29" s="128"/>
+      <c r="K29" s="226" t="s">
+        <v>68</v>
+      </c>
       <c r="L29" s="144"/>
       <c r="M29" s="144"/>
       <c r="N29" s="145"/>
@@ -5646,7 +5854,7 @@
       <c r="V51" s="57"/>
       <c r="W51" s="166"/>
       <c r="X51" s="214" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="Y51" s="215"/>
       <c r="AA51" s="31"/>
@@ -5666,7 +5874,7 @@
         <v>1</v>
       </c>
       <c r="K52" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="L52" s="61"/>
       <c r="M52" s="61"/>
@@ -5699,7 +5907,7 @@
         <v>2</v>
       </c>
       <c r="K53" t="s">
-        <v>65</v>
+        <v>47</v>
       </c>
       <c r="L53" s="61"/>
       <c r="M53" s="61"/>
@@ -5732,7 +5940,7 @@
         <v>3</v>
       </c>
       <c r="K54" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="L54" s="42"/>
       <c r="M54" s="42"/>
@@ -5900,7 +6108,7 @@
       <c r="C59" s="89"/>
       <c r="D59" s="178"/>
       <c r="E59" s="187" t="s">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="F59" s="178"/>
       <c r="G59" s="178"/>
@@ -5929,23 +6137,23 @@
     </row>
     <row r="60" spans="1:29" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="204" t="s">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="C60" s="204" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="D60" s="185" t="s">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="E60" s="188"/>
       <c r="F60" s="185" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="G60" s="185" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="H60" s="185" t="s">
-        <v>63</v>
+        <v>45</v>
       </c>
       <c r="I60" s="185"/>
       <c r="J60" s="101"/>
@@ -6676,7 +6884,7 @@
       <formula>"L"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O6:W7 N8:W19 N20:Q27">
+  <conditionalFormatting sqref="O6:W7 N14:W19 N20:Q27 N8:R13 T8:W13">
     <cfRule type="cellIs" dxfId="14" priority="49" stopIfTrue="1" operator="equal">
       <formula>"S"</formula>
     </cfRule>

</xml_diff>

<commit_message>
UC: Show list Job
</commit_message>
<xml_diff>
--- a/document/02_c_LAB301x_VN_v0.01_OPPM.xlsx
+++ b/document/02_c_LAB301x_VN_v0.01_OPPM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thanh\Downloads\FU\LAB\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06FE7CA6-4E23-453E-B5DC-EBB3217AD792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A94DE849-20D3-4492-89B1-B10B490A6BB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="69">
   <si>
     <t>Sub-Objectives</t>
   </si>
@@ -2131,6 +2131,10 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="66" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90"/>
       <protection locked="0"/>
@@ -2278,10 +2282,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="51" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -4272,24 +4272,24 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
       <c r="I3" s="17"/>
-      <c r="J3" s="190" t="s">
+      <c r="J3" s="191" t="s">
         <v>38</v>
       </c>
-      <c r="K3" s="191"/>
-      <c r="L3" s="191"/>
-      <c r="M3" s="191"/>
-      <c r="N3" s="191"/>
-      <c r="O3" s="191"/>
-      <c r="P3" s="191"/>
-      <c r="Q3" s="191"/>
-      <c r="R3" s="191"/>
-      <c r="S3" s="191"/>
-      <c r="T3" s="191"/>
-      <c r="U3" s="191"/>
-      <c r="V3" s="191"/>
-      <c r="W3" s="191"/>
-      <c r="X3" s="191"/>
-      <c r="Y3" s="192"/>
+      <c r="K3" s="192"/>
+      <c r="L3" s="192"/>
+      <c r="M3" s="192"/>
+      <c r="N3" s="192"/>
+      <c r="O3" s="192"/>
+      <c r="P3" s="192"/>
+      <c r="Q3" s="192"/>
+      <c r="R3" s="192"/>
+      <c r="S3" s="192"/>
+      <c r="T3" s="192"/>
+      <c r="U3" s="192"/>
+      <c r="V3" s="192"/>
+      <c r="W3" s="192"/>
+      <c r="X3" s="192"/>
+      <c r="Y3" s="193"/>
       <c r="AA3" s="13"/>
       <c r="AB3" s="14"/>
       <c r="AC3" s="14"/>
@@ -4303,59 +4303,59 @@
       <c r="G4" s="20"/>
       <c r="H4" s="20"/>
       <c r="I4" s="20"/>
-      <c r="J4" s="193"/>
-      <c r="K4" s="194"/>
-      <c r="L4" s="194"/>
-      <c r="M4" s="194"/>
-      <c r="N4" s="194"/>
-      <c r="O4" s="194"/>
-      <c r="P4" s="194"/>
-      <c r="Q4" s="194"/>
-      <c r="R4" s="194"/>
-      <c r="S4" s="194"/>
-      <c r="T4" s="194"/>
-      <c r="U4" s="194"/>
-      <c r="V4" s="194"/>
-      <c r="W4" s="194"/>
-      <c r="X4" s="194"/>
-      <c r="Y4" s="195"/>
+      <c r="J4" s="194"/>
+      <c r="K4" s="195"/>
+      <c r="L4" s="195"/>
+      <c r="M4" s="195"/>
+      <c r="N4" s="195"/>
+      <c r="O4" s="195"/>
+      <c r="P4" s="195"/>
+      <c r="Q4" s="195"/>
+      <c r="R4" s="195"/>
+      <c r="S4" s="195"/>
+      <c r="T4" s="195"/>
+      <c r="U4" s="195"/>
+      <c r="V4" s="195"/>
+      <c r="W4" s="195"/>
+      <c r="X4" s="195"/>
+      <c r="Y4" s="196"/>
       <c r="AA4" s="21"/>
       <c r="AB4" s="22"/>
       <c r="AC4" s="22"/>
     </row>
     <row r="5" spans="1:29" s="1" customFormat="1" ht="26.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="196" t="s">
+      <c r="B5" s="197" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="197"/>
-      <c r="D5" s="197"/>
-      <c r="E5" s="197"/>
-      <c r="F5" s="197"/>
-      <c r="G5" s="197"/>
-      <c r="H5" s="197"/>
-      <c r="I5" s="198"/>
+      <c r="C5" s="198"/>
+      <c r="D5" s="198"/>
+      <c r="E5" s="198"/>
+      <c r="F5" s="198"/>
+      <c r="G5" s="198"/>
+      <c r="H5" s="198"/>
+      <c r="I5" s="199"/>
       <c r="J5" s="168"/>
       <c r="K5" s="169" t="s">
         <v>1</v>
       </c>
       <c r="L5" s="170"/>
       <c r="M5" s="170"/>
-      <c r="N5" s="199" t="s">
+      <c r="N5" s="200" t="s">
         <v>2</v>
       </c>
-      <c r="O5" s="200"/>
-      <c r="P5" s="200"/>
-      <c r="Q5" s="200"/>
-      <c r="R5" s="200"/>
-      <c r="S5" s="200"/>
-      <c r="T5" s="200"/>
-      <c r="U5" s="200"/>
-      <c r="V5" s="200"/>
-      <c r="W5" s="201"/>
-      <c r="X5" s="202" t="s">
+      <c r="O5" s="201"/>
+      <c r="P5" s="201"/>
+      <c r="Q5" s="201"/>
+      <c r="R5" s="201"/>
+      <c r="S5" s="201"/>
+      <c r="T5" s="201"/>
+      <c r="U5" s="201"/>
+      <c r="V5" s="201"/>
+      <c r="W5" s="202"/>
+      <c r="X5" s="203" t="s">
         <v>3</v>
       </c>
-      <c r="Y5" s="203"/>
+      <c r="Y5" s="204"/>
       <c r="AA5" s="23"/>
       <c r="AB5" s="24"/>
       <c r="AC5" s="24"/>
@@ -4710,8 +4710,10 @@
       <c r="P14" s="37"/>
       <c r="Q14" s="37"/>
       <c r="R14" s="37"/>
-      <c r="S14" s="37"/>
-      <c r="T14" s="37"/>
+      <c r="S14" s="124"/>
+      <c r="T14" s="124" t="s">
+        <v>10</v>
+      </c>
       <c r="U14" s="37"/>
       <c r="V14" s="37"/>
       <c r="W14" s="39"/>
@@ -4745,8 +4747,10 @@
       <c r="P15" s="37"/>
       <c r="Q15" s="37"/>
       <c r="R15" s="37"/>
-      <c r="S15" s="37"/>
-      <c r="T15" s="37"/>
+      <c r="S15" s="124"/>
+      <c r="T15" s="124" t="s">
+        <v>10</v>
+      </c>
       <c r="U15" s="37"/>
       <c r="V15" s="37"/>
       <c r="W15" s="39"/>
@@ -4784,7 +4788,9 @@
       <c r="T16" s="37"/>
       <c r="U16" s="37"/>
       <c r="V16" s="37"/>
-      <c r="W16" s="39"/>
+      <c r="W16" s="39" t="s">
+        <v>10</v>
+      </c>
       <c r="X16" s="130"/>
       <c r="Y16" s="129"/>
       <c r="AA16" s="31"/>
@@ -4819,7 +4825,9 @@
       <c r="T17" s="37"/>
       <c r="U17" s="37"/>
       <c r="V17" s="37"/>
-      <c r="W17" s="39"/>
+      <c r="W17" s="39" t="s">
+        <v>10</v>
+      </c>
       <c r="X17" s="130"/>
       <c r="Y17" s="155"/>
       <c r="AA17" s="31"/>
@@ -4856,7 +4864,9 @@
       <c r="T18" s="37"/>
       <c r="U18" s="37"/>
       <c r="V18" s="37"/>
-      <c r="W18" s="39"/>
+      <c r="W18" s="39" t="s">
+        <v>10</v>
+      </c>
       <c r="X18" s="130"/>
       <c r="Y18" s="129"/>
       <c r="AA18" s="31"/>
@@ -5184,7 +5194,7 @@
       <c r="J28" s="127">
         <v>23</v>
       </c>
-      <c r="K28" s="226" t="s">
+      <c r="K28" s="185" t="s">
         <v>67</v>
       </c>
       <c r="L28" s="42"/>
@@ -5216,7 +5226,7 @@
       <c r="J29" s="143">
         <v>24</v>
       </c>
-      <c r="K29" s="226" t="s">
+      <c r="K29" s="185" t="s">
         <v>68</v>
       </c>
       <c r="L29" s="144"/>
@@ -5853,10 +5863,10 @@
       <c r="U51" s="57"/>
       <c r="V51" s="57"/>
       <c r="W51" s="166"/>
-      <c r="X51" s="214" t="s">
+      <c r="X51" s="215" t="s">
         <v>37</v>
       </c>
-      <c r="Y51" s="215"/>
+      <c r="Y51" s="216"/>
       <c r="AA51" s="31"/>
       <c r="AB51" s="32"/>
       <c r="AC51" s="32"/>
@@ -6107,7 +6117,7 @@
       <c r="B59" s="88"/>
       <c r="C59" s="89"/>
       <c r="D59" s="178"/>
-      <c r="E59" s="187" t="s">
+      <c r="E59" s="188" t="s">
         <v>42</v>
       </c>
       <c r="F59" s="178"/>
@@ -6136,64 +6146,64 @@
       <c r="AC59" s="32"/>
     </row>
     <row r="60" spans="1:29" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="204" t="s">
+      <c r="B60" s="205" t="s">
         <v>39</v>
       </c>
-      <c r="C60" s="204" t="s">
+      <c r="C60" s="205" t="s">
         <v>40</v>
       </c>
-      <c r="D60" s="185" t="s">
+      <c r="D60" s="186" t="s">
         <v>41</v>
       </c>
-      <c r="E60" s="188"/>
-      <c r="F60" s="185" t="s">
+      <c r="E60" s="189"/>
+      <c r="F60" s="186" t="s">
         <v>43</v>
       </c>
-      <c r="G60" s="185" t="s">
+      <c r="G60" s="186" t="s">
         <v>44</v>
       </c>
-      <c r="H60" s="185" t="s">
+      <c r="H60" s="186" t="s">
         <v>45</v>
       </c>
-      <c r="I60" s="185"/>
+      <c r="I60" s="186"/>
       <c r="J60" s="101"/>
       <c r="K60" s="96"/>
       <c r="L60" s="97"/>
       <c r="M60" s="97"/>
-      <c r="N60" s="207">
+      <c r="N60" s="208">
         <v>46099</v>
       </c>
-      <c r="O60" s="207">
+      <c r="O60" s="208">
         <v>46100</v>
       </c>
-      <c r="P60" s="207">
+      <c r="P60" s="208">
         <v>46101</v>
       </c>
-      <c r="Q60" s="207">
+      <c r="Q60" s="208">
         <v>46102</v>
       </c>
-      <c r="R60" s="207">
+      <c r="R60" s="208">
         <v>46103</v>
       </c>
-      <c r="S60" s="207">
+      <c r="S60" s="208">
         <v>46104</v>
       </c>
-      <c r="T60" s="207">
+      <c r="T60" s="208">
         <v>46105</v>
       </c>
-      <c r="U60" s="207">
+      <c r="U60" s="208">
         <v>46106</v>
       </c>
-      <c r="V60" s="207">
+      <c r="V60" s="208">
         <v>46107</v>
       </c>
-      <c r="W60" s="207">
+      <c r="W60" s="208">
         <v>46108</v>
       </c>
-      <c r="X60" s="211" t="s">
+      <c r="X60" s="212" t="s">
         <v>18</v>
       </c>
-      <c r="Y60" s="223" t="s">
+      <c r="Y60" s="224" t="s">
         <v>19</v>
       </c>
       <c r="AA60" s="31"/>
@@ -6201,157 +6211,157 @@
       <c r="AC60" s="32"/>
     </row>
     <row r="61" spans="1:29" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="205"/>
-      <c r="C61" s="205"/>
-      <c r="D61" s="185"/>
-      <c r="E61" s="188"/>
-      <c r="F61" s="185"/>
-      <c r="G61" s="185"/>
-      <c r="H61" s="185"/>
-      <c r="I61" s="185"/>
+      <c r="B61" s="206"/>
+      <c r="C61" s="206"/>
+      <c r="D61" s="186"/>
+      <c r="E61" s="189"/>
+      <c r="F61" s="186"/>
+      <c r="G61" s="186"/>
+      <c r="H61" s="186"/>
+      <c r="I61" s="186"/>
       <c r="J61" s="101"/>
       <c r="K61" s="98"/>
       <c r="L61" s="97"/>
       <c r="M61" s="97"/>
-      <c r="N61" s="207"/>
-      <c r="O61" s="207"/>
-      <c r="P61" s="207"/>
-      <c r="Q61" s="207"/>
-      <c r="R61" s="207"/>
-      <c r="S61" s="207"/>
-      <c r="T61" s="207"/>
-      <c r="U61" s="207"/>
-      <c r="V61" s="207"/>
-      <c r="W61" s="207"/>
-      <c r="X61" s="212"/>
-      <c r="Y61" s="224"/>
+      <c r="N61" s="208"/>
+      <c r="O61" s="208"/>
+      <c r="P61" s="208"/>
+      <c r="Q61" s="208"/>
+      <c r="R61" s="208"/>
+      <c r="S61" s="208"/>
+      <c r="T61" s="208"/>
+      <c r="U61" s="208"/>
+      <c r="V61" s="208"/>
+      <c r="W61" s="208"/>
+      <c r="X61" s="213"/>
+      <c r="Y61" s="225"/>
       <c r="AA61" s="31"/>
       <c r="AB61" s="32"/>
       <c r="AC61" s="32"/>
     </row>
     <row r="62" spans="1:29" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B62" s="205"/>
-      <c r="C62" s="205"/>
-      <c r="D62" s="185"/>
-      <c r="E62" s="188"/>
-      <c r="F62" s="185"/>
-      <c r="G62" s="185"/>
-      <c r="H62" s="185"/>
-      <c r="I62" s="185"/>
+      <c r="B62" s="206"/>
+      <c r="C62" s="206"/>
+      <c r="D62" s="186"/>
+      <c r="E62" s="189"/>
+      <c r="F62" s="186"/>
+      <c r="G62" s="186"/>
+      <c r="H62" s="186"/>
+      <c r="I62" s="186"/>
       <c r="J62" s="101"/>
       <c r="K62" s="98"/>
       <c r="L62" s="97"/>
       <c r="M62" s="97"/>
-      <c r="N62" s="207"/>
-      <c r="O62" s="207"/>
-      <c r="P62" s="207"/>
-      <c r="Q62" s="207"/>
-      <c r="R62" s="207"/>
-      <c r="S62" s="207"/>
-      <c r="T62" s="207"/>
-      <c r="U62" s="207"/>
-      <c r="V62" s="207"/>
-      <c r="W62" s="207"/>
-      <c r="X62" s="212"/>
-      <c r="Y62" s="224"/>
+      <c r="N62" s="208"/>
+      <c r="O62" s="208"/>
+      <c r="P62" s="208"/>
+      <c r="Q62" s="208"/>
+      <c r="R62" s="208"/>
+      <c r="S62" s="208"/>
+      <c r="T62" s="208"/>
+      <c r="U62" s="208"/>
+      <c r="V62" s="208"/>
+      <c r="W62" s="208"/>
+      <c r="X62" s="213"/>
+      <c r="Y62" s="225"/>
       <c r="AA62" s="31"/>
       <c r="AB62" s="32"/>
       <c r="AC62" s="32"/>
     </row>
     <row r="63" spans="1:29" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B63" s="205"/>
-      <c r="C63" s="205"/>
-      <c r="D63" s="185"/>
-      <c r="E63" s="188"/>
-      <c r="F63" s="185"/>
-      <c r="G63" s="185"/>
-      <c r="H63" s="185"/>
-      <c r="I63" s="185"/>
+      <c r="B63" s="206"/>
+      <c r="C63" s="206"/>
+      <c r="D63" s="186"/>
+      <c r="E63" s="189"/>
+      <c r="F63" s="186"/>
+      <c r="G63" s="186"/>
+      <c r="H63" s="186"/>
+      <c r="I63" s="186"/>
       <c r="J63" s="101"/>
       <c r="K63" s="99"/>
       <c r="L63" s="97"/>
       <c r="M63" s="97"/>
-      <c r="N63" s="207"/>
-      <c r="O63" s="207"/>
-      <c r="P63" s="207"/>
-      <c r="Q63" s="207"/>
-      <c r="R63" s="207"/>
-      <c r="S63" s="207"/>
-      <c r="T63" s="207"/>
-      <c r="U63" s="207"/>
-      <c r="V63" s="207"/>
-      <c r="W63" s="207"/>
-      <c r="X63" s="212"/>
-      <c r="Y63" s="224"/>
+      <c r="N63" s="208"/>
+      <c r="O63" s="208"/>
+      <c r="P63" s="208"/>
+      <c r="Q63" s="208"/>
+      <c r="R63" s="208"/>
+      <c r="S63" s="208"/>
+      <c r="T63" s="208"/>
+      <c r="U63" s="208"/>
+      <c r="V63" s="208"/>
+      <c r="W63" s="208"/>
+      <c r="X63" s="213"/>
+      <c r="Y63" s="225"/>
       <c r="AB63" s="32"/>
       <c r="AC63" s="32"/>
     </row>
     <row r="64" spans="1:29" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B64" s="205"/>
-      <c r="C64" s="205"/>
-      <c r="D64" s="185"/>
-      <c r="E64" s="188"/>
-      <c r="F64" s="185"/>
-      <c r="G64" s="185"/>
-      <c r="H64" s="185"/>
-      <c r="I64" s="185"/>
+      <c r="B64" s="206"/>
+      <c r="C64" s="206"/>
+      <c r="D64" s="186"/>
+      <c r="E64" s="189"/>
+      <c r="F64" s="186"/>
+      <c r="G64" s="186"/>
+      <c r="H64" s="186"/>
+      <c r="I64" s="186"/>
       <c r="J64" s="101"/>
       <c r="K64" s="96"/>
       <c r="L64" s="97"/>
       <c r="M64" s="97"/>
-      <c r="N64" s="207"/>
-      <c r="O64" s="207"/>
-      <c r="P64" s="207"/>
-      <c r="Q64" s="207"/>
-      <c r="R64" s="207"/>
-      <c r="S64" s="207"/>
-      <c r="T64" s="207"/>
-      <c r="U64" s="207"/>
-      <c r="V64" s="207"/>
-      <c r="W64" s="207"/>
-      <c r="X64" s="212"/>
-      <c r="Y64" s="224"/>
+      <c r="N64" s="208"/>
+      <c r="O64" s="208"/>
+      <c r="P64" s="208"/>
+      <c r="Q64" s="208"/>
+      <c r="R64" s="208"/>
+      <c r="S64" s="208"/>
+      <c r="T64" s="208"/>
+      <c r="U64" s="208"/>
+      <c r="V64" s="208"/>
+      <c r="W64" s="208"/>
+      <c r="X64" s="213"/>
+      <c r="Y64" s="225"/>
       <c r="AB64" s="32"/>
       <c r="AC64" s="32"/>
     </row>
     <row r="65" spans="2:29" ht="12.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B65" s="205"/>
-      <c r="C65" s="205"/>
-      <c r="D65" s="185"/>
-      <c r="E65" s="188"/>
-      <c r="F65" s="185"/>
-      <c r="G65" s="185"/>
-      <c r="H65" s="185"/>
-      <c r="I65" s="185"/>
+      <c r="B65" s="206"/>
+      <c r="C65" s="206"/>
+      <c r="D65" s="186"/>
+      <c r="E65" s="189"/>
+      <c r="F65" s="186"/>
+      <c r="G65" s="186"/>
+      <c r="H65" s="186"/>
+      <c r="I65" s="186"/>
       <c r="J65" s="101"/>
       <c r="K65" s="100"/>
       <c r="L65" s="97"/>
       <c r="M65" s="97"/>
-      <c r="N65" s="208"/>
-      <c r="O65" s="208"/>
-      <c r="P65" s="208"/>
-      <c r="Q65" s="208"/>
-      <c r="R65" s="208"/>
-      <c r="S65" s="208"/>
-      <c r="T65" s="208"/>
-      <c r="U65" s="208"/>
-      <c r="V65" s="208"/>
-      <c r="W65" s="208"/>
-      <c r="X65" s="213"/>
-      <c r="Y65" s="225"/>
+      <c r="N65" s="209"/>
+      <c r="O65" s="209"/>
+      <c r="P65" s="209"/>
+      <c r="Q65" s="209"/>
+      <c r="R65" s="209"/>
+      <c r="S65" s="209"/>
+      <c r="T65" s="209"/>
+      <c r="U65" s="209"/>
+      <c r="V65" s="209"/>
+      <c r="W65" s="209"/>
+      <c r="X65" s="214"/>
+      <c r="Y65" s="226"/>
       <c r="AA65" s="23"/>
       <c r="AB65" s="23"/>
       <c r="AC65" s="23"/>
     </row>
     <row r="66" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="205"/>
-      <c r="C66" s="205"/>
-      <c r="D66" s="185"/>
-      <c r="E66" s="188"/>
-      <c r="F66" s="185"/>
-      <c r="G66" s="185"/>
-      <c r="H66" s="185"/>
-      <c r="I66" s="185"/>
+      <c r="B66" s="206"/>
+      <c r="C66" s="206"/>
+      <c r="D66" s="186"/>
+      <c r="E66" s="189"/>
+      <c r="F66" s="186"/>
+      <c r="G66" s="186"/>
+      <c r="H66" s="186"/>
+      <c r="I66" s="186"/>
       <c r="J66" s="101"/>
       <c r="K66" s="100"/>
       <c r="L66" s="100"/>
@@ -6369,20 +6379,20 @@
       <c r="X66" s="103"/>
       <c r="Y66" s="104"/>
       <c r="AA66" s="23"/>
-      <c r="AB66" s="216" t="s">
+      <c r="AB66" s="217" t="s">
         <v>6</v>
       </c>
-      <c r="AC66" s="216"/>
+      <c r="AC66" s="217"/>
     </row>
     <row r="67" spans="2:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B67" s="205"/>
-      <c r="C67" s="205"/>
-      <c r="D67" s="185"/>
-      <c r="E67" s="188"/>
-      <c r="F67" s="185"/>
-      <c r="G67" s="185"/>
-      <c r="H67" s="185"/>
-      <c r="I67" s="185"/>
+      <c r="B67" s="206"/>
+      <c r="C67" s="206"/>
+      <c r="D67" s="186"/>
+      <c r="E67" s="189"/>
+      <c r="F67" s="186"/>
+      <c r="G67" s="186"/>
+      <c r="H67" s="186"/>
+      <c r="I67" s="186"/>
       <c r="J67" s="105"/>
       <c r="K67" s="100"/>
       <c r="L67" s="98"/>
@@ -6410,14 +6420,14 @@
       </c>
     </row>
     <row r="68" spans="2:29" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B68" s="205"/>
-      <c r="C68" s="205"/>
-      <c r="D68" s="185"/>
-      <c r="E68" s="188"/>
-      <c r="F68" s="185"/>
-      <c r="G68" s="185"/>
-      <c r="H68" s="185"/>
-      <c r="I68" s="185"/>
+      <c r="B68" s="206"/>
+      <c r="C68" s="206"/>
+      <c r="D68" s="186"/>
+      <c r="E68" s="189"/>
+      <c r="F68" s="186"/>
+      <c r="G68" s="186"/>
+      <c r="H68" s="186"/>
+      <c r="I68" s="186"/>
       <c r="J68" s="101"/>
       <c r="K68" s="96"/>
       <c r="L68" s="98"/>
@@ -6441,14 +6451,14 @@
       <c r="AC68" s="111"/>
     </row>
     <row r="69" spans="2:29" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B69" s="205"/>
-      <c r="C69" s="205"/>
-      <c r="D69" s="185"/>
-      <c r="E69" s="188"/>
-      <c r="F69" s="185"/>
-      <c r="G69" s="185"/>
-      <c r="H69" s="185"/>
-      <c r="I69" s="185"/>
+      <c r="B69" s="206"/>
+      <c r="C69" s="206"/>
+      <c r="D69" s="186"/>
+      <c r="E69" s="189"/>
+      <c r="F69" s="186"/>
+      <c r="G69" s="186"/>
+      <c r="H69" s="186"/>
+      <c r="I69" s="186"/>
       <c r="J69" s="101"/>
       <c r="K69" s="96"/>
       <c r="L69" s="98"/>
@@ -6472,14 +6482,14 @@
       <c r="AC69" s="113"/>
     </row>
     <row r="70" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B70" s="205"/>
-      <c r="C70" s="205"/>
-      <c r="D70" s="185"/>
-      <c r="E70" s="188"/>
-      <c r="F70" s="185"/>
-      <c r="G70" s="185"/>
-      <c r="H70" s="185"/>
-      <c r="I70" s="185"/>
+      <c r="B70" s="206"/>
+      <c r="C70" s="206"/>
+      <c r="D70" s="186"/>
+      <c r="E70" s="189"/>
+      <c r="F70" s="186"/>
+      <c r="G70" s="186"/>
+      <c r="H70" s="186"/>
+      <c r="I70" s="186"/>
       <c r="J70" s="101"/>
       <c r="K70" s="96"/>
       <c r="L70" s="96"/>
@@ -6503,14 +6513,14 @@
       <c r="AC70" s="111"/>
     </row>
     <row r="71" spans="2:29" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B71" s="205"/>
-      <c r="C71" s="205"/>
-      <c r="D71" s="185"/>
-      <c r="E71" s="188"/>
-      <c r="F71" s="185"/>
-      <c r="G71" s="185"/>
-      <c r="H71" s="185"/>
-      <c r="I71" s="185"/>
+      <c r="B71" s="206"/>
+      <c r="C71" s="206"/>
+      <c r="D71" s="186"/>
+      <c r="E71" s="189"/>
+      <c r="F71" s="186"/>
+      <c r="G71" s="186"/>
+      <c r="H71" s="186"/>
+      <c r="I71" s="186"/>
       <c r="J71" s="101"/>
       <c r="K71" s="114"/>
       <c r="L71" s="101"/>
@@ -6531,14 +6541,14 @@
       <c r="AB71" s="115"/>
     </row>
     <row r="72" spans="2:29" ht="15.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B72" s="205"/>
-      <c r="C72" s="205"/>
-      <c r="D72" s="185"/>
-      <c r="E72" s="188"/>
-      <c r="F72" s="185"/>
-      <c r="G72" s="185"/>
-      <c r="H72" s="185"/>
-      <c r="I72" s="185"/>
+      <c r="B72" s="206"/>
+      <c r="C72" s="206"/>
+      <c r="D72" s="186"/>
+      <c r="E72" s="189"/>
+      <c r="F72" s="186"/>
+      <c r="G72" s="186"/>
+      <c r="H72" s="186"/>
+      <c r="I72" s="186"/>
       <c r="J72" s="117"/>
       <c r="K72" s="116"/>
       <c r="L72" s="117"/>
@@ -6559,108 +6569,108 @@
       <c r="AC72" s="115"/>
     </row>
     <row r="73" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B73" s="205"/>
-      <c r="C73" s="205"/>
-      <c r="D73" s="185"/>
-      <c r="E73" s="188"/>
-      <c r="F73" s="185"/>
-      <c r="G73" s="185"/>
-      <c r="H73" s="185"/>
-      <c r="I73" s="185"/>
-      <c r="J73" s="217"/>
-      <c r="K73" s="217"/>
-      <c r="L73" s="217"/>
-      <c r="M73" s="217"/>
-      <c r="N73" s="217"/>
-      <c r="O73" s="217"/>
-      <c r="P73" s="217"/>
-      <c r="Q73" s="217"/>
-      <c r="R73" s="217"/>
-      <c r="S73" s="217"/>
-      <c r="T73" s="217"/>
-      <c r="U73" s="217"/>
-      <c r="V73" s="217"/>
-      <c r="W73" s="217"/>
-      <c r="X73" s="217"/>
-      <c r="Y73" s="218"/>
+      <c r="B73" s="206"/>
+      <c r="C73" s="206"/>
+      <c r="D73" s="186"/>
+      <c r="E73" s="189"/>
+      <c r="F73" s="186"/>
+      <c r="G73" s="186"/>
+      <c r="H73" s="186"/>
+      <c r="I73" s="186"/>
+      <c r="J73" s="218"/>
+      <c r="K73" s="218"/>
+      <c r="L73" s="218"/>
+      <c r="M73" s="218"/>
+      <c r="N73" s="218"/>
+      <c r="O73" s="218"/>
+      <c r="P73" s="218"/>
+      <c r="Q73" s="218"/>
+      <c r="R73" s="218"/>
+      <c r="S73" s="218"/>
+      <c r="T73" s="218"/>
+      <c r="U73" s="218"/>
+      <c r="V73" s="218"/>
+      <c r="W73" s="218"/>
+      <c r="X73" s="218"/>
+      <c r="Y73" s="219"/>
     </row>
     <row r="74" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B74" s="205"/>
-      <c r="C74" s="205"/>
-      <c r="D74" s="185"/>
-      <c r="E74" s="188"/>
-      <c r="F74" s="185"/>
-      <c r="G74" s="185"/>
-      <c r="H74" s="185"/>
-      <c r="I74" s="185"/>
-      <c r="J74" s="219"/>
-      <c r="K74" s="219"/>
-      <c r="L74" s="219"/>
-      <c r="M74" s="219"/>
-      <c r="N74" s="219"/>
-      <c r="O74" s="219"/>
-      <c r="P74" s="219"/>
-      <c r="Q74" s="219"/>
-      <c r="R74" s="219"/>
-      <c r="S74" s="219"/>
-      <c r="T74" s="219"/>
-      <c r="U74" s="219"/>
-      <c r="V74" s="219"/>
-      <c r="W74" s="219"/>
-      <c r="X74" s="219"/>
-      <c r="Y74" s="220"/>
+      <c r="B74" s="206"/>
+      <c r="C74" s="206"/>
+      <c r="D74" s="186"/>
+      <c r="E74" s="189"/>
+      <c r="F74" s="186"/>
+      <c r="G74" s="186"/>
+      <c r="H74" s="186"/>
+      <c r="I74" s="186"/>
+      <c r="J74" s="220"/>
+      <c r="K74" s="220"/>
+      <c r="L74" s="220"/>
+      <c r="M74" s="220"/>
+      <c r="N74" s="220"/>
+      <c r="O74" s="220"/>
+      <c r="P74" s="220"/>
+      <c r="Q74" s="220"/>
+      <c r="R74" s="220"/>
+      <c r="S74" s="220"/>
+      <c r="T74" s="220"/>
+      <c r="U74" s="220"/>
+      <c r="V74" s="220"/>
+      <c r="W74" s="220"/>
+      <c r="X74" s="220"/>
+      <c r="Y74" s="221"/>
     </row>
     <row r="75" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B75" s="205"/>
-      <c r="C75" s="205"/>
-      <c r="D75" s="185"/>
-      <c r="E75" s="188"/>
-      <c r="F75" s="185"/>
-      <c r="G75" s="185"/>
-      <c r="H75" s="185"/>
-      <c r="I75" s="185"/>
-      <c r="J75" s="219"/>
-      <c r="K75" s="219"/>
-      <c r="L75" s="219"/>
-      <c r="M75" s="219"/>
-      <c r="N75" s="219"/>
-      <c r="O75" s="219"/>
-      <c r="P75" s="219"/>
-      <c r="Q75" s="219"/>
-      <c r="R75" s="219"/>
-      <c r="S75" s="219"/>
-      <c r="T75" s="219"/>
-      <c r="U75" s="219"/>
-      <c r="V75" s="219"/>
-      <c r="W75" s="219"/>
-      <c r="X75" s="219"/>
-      <c r="Y75" s="220"/>
+      <c r="B75" s="206"/>
+      <c r="C75" s="206"/>
+      <c r="D75" s="186"/>
+      <c r="E75" s="189"/>
+      <c r="F75" s="186"/>
+      <c r="G75" s="186"/>
+      <c r="H75" s="186"/>
+      <c r="I75" s="186"/>
+      <c r="J75" s="220"/>
+      <c r="K75" s="220"/>
+      <c r="L75" s="220"/>
+      <c r="M75" s="220"/>
+      <c r="N75" s="220"/>
+      <c r="O75" s="220"/>
+      <c r="P75" s="220"/>
+      <c r="Q75" s="220"/>
+      <c r="R75" s="220"/>
+      <c r="S75" s="220"/>
+      <c r="T75" s="220"/>
+      <c r="U75" s="220"/>
+      <c r="V75" s="220"/>
+      <c r="W75" s="220"/>
+      <c r="X75" s="220"/>
+      <c r="Y75" s="221"/>
     </row>
     <row r="76" spans="2:29" s="1" customFormat="1" ht="15.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B76" s="206"/>
-      <c r="C76" s="206"/>
-      <c r="D76" s="186"/>
-      <c r="E76" s="189"/>
-      <c r="F76" s="186"/>
-      <c r="G76" s="186"/>
-      <c r="H76" s="186"/>
-      <c r="I76" s="186"/>
-      <c r="J76" s="209"/>
-      <c r="K76" s="209"/>
-      <c r="L76" s="209"/>
-      <c r="M76" s="209"/>
-      <c r="N76" s="209"/>
-      <c r="O76" s="209"/>
-      <c r="P76" s="209"/>
-      <c r="Q76" s="209"/>
-      <c r="R76" s="209"/>
-      <c r="S76" s="209"/>
-      <c r="T76" s="209"/>
-      <c r="U76" s="209"/>
-      <c r="V76" s="209"/>
-      <c r="W76" s="209"/>
-      <c r="X76" s="209"/>
-      <c r="Y76" s="210"/>
+      <c r="B76" s="207"/>
+      <c r="C76" s="207"/>
+      <c r="D76" s="187"/>
+      <c r="E76" s="190"/>
+      <c r="F76" s="187"/>
+      <c r="G76" s="187"/>
+      <c r="H76" s="187"/>
+      <c r="I76" s="187"/>
+      <c r="J76" s="210"/>
+      <c r="K76" s="210"/>
+      <c r="L76" s="210"/>
+      <c r="M76" s="210"/>
+      <c r="N76" s="210"/>
+      <c r="O76" s="210"/>
+      <c r="P76" s="210"/>
+      <c r="Q76" s="210"/>
+      <c r="R76" s="210"/>
+      <c r="S76" s="210"/>
+      <c r="T76" s="210"/>
+      <c r="U76" s="210"/>
+      <c r="V76" s="210"/>
+      <c r="W76" s="210"/>
+      <c r="X76" s="210"/>
+      <c r="Y76" s="211"/>
       <c r="AA76" s="23"/>
       <c r="AB76" s="24"/>
       <c r="AC76" s="24"/>
@@ -6690,10 +6700,10 @@
       <c r="U78" s="131" t="s">
         <v>15</v>
       </c>
-      <c r="V78" s="221" t="s">
+      <c r="V78" s="222" t="s">
         <v>23</v>
       </c>
-      <c r="W78" s="222"/>
+      <c r="W78" s="223"/>
       <c r="Y78" s="123"/>
       <c r="Z78" s="123"/>
       <c r="AA78" s="123"/>
@@ -6722,10 +6732,10 @@
       <c r="U79" s="138" t="s">
         <v>16</v>
       </c>
-      <c r="V79" s="221" t="s">
+      <c r="V79" s="222" t="s">
         <v>24</v>
       </c>
-      <c r="W79" s="222"/>
+      <c r="W79" s="223"/>
       <c r="Y79" s="125"/>
       <c r="Z79" s="125"/>
       <c r="AA79" s="125"/>
@@ -6755,10 +6765,10 @@
       <c r="U80" s="146" t="s">
         <v>17</v>
       </c>
-      <c r="V80" s="221" t="s">
+      <c r="V80" s="222" t="s">
         <v>25</v>
       </c>
-      <c r="W80" s="222"/>
+      <c r="W80" s="223"/>
       <c r="Y80" s="121"/>
       <c r="Z80" s="121"/>
       <c r="AA80" s="121"/>
@@ -6884,7 +6894,7 @@
       <formula>"L"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O6:W7 N14:W19 N20:Q27 N8:R13 T8:W13">
+  <conditionalFormatting sqref="O6:W7 T8:W13 N8:R15 U14:W15 N20:Q27 N16:W19">
     <cfRule type="cellIs" dxfId="14" priority="49" stopIfTrue="1" operator="equal">
       <formula>"S"</formula>
     </cfRule>

</xml_diff>

<commit_message>
update create, update UC: 7
</commit_message>
<xml_diff>
--- a/document/02_c_LAB301x_VN_v0.01_OPPM.xlsx
+++ b/document/02_c_LAB301x_VN_v0.01_OPPM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thanh\Downloads\FU\LAB\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A94DE849-20D3-4492-89B1-B10B490A6BB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FC2F255-4FA4-4393-A6FD-ECD4F8F52FBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Start" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Start!$B$2:$Y$76</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Start!$B$2:$AD$76</definedName>
   </definedNames>
   <calcPr calcId="152511" iterate="1" iterateCount="10000" iterateDelta="1.0000000000000001E-5"/>
 </workbook>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="69">
   <si>
     <t>Sub-Objectives</t>
   </si>
@@ -583,7 +583,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="73">
+  <borders count="75">
     <border>
       <left/>
       <right/>
@@ -1501,6 +1501,30 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1512,7 +1536,7 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="227">
+  <cellXfs count="229">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyProtection="1"/>
@@ -2135,6 +2159,107 @@
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="56" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="49" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="51" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="63" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="56" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="56" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="49" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="66" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90"/>
       <protection locked="0"/>
@@ -2143,6 +2268,34 @@
       <alignment horizontal="center" vertical="top" textRotation="90"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="59" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="60" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="49" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="71" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="72" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90"/>
       <protection locked="0"/>
@@ -2155,132 +2308,11 @@
       <alignment horizontal="center" vertical="top" textRotation="90"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="56" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="56" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="49" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="56" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="73" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="49" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="59" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="60" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="49" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="71" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="72" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="63" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="51" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="74" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -2295,7 +2327,37 @@
     <cellStyle name="Normal_Project Matrix" xfId="1" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
     <cellStyle name="Normal_Project Matrix Collection II" xfId="2" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
   </cellStyles>
-  <dxfs count="23">
+  <dxfs count="26">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="mediumGray">
+          <fgColor indexed="10"/>
+          <bgColor indexed="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="mediumGray">
+          <fgColor indexed="42"/>
+          <bgColor indexed="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="mediumGray">
+          <fgColor indexed="43"/>
+          <bgColor indexed="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="mediumGray">
@@ -2569,7 +2631,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Start!$AB$67</c:f>
+              <c:f>Start!$AG$67</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2632,7 +2694,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Start!$AA$68:$AA$70</c:f>
+              <c:f>Start!$AF$68:$AF$70</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -2649,7 +2711,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Start!$AB$68:$AB$70</c:f>
+              <c:f>Start!$AG$68:$AG$70</c:f>
               <c:numCache>
                 <c:formatCode>_("$"* #</c:formatCode>
                 <c:ptCount val="3"/>
@@ -2719,7 +2781,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Start!$AA$68:$AA$70</c:f>
+              <c:f>Start!$AF$68:$AF$70</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -2736,7 +2798,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Start!$AC$68:$AC$70</c:f>
+              <c:f>Start!$AH$68:$AH$70</c:f>
               <c:numCache>
                 <c:formatCode>_("$"* #,##0.0"M";_("$"* \(#,##0.0"M"\);_("$"* "-"_);_(@_)</c:formatCode>
                 <c:ptCount val="3"/>
@@ -2953,7 +3015,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:noFill/>
             </a14:hiddenFill>
           </a:ext>
@@ -3007,7 +3069,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:noFill/>
             </a14:hiddenFill>
           </a:ext>
@@ -3280,7 +3342,7 @@
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
+      <xdr:col>29</xdr:col>
       <xdr:colOff>276225</xdr:colOff>
       <xdr:row>71</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
@@ -3363,14 +3425,14 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="3175">
+            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="3175">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -3429,7 +3491,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:noFill/>
             </a14:hiddenFill>
           </a:ext>
@@ -3483,7 +3545,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:noFill/>
             </a14:hiddenFill>
           </a:ext>
@@ -3537,7 +3599,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:noFill/>
             </a14:hiddenFill>
           </a:ext>
@@ -3644,13 +3706,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>28</xdr:col>
+      <xdr:col>33</xdr:col>
       <xdr:colOff>395817</xdr:colOff>
       <xdr:row>49</xdr:row>
       <xdr:rowOff>84666</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
+      <xdr:col>35</xdr:col>
       <xdr:colOff>156634</xdr:colOff>
       <xdr:row>56</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -3705,13 +3767,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>26</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>36</xdr:col>
+      <xdr:col>41</xdr:col>
       <xdr:colOff>676373</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>68106</xdr:rowOff>
@@ -3749,13 +3811,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>26</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>37</xdr:col>
+      <xdr:col>42</xdr:col>
       <xdr:colOff>39339</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>156629</xdr:rowOff>
@@ -3793,13 +3855,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>26</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>37</xdr:col>
+      <xdr:col>42</xdr:col>
       <xdr:colOff>191760</xdr:colOff>
       <xdr:row>42</xdr:row>
       <xdr:rowOff>62511</xdr:rowOff>
@@ -3837,13 +3899,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>26</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>43</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>36</xdr:col>
+      <xdr:col>41</xdr:col>
       <xdr:colOff>733531</xdr:colOff>
       <xdr:row>56</xdr:row>
       <xdr:rowOff>20495</xdr:rowOff>
@@ -4207,7 +4269,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AC84"/>
+  <dimension ref="A1:AH84"/>
   <sheetFormatPr defaultColWidth="10.19921875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" style="2" customWidth="1"/>
@@ -4215,20 +4277,20 @@
     <col min="11" max="11" width="21.19921875" style="2" customWidth="1"/>
     <col min="12" max="12" width="25" style="2" customWidth="1"/>
     <col min="13" max="13" width="11.296875" style="2" customWidth="1"/>
-    <col min="14" max="23" width="5.796875" style="2" customWidth="1"/>
-    <col min="24" max="24" width="4.796875" style="2" customWidth="1"/>
-    <col min="25" max="25" width="5.19921875" style="2" customWidth="1"/>
-    <col min="26" max="26" width="3" style="2" customWidth="1"/>
-    <col min="27" max="27" width="15.296875" style="3" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="9.19921875" style="4" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="9.69921875" style="4" bestFit="1" customWidth="1"/>
-    <col min="30" max="16384" width="10.19921875" style="2"/>
+    <col min="14" max="28" width="5.796875" style="2" customWidth="1"/>
+    <col min="29" max="29" width="4.796875" style="2" customWidth="1"/>
+    <col min="30" max="30" width="5.19921875" style="2" customWidth="1"/>
+    <col min="31" max="31" width="3" style="2" customWidth="1"/>
+    <col min="32" max="32" width="15.296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="9.19921875" style="4" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="9.69921875" style="4" bestFit="1" customWidth="1"/>
+    <col min="35" max="16384" width="10.19921875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:34" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
     </row>
-    <row r="2" spans="1:29" s="5" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:34" s="5" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="B2" s="6"/>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
@@ -4255,15 +4317,20 @@
       <c r="U2" s="11"/>
       <c r="V2" s="11"/>
       <c r="W2" s="11"/>
-      <c r="X2" s="12"/>
-      <c r="Y2" s="137" t="s">
+      <c r="X2" s="11"/>
+      <c r="Y2" s="11"/>
+      <c r="Z2" s="11"/>
+      <c r="AA2" s="11"/>
+      <c r="AB2" s="11"/>
+      <c r="AC2" s="12"/>
+      <c r="AD2" s="137" t="s">
         <v>36</v>
       </c>
-      <c r="AA2" s="13"/>
-      <c r="AB2" s="14"/>
-      <c r="AC2" s="14"/>
-    </row>
-    <row r="3" spans="1:29" s="5" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AF2" s="13"/>
+      <c r="AG2" s="14"/>
+      <c r="AH2" s="14"/>
+    </row>
+    <row r="3" spans="1:34" s="5" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="15"/>
       <c r="C3" s="16"/>
       <c r="D3" s="16"/>
@@ -4272,29 +4339,34 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
       <c r="I3" s="17"/>
-      <c r="J3" s="191" t="s">
+      <c r="J3" s="198" t="s">
         <v>38</v>
       </c>
-      <c r="K3" s="192"/>
-      <c r="L3" s="192"/>
-      <c r="M3" s="192"/>
-      <c r="N3" s="192"/>
-      <c r="O3" s="192"/>
-      <c r="P3" s="192"/>
-      <c r="Q3" s="192"/>
-      <c r="R3" s="192"/>
-      <c r="S3" s="192"/>
-      <c r="T3" s="192"/>
-      <c r="U3" s="192"/>
-      <c r="V3" s="192"/>
-      <c r="W3" s="192"/>
-      <c r="X3" s="192"/>
-      <c r="Y3" s="193"/>
-      <c r="AA3" s="13"/>
-      <c r="AB3" s="14"/>
-      <c r="AC3" s="14"/>
-    </row>
-    <row r="4" spans="1:29" s="18" customFormat="1" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K3" s="199"/>
+      <c r="L3" s="199"/>
+      <c r="M3" s="199"/>
+      <c r="N3" s="199"/>
+      <c r="O3" s="199"/>
+      <c r="P3" s="199"/>
+      <c r="Q3" s="199"/>
+      <c r="R3" s="199"/>
+      <c r="S3" s="199"/>
+      <c r="T3" s="199"/>
+      <c r="U3" s="199"/>
+      <c r="V3" s="199"/>
+      <c r="W3" s="199"/>
+      <c r="X3" s="199"/>
+      <c r="Y3" s="199"/>
+      <c r="Z3" s="199"/>
+      <c r="AA3" s="199"/>
+      <c r="AB3" s="199"/>
+      <c r="AC3" s="199"/>
+      <c r="AD3" s="200"/>
+      <c r="AF3" s="13"/>
+      <c r="AG3" s="14"/>
+      <c r="AH3" s="14"/>
+    </row>
+    <row r="4" spans="1:34" s="18" customFormat="1" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="19"/>
       <c r="C4" s="20"/>
       <c r="D4" s="20"/>
@@ -4303,64 +4375,74 @@
       <c r="G4" s="20"/>
       <c r="H4" s="20"/>
       <c r="I4" s="20"/>
-      <c r="J4" s="194"/>
-      <c r="K4" s="195"/>
-      <c r="L4" s="195"/>
-      <c r="M4" s="195"/>
-      <c r="N4" s="195"/>
-      <c r="O4" s="195"/>
-      <c r="P4" s="195"/>
-      <c r="Q4" s="195"/>
-      <c r="R4" s="195"/>
-      <c r="S4" s="195"/>
-      <c r="T4" s="195"/>
-      <c r="U4" s="195"/>
-      <c r="V4" s="195"/>
-      <c r="W4" s="195"/>
-      <c r="X4" s="195"/>
-      <c r="Y4" s="196"/>
-      <c r="AA4" s="21"/>
-      <c r="AB4" s="22"/>
-      <c r="AC4" s="22"/>
-    </row>
-    <row r="5" spans="1:29" s="1" customFormat="1" ht="26.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="197" t="s">
+      <c r="J4" s="201"/>
+      <c r="K4" s="202"/>
+      <c r="L4" s="202"/>
+      <c r="M4" s="202"/>
+      <c r="N4" s="202"/>
+      <c r="O4" s="202"/>
+      <c r="P4" s="202"/>
+      <c r="Q4" s="202"/>
+      <c r="R4" s="202"/>
+      <c r="S4" s="202"/>
+      <c r="T4" s="202"/>
+      <c r="U4" s="202"/>
+      <c r="V4" s="202"/>
+      <c r="W4" s="202"/>
+      <c r="X4" s="202"/>
+      <c r="Y4" s="202"/>
+      <c r="Z4" s="202"/>
+      <c r="AA4" s="202"/>
+      <c r="AB4" s="202"/>
+      <c r="AC4" s="202"/>
+      <c r="AD4" s="203"/>
+      <c r="AF4" s="21"/>
+      <c r="AG4" s="22"/>
+      <c r="AH4" s="22"/>
+    </row>
+    <row r="5" spans="1:34" s="1" customFormat="1" ht="26.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="204" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="198"/>
-      <c r="D5" s="198"/>
-      <c r="E5" s="198"/>
-      <c r="F5" s="198"/>
-      <c r="G5" s="198"/>
-      <c r="H5" s="198"/>
-      <c r="I5" s="199"/>
+      <c r="C5" s="205"/>
+      <c r="D5" s="205"/>
+      <c r="E5" s="205"/>
+      <c r="F5" s="205"/>
+      <c r="G5" s="205"/>
+      <c r="H5" s="205"/>
+      <c r="I5" s="206"/>
       <c r="J5" s="168"/>
       <c r="K5" s="169" t="s">
         <v>1</v>
       </c>
       <c r="L5" s="170"/>
       <c r="M5" s="170"/>
-      <c r="N5" s="200" t="s">
+      <c r="N5" s="207" t="s">
         <v>2</v>
       </c>
-      <c r="O5" s="201"/>
-      <c r="P5" s="201"/>
-      <c r="Q5" s="201"/>
-      <c r="R5" s="201"/>
-      <c r="S5" s="201"/>
-      <c r="T5" s="201"/>
-      <c r="U5" s="201"/>
-      <c r="V5" s="201"/>
-      <c r="W5" s="202"/>
-      <c r="X5" s="203" t="s">
+      <c r="O5" s="208"/>
+      <c r="P5" s="208"/>
+      <c r="Q5" s="208"/>
+      <c r="R5" s="208"/>
+      <c r="S5" s="208"/>
+      <c r="T5" s="208"/>
+      <c r="U5" s="208"/>
+      <c r="V5" s="208"/>
+      <c r="W5" s="209"/>
+      <c r="X5" s="209"/>
+      <c r="Y5" s="209"/>
+      <c r="Z5" s="209"/>
+      <c r="AA5" s="209"/>
+      <c r="AB5" s="209"/>
+      <c r="AC5" s="210" t="s">
         <v>3</v>
       </c>
-      <c r="Y5" s="204"/>
-      <c r="AA5" s="23"/>
-      <c r="AB5" s="24"/>
-      <c r="AC5" s="24"/>
-    </row>
-    <row r="6" spans="1:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="AD5" s="211"/>
+      <c r="AF5" s="23"/>
+      <c r="AG5" s="24"/>
+      <c r="AH5" s="24"/>
+    </row>
+    <row r="6" spans="1:34" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B6" s="26" t="s">
         <v>10</v>
       </c>
@@ -4403,15 +4485,20 @@
       <c r="U6" s="30"/>
       <c r="V6" s="30"/>
       <c r="W6" s="163"/>
-      <c r="X6" s="182" t="s">
+      <c r="X6" s="163"/>
+      <c r="Y6" s="163"/>
+      <c r="Z6" s="163"/>
+      <c r="AA6" s="163"/>
+      <c r="AB6" s="163"/>
+      <c r="AC6" s="182" t="s">
         <v>15</v>
       </c>
-      <c r="Y6" s="179"/>
-      <c r="AA6" s="31"/>
-      <c r="AB6" s="32"/>
-      <c r="AC6" s="32"/>
-    </row>
-    <row r="7" spans="1:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="AD6" s="179"/>
+      <c r="AF6" s="31"/>
+      <c r="AG6" s="32"/>
+      <c r="AH6" s="32"/>
+    </row>
+    <row r="7" spans="1:34" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B7" s="26"/>
       <c r="C7" s="59"/>
       <c r="D7" s="172"/>
@@ -4440,15 +4527,20 @@
       <c r="U7" s="41"/>
       <c r="V7" s="41"/>
       <c r="W7" s="164"/>
-      <c r="X7" s="183" t="s">
+      <c r="X7" s="164"/>
+      <c r="Y7" s="164"/>
+      <c r="Z7" s="164"/>
+      <c r="AA7" s="164"/>
+      <c r="AB7" s="164"/>
+      <c r="AC7" s="183" t="s">
         <v>15</v>
       </c>
-      <c r="Y7" s="180"/>
-      <c r="AA7" s="31"/>
-      <c r="AB7" s="32"/>
-      <c r="AC7" s="32"/>
-    </row>
-    <row r="8" spans="1:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="AD7" s="180"/>
+      <c r="AF7" s="31"/>
+      <c r="AG7" s="32"/>
+      <c r="AH7" s="32"/>
+    </row>
+    <row r="8" spans="1:34" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="26"/>
       <c r="C8" s="33"/>
       <c r="D8" s="173"/>
@@ -4477,15 +4569,20 @@
       <c r="U8" s="37"/>
       <c r="V8" s="37"/>
       <c r="W8" s="39"/>
-      <c r="X8" s="183" t="s">
+      <c r="X8" s="39"/>
+      <c r="Y8" s="39"/>
+      <c r="Z8" s="39"/>
+      <c r="AA8" s="39"/>
+      <c r="AB8" s="39"/>
+      <c r="AC8" s="183" t="s">
         <v>15</v>
       </c>
-      <c r="Y8" s="181"/>
-      <c r="AA8" s="31"/>
-      <c r="AB8" s="32"/>
-      <c r="AC8" s="32"/>
-    </row>
-    <row r="9" spans="1:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="AD8" s="181"/>
+      <c r="AF8" s="31"/>
+      <c r="AG8" s="32"/>
+      <c r="AH8" s="32"/>
+    </row>
+    <row r="9" spans="1:34" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="26"/>
       <c r="C9" s="33"/>
       <c r="D9" s="173"/>
@@ -4514,15 +4611,20 @@
       <c r="U9" s="37"/>
       <c r="V9" s="37"/>
       <c r="W9" s="39"/>
-      <c r="X9" s="183" t="s">
+      <c r="X9" s="39"/>
+      <c r="Y9" s="39"/>
+      <c r="Z9" s="39"/>
+      <c r="AA9" s="39"/>
+      <c r="AB9" s="39"/>
+      <c r="AC9" s="183" t="s">
         <v>15</v>
       </c>
-      <c r="Y9" s="180"/>
-      <c r="AA9" s="31"/>
-      <c r="AB9" s="32"/>
-      <c r="AC9" s="32"/>
-    </row>
-    <row r="10" spans="1:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AD9" s="180"/>
+      <c r="AF9" s="31"/>
+      <c r="AG9" s="32"/>
+      <c r="AH9" s="32"/>
+    </row>
+    <row r="10" spans="1:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B10" s="26" t="s">
         <v>11</v>
       </c>
@@ -4555,17 +4657,22 @@
       <c r="U10" s="37"/>
       <c r="V10" s="37"/>
       <c r="W10" s="39"/>
-      <c r="X10" s="183" t="s">
+      <c r="X10" s="39"/>
+      <c r="Y10" s="39"/>
+      <c r="Z10" s="39"/>
+      <c r="AA10" s="39"/>
+      <c r="AB10" s="39"/>
+      <c r="AC10" s="183" t="s">
         <v>15</v>
       </c>
-      <c r="Y10" s="184" t="s">
+      <c r="AD10" s="184" t="s">
         <v>15</v>
       </c>
-      <c r="AA10" s="31"/>
-      <c r="AB10" s="32"/>
-      <c r="AC10" s="32"/>
-    </row>
-    <row r="11" spans="1:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AF10" s="31"/>
+      <c r="AG10" s="32"/>
+      <c r="AH10" s="32"/>
+    </row>
+    <row r="11" spans="1:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B11" s="26" t="s">
         <v>11</v>
       </c>
@@ -4598,17 +4705,22 @@
       <c r="U11" s="37"/>
       <c r="V11" s="37"/>
       <c r="W11" s="39"/>
-      <c r="X11" s="183" t="s">
+      <c r="X11" s="39"/>
+      <c r="Y11" s="39"/>
+      <c r="Z11" s="39"/>
+      <c r="AA11" s="39"/>
+      <c r="AB11" s="39"/>
+      <c r="AC11" s="183" t="s">
         <v>15</v>
       </c>
-      <c r="Y11" s="184" t="s">
+      <c r="AD11" s="184" t="s">
         <v>15</v>
       </c>
-      <c r="AA11" s="31"/>
-      <c r="AB11" s="32"/>
-      <c r="AC11" s="32"/>
-    </row>
-    <row r="12" spans="1:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AF11" s="31"/>
+      <c r="AG11" s="32"/>
+      <c r="AH11" s="32"/>
+    </row>
+    <row r="12" spans="1:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B12" s="26" t="s">
         <v>11</v>
       </c>
@@ -4639,17 +4751,22 @@
       <c r="U12" s="37"/>
       <c r="V12" s="37"/>
       <c r="W12" s="39"/>
-      <c r="X12" s="183" t="s">
+      <c r="X12" s="39"/>
+      <c r="Y12" s="39"/>
+      <c r="Z12" s="39"/>
+      <c r="AA12" s="39"/>
+      <c r="AB12" s="39"/>
+      <c r="AC12" s="183" t="s">
         <v>15</v>
       </c>
-      <c r="Y12" s="184" t="s">
+      <c r="AD12" s="184" t="s">
         <v>15</v>
       </c>
-      <c r="AA12" s="31"/>
-      <c r="AB12" s="32"/>
-      <c r="AC12" s="32"/>
-    </row>
-    <row r="13" spans="1:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AF12" s="31"/>
+      <c r="AG12" s="32"/>
+      <c r="AH12" s="32"/>
+    </row>
+    <row r="13" spans="1:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B13" s="26" t="s">
         <v>11</v>
       </c>
@@ -4680,13 +4797,22 @@
       <c r="U13" s="37"/>
       <c r="V13" s="37"/>
       <c r="W13" s="39"/>
-      <c r="X13" s="130"/>
-      <c r="Y13" s="155"/>
-      <c r="AA13" s="31"/>
-      <c r="AB13" s="32"/>
-      <c r="AC13" s="32"/>
-    </row>
-    <row r="14" spans="1:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X13" s="39"/>
+      <c r="Y13" s="39"/>
+      <c r="Z13" s="39"/>
+      <c r="AA13" s="39"/>
+      <c r="AB13" s="39"/>
+      <c r="AC13" s="183" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD13" s="184" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF13" s="31"/>
+      <c r="AG13" s="32"/>
+      <c r="AH13" s="32"/>
+    </row>
+    <row r="14" spans="1:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B14" s="26"/>
       <c r="C14" s="33"/>
       <c r="D14" s="173" t="s">
@@ -4717,13 +4843,22 @@
       <c r="U14" s="37"/>
       <c r="V14" s="37"/>
       <c r="W14" s="39"/>
-      <c r="X14" s="130"/>
-      <c r="Y14" s="155"/>
-      <c r="AA14" s="31"/>
-      <c r="AB14" s="32"/>
-      <c r="AC14" s="32"/>
-    </row>
-    <row r="15" spans="1:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X14" s="39"/>
+      <c r="Y14" s="39"/>
+      <c r="Z14" s="39"/>
+      <c r="AA14" s="39"/>
+      <c r="AB14" s="39"/>
+      <c r="AC14" s="183" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD14" s="184" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF14" s="31"/>
+      <c r="AG14" s="32"/>
+      <c r="AH14" s="32"/>
+    </row>
+    <row r="15" spans="1:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B15" s="26"/>
       <c r="C15" s="33"/>
       <c r="D15" s="173" t="s">
@@ -4754,13 +4889,22 @@
       <c r="U15" s="37"/>
       <c r="V15" s="37"/>
       <c r="W15" s="39"/>
-      <c r="X15" s="130"/>
-      <c r="Y15" s="155"/>
-      <c r="AA15" s="31"/>
-      <c r="AB15" s="32"/>
-      <c r="AC15" s="32"/>
-    </row>
-    <row r="16" spans="1:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X15" s="39"/>
+      <c r="Y15" s="39"/>
+      <c r="Z15" s="39"/>
+      <c r="AA15" s="39"/>
+      <c r="AB15" s="39"/>
+      <c r="AC15" s="183" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD15" s="184" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF15" s="31"/>
+      <c r="AG15" s="32"/>
+      <c r="AH15" s="32"/>
+    </row>
+    <row r="16" spans="1:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B16" s="26"/>
       <c r="C16" s="33"/>
       <c r="D16" s="173" t="s">
@@ -4786,18 +4930,27 @@
       <c r="R16" s="37"/>
       <c r="S16" s="37"/>
       <c r="T16" s="37"/>
-      <c r="U16" s="37"/>
+      <c r="U16" s="37" t="s">
+        <v>10</v>
+      </c>
       <c r="V16" s="37"/>
-      <c r="W16" s="39" t="s">
-        <v>10</v>
-      </c>
-      <c r="X16" s="130"/>
-      <c r="Y16" s="129"/>
-      <c r="AA16" s="31"/>
-      <c r="AB16" s="32"/>
-      <c r="AC16" s="32"/>
-    </row>
-    <row r="17" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="W16" s="39"/>
+      <c r="X16" s="39"/>
+      <c r="Y16" s="39"/>
+      <c r="Z16" s="39"/>
+      <c r="AA16" s="39"/>
+      <c r="AB16" s="39"/>
+      <c r="AC16" s="183" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD16" s="184" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF16" s="31"/>
+      <c r="AG16" s="32"/>
+      <c r="AH16" s="32"/>
+    </row>
+    <row r="17" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B17" s="26"/>
       <c r="C17" s="33"/>
       <c r="D17" s="173" t="s">
@@ -4823,18 +4976,27 @@
       <c r="R17" s="37"/>
       <c r="S17" s="37"/>
       <c r="T17" s="37"/>
-      <c r="U17" s="37"/>
+      <c r="U17" s="37" t="s">
+        <v>10</v>
+      </c>
       <c r="V17" s="37"/>
-      <c r="W17" s="39" t="s">
-        <v>10</v>
-      </c>
-      <c r="X17" s="130"/>
-      <c r="Y17" s="155"/>
-      <c r="AA17" s="31"/>
-      <c r="AB17" s="32"/>
-      <c r="AC17" s="32"/>
-    </row>
-    <row r="18" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="W17" s="39"/>
+      <c r="X17" s="39"/>
+      <c r="Y17" s="39"/>
+      <c r="Z17" s="39"/>
+      <c r="AA17" s="39"/>
+      <c r="AB17" s="39"/>
+      <c r="AC17" s="183" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD17" s="184" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF17" s="31"/>
+      <c r="AG17" s="32"/>
+      <c r="AH17" s="32"/>
+    </row>
+    <row r="18" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B18" s="26" t="s">
         <v>11</v>
       </c>
@@ -4862,18 +5024,27 @@
       <c r="R18" s="37"/>
       <c r="S18" s="37"/>
       <c r="T18" s="37"/>
-      <c r="U18" s="37"/>
+      <c r="U18" s="37" t="s">
+        <v>10</v>
+      </c>
       <c r="V18" s="37"/>
-      <c r="W18" s="39" t="s">
-        <v>10</v>
-      </c>
-      <c r="X18" s="130"/>
-      <c r="Y18" s="129"/>
-      <c r="AA18" s="31"/>
-      <c r="AB18" s="32"/>
-      <c r="AC18" s="32"/>
-    </row>
-    <row r="19" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="W18" s="39"/>
+      <c r="X18" s="39"/>
+      <c r="Y18" s="39"/>
+      <c r="Z18" s="39"/>
+      <c r="AA18" s="39"/>
+      <c r="AB18" s="39"/>
+      <c r="AC18" s="183" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD18" s="184" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF18" s="31"/>
+      <c r="AG18" s="32"/>
+      <c r="AH18" s="32"/>
+    </row>
+    <row r="19" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B19" s="26"/>
       <c r="C19" s="33"/>
       <c r="D19" s="173"/>
@@ -4899,16 +5070,27 @@
       <c r="R19" s="37"/>
       <c r="S19" s="37"/>
       <c r="T19" s="37"/>
-      <c r="U19" s="37"/>
+      <c r="U19" s="37" t="s">
+        <v>10</v>
+      </c>
       <c r="V19" s="37"/>
       <c r="W19" s="39"/>
-      <c r="X19" s="130"/>
-      <c r="Y19" s="155"/>
-      <c r="AA19" s="31"/>
-      <c r="AB19" s="32"/>
-      <c r="AC19" s="32"/>
-    </row>
-    <row r="20" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X19" s="39"/>
+      <c r="Y19" s="39"/>
+      <c r="Z19" s="39"/>
+      <c r="AA19" s="39"/>
+      <c r="AB19" s="39"/>
+      <c r="AC19" s="183" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD19" s="184" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF19" s="31"/>
+      <c r="AG19" s="32"/>
+      <c r="AH19" s="32"/>
+    </row>
+    <row r="20" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B20" s="26"/>
       <c r="C20" s="33"/>
       <c r="D20" s="173"/>
@@ -4934,16 +5116,27 @@
       <c r="R20" s="37"/>
       <c r="S20" s="37"/>
       <c r="T20" s="37"/>
-      <c r="U20" s="37"/>
+      <c r="U20" s="37" t="s">
+        <v>10</v>
+      </c>
       <c r="V20" s="37"/>
       <c r="W20" s="39"/>
-      <c r="X20" s="130"/>
-      <c r="Y20" s="129"/>
-      <c r="AA20" s="31"/>
-      <c r="AB20" s="32"/>
-      <c r="AC20" s="32"/>
-    </row>
-    <row r="21" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X20" s="39"/>
+      <c r="Y20" s="39"/>
+      <c r="Z20" s="39"/>
+      <c r="AA20" s="39"/>
+      <c r="AB20" s="39"/>
+      <c r="AC20" s="183" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD20" s="184" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF20" s="31"/>
+      <c r="AG20" s="32"/>
+      <c r="AH20" s="32"/>
+    </row>
+    <row r="21" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B21" s="26"/>
       <c r="C21" s="33"/>
       <c r="D21" s="173"/>
@@ -4970,15 +5163,26 @@
       <c r="S21" s="37"/>
       <c r="T21" s="37"/>
       <c r="U21" s="37"/>
-      <c r="V21" s="37"/>
+      <c r="V21" s="37" t="s">
+        <v>11</v>
+      </c>
       <c r="W21" s="39"/>
-      <c r="X21" s="130"/>
-      <c r="Y21" s="155"/>
-      <c r="AA21" s="31"/>
-      <c r="AB21" s="32"/>
-      <c r="AC21" s="32"/>
-    </row>
-    <row r="22" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X21" s="39"/>
+      <c r="Y21" s="39"/>
+      <c r="Z21" s="39"/>
+      <c r="AA21" s="39"/>
+      <c r="AB21" s="39"/>
+      <c r="AC21" s="183" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD21" s="184" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF21" s="31"/>
+      <c r="AG21" s="32"/>
+      <c r="AH21" s="32"/>
+    </row>
+    <row r="22" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B22" s="26"/>
       <c r="C22" s="33"/>
       <c r="D22" s="173"/>
@@ -5005,15 +5209,26 @@
       <c r="S22" s="37"/>
       <c r="T22" s="37"/>
       <c r="U22" s="37"/>
-      <c r="V22" s="37"/>
+      <c r="V22" s="37" t="s">
+        <v>11</v>
+      </c>
       <c r="W22" s="39"/>
-      <c r="X22" s="130"/>
-      <c r="Y22" s="129"/>
-      <c r="AA22" s="31"/>
-      <c r="AB22" s="32"/>
-      <c r="AC22" s="32"/>
-    </row>
-    <row r="23" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X22" s="39"/>
+      <c r="Y22" s="39"/>
+      <c r="Z22" s="39"/>
+      <c r="AA22" s="39"/>
+      <c r="AB22" s="39"/>
+      <c r="AC22" s="183" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD22" s="184" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF22" s="31"/>
+      <c r="AG22" s="32"/>
+      <c r="AH22" s="32"/>
+    </row>
+    <row r="23" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B23" s="26"/>
       <c r="C23" s="33"/>
       <c r="D23" s="173"/>
@@ -5041,14 +5256,25 @@
       <c r="T23" s="37"/>
       <c r="U23" s="37"/>
       <c r="V23" s="37"/>
-      <c r="W23" s="39"/>
-      <c r="X23" s="130"/>
-      <c r="Y23" s="155"/>
-      <c r="AA23" s="31"/>
-      <c r="AB23" s="32"/>
-      <c r="AC23" s="32"/>
-    </row>
-    <row r="24" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="W23" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="X23" s="39"/>
+      <c r="Y23" s="39"/>
+      <c r="Z23" s="39"/>
+      <c r="AA23" s="39"/>
+      <c r="AB23" s="39"/>
+      <c r="AC23" s="183" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD23" s="184" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF23" s="31"/>
+      <c r="AG23" s="32"/>
+      <c r="AH23" s="32"/>
+    </row>
+    <row r="24" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B24" s="26"/>
       <c r="C24" s="33"/>
       <c r="D24" s="173"/>
@@ -5076,14 +5302,25 @@
       <c r="T24" s="37"/>
       <c r="U24" s="37"/>
       <c r="V24" s="37"/>
-      <c r="W24" s="39"/>
-      <c r="X24" s="130"/>
-      <c r="Y24" s="129"/>
-      <c r="AA24" s="31"/>
-      <c r="AB24" s="32"/>
-      <c r="AC24" s="32"/>
-    </row>
-    <row r="25" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="W24" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="X24" s="39"/>
+      <c r="Y24" s="39"/>
+      <c r="Z24" s="39"/>
+      <c r="AA24" s="39"/>
+      <c r="AB24" s="39"/>
+      <c r="AC24" s="183" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD24" s="184" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF24" s="31"/>
+      <c r="AG24" s="32"/>
+      <c r="AH24" s="32"/>
+    </row>
+    <row r="25" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B25" s="26"/>
       <c r="C25" s="33"/>
       <c r="D25" s="173"/>
@@ -5109,14 +5346,25 @@
       <c r="T25" s="37"/>
       <c r="U25" s="37"/>
       <c r="V25" s="37"/>
-      <c r="W25" s="39"/>
-      <c r="X25" s="130"/>
-      <c r="Y25" s="155"/>
-      <c r="AA25" s="31"/>
-      <c r="AB25" s="32"/>
-      <c r="AC25" s="32"/>
-    </row>
-    <row r="26" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="W25" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="X25" s="39"/>
+      <c r="Y25" s="39"/>
+      <c r="Z25" s="39"/>
+      <c r="AA25" s="39"/>
+      <c r="AB25" s="39"/>
+      <c r="AC25" s="183" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD25" s="184" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF25" s="31"/>
+      <c r="AG25" s="32"/>
+      <c r="AH25" s="32"/>
+    </row>
+    <row r="26" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B26" s="26"/>
       <c r="C26" s="33"/>
       <c r="D26" s="173"/>
@@ -5142,14 +5390,25 @@
       <c r="T26" s="37"/>
       <c r="U26" s="37"/>
       <c r="V26" s="37"/>
-      <c r="W26" s="39"/>
-      <c r="X26" s="130"/>
-      <c r="Y26" s="129"/>
-      <c r="AA26" s="31"/>
-      <c r="AB26" s="32"/>
-      <c r="AC26" s="32"/>
-    </row>
-    <row r="27" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="W26" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="X26" s="39"/>
+      <c r="Y26" s="39"/>
+      <c r="Z26" s="39"/>
+      <c r="AA26" s="39"/>
+      <c r="AB26" s="39"/>
+      <c r="AC26" s="183" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD26" s="184" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF26" s="31"/>
+      <c r="AG26" s="32"/>
+      <c r="AH26" s="32"/>
+    </row>
+    <row r="27" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B27" s="26"/>
       <c r="C27" s="33"/>
       <c r="D27" s="173"/>
@@ -5176,13 +5435,24 @@
       <c r="U27" s="37"/>
       <c r="V27" s="37"/>
       <c r="W27" s="39"/>
-      <c r="X27" s="133"/>
-      <c r="Y27" s="155"/>
-      <c r="AA27" s="31"/>
-      <c r="AB27" s="32"/>
-      <c r="AC27" s="32"/>
-    </row>
-    <row r="28" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X27" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="Y27" s="39"/>
+      <c r="Z27" s="39"/>
+      <c r="AA27" s="39"/>
+      <c r="AB27" s="39"/>
+      <c r="AC27" s="183" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD27" s="184" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF27" s="31"/>
+      <c r="AG27" s="32"/>
+      <c r="AH27" s="32"/>
+    </row>
+    <row r="28" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B28" s="26"/>
       <c r="C28" s="33"/>
       <c r="D28" s="173"/>
@@ -5207,14 +5477,26 @@
       <c r="S28" s="37"/>
       <c r="T28" s="37"/>
       <c r="U28" s="37"/>
-      <c r="W28" s="39"/>
-      <c r="X28" s="130"/>
-      <c r="Y28" s="129"/>
-      <c r="AA28" s="31"/>
-      <c r="AB28" s="32"/>
-      <c r="AC28" s="32"/>
-    </row>
-    <row r="29" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="V28" s="37"/>
+      <c r="W28" s="37"/>
+      <c r="X28" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="Y28" s="39"/>
+      <c r="Z28" s="39"/>
+      <c r="AA28" s="39"/>
+      <c r="AB28" s="39"/>
+      <c r="AC28" s="183" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD28" s="184" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF28" s="31"/>
+      <c r="AG28" s="32"/>
+      <c r="AH28" s="32"/>
+    </row>
+    <row r="29" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B29" s="44"/>
       <c r="C29" s="45"/>
       <c r="D29" s="174"/>
@@ -5238,15 +5520,27 @@
       <c r="R29" s="38"/>
       <c r="S29" s="38"/>
       <c r="T29" s="38"/>
+      <c r="U29" s="38"/>
       <c r="V29" s="38"/>
       <c r="W29" s="165"/>
-      <c r="X29" s="133"/>
-      <c r="Y29" s="155"/>
-      <c r="AA29" s="31"/>
-      <c r="AB29" s="32"/>
-      <c r="AC29" s="32"/>
-    </row>
-    <row r="30" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X29" s="165" t="s">
+        <v>11</v>
+      </c>
+      <c r="Y29" s="165"/>
+      <c r="Z29" s="165"/>
+      <c r="AA29" s="165"/>
+      <c r="AB29" s="165"/>
+      <c r="AC29" s="183" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD29" s="184" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF29" s="31"/>
+      <c r="AG29" s="32"/>
+      <c r="AH29" s="32"/>
+    </row>
+    <row r="30" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B30" s="44"/>
       <c r="C30" s="45"/>
       <c r="D30" s="174"/>
@@ -5266,15 +5560,21 @@
       <c r="R30" s="38"/>
       <c r="S30" s="38"/>
       <c r="T30" s="38"/>
+      <c r="U30" s="38"/>
       <c r="V30" s="38"/>
       <c r="W30" s="165"/>
-      <c r="X30" s="133"/>
-      <c r="Y30" s="155"/>
-      <c r="AA30" s="31"/>
-      <c r="AB30" s="32"/>
-      <c r="AC30" s="32"/>
-    </row>
-    <row r="31" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X30" s="165"/>
+      <c r="Y30" s="165"/>
+      <c r="Z30" s="165"/>
+      <c r="AA30" s="165"/>
+      <c r="AB30" s="165"/>
+      <c r="AC30" s="133"/>
+      <c r="AD30" s="155"/>
+      <c r="AF30" s="31"/>
+      <c r="AG30" s="32"/>
+      <c r="AH30" s="32"/>
+    </row>
+    <row r="31" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B31" s="44"/>
       <c r="C31" s="45"/>
       <c r="D31" s="174"/>
@@ -5294,15 +5594,21 @@
       <c r="R31" s="38"/>
       <c r="S31" s="38"/>
       <c r="T31" s="38"/>
+      <c r="U31" s="38"/>
       <c r="V31" s="38"/>
       <c r="W31" s="165"/>
-      <c r="X31" s="133"/>
-      <c r="Y31" s="155"/>
-      <c r="AA31" s="31"/>
-      <c r="AB31" s="32"/>
-      <c r="AC31" s="32"/>
-    </row>
-    <row r="32" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X31" s="165"/>
+      <c r="Y31" s="165"/>
+      <c r="Z31" s="165"/>
+      <c r="AA31" s="165"/>
+      <c r="AB31" s="165"/>
+      <c r="AC31" s="133"/>
+      <c r="AD31" s="155"/>
+      <c r="AF31" s="31"/>
+      <c r="AG31" s="32"/>
+      <c r="AH31" s="32"/>
+    </row>
+    <row r="32" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B32" s="44"/>
       <c r="C32" s="45"/>
       <c r="D32" s="174"/>
@@ -5322,15 +5628,21 @@
       <c r="R32" s="38"/>
       <c r="S32" s="38"/>
       <c r="T32" s="38"/>
+      <c r="U32" s="38"/>
       <c r="V32" s="38"/>
       <c r="W32" s="165"/>
-      <c r="X32" s="133"/>
-      <c r="Y32" s="155"/>
-      <c r="AA32" s="31"/>
-      <c r="AB32" s="32"/>
-      <c r="AC32" s="32"/>
-    </row>
-    <row r="33" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X32" s="165"/>
+      <c r="Y32" s="165"/>
+      <c r="Z32" s="165"/>
+      <c r="AA32" s="165"/>
+      <c r="AB32" s="165"/>
+      <c r="AC32" s="133"/>
+      <c r="AD32" s="155"/>
+      <c r="AF32" s="31"/>
+      <c r="AG32" s="32"/>
+      <c r="AH32" s="32"/>
+    </row>
+    <row r="33" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B33" s="44"/>
       <c r="C33" s="45"/>
       <c r="D33" s="174"/>
@@ -5350,15 +5662,21 @@
       <c r="R33" s="38"/>
       <c r="S33" s="38"/>
       <c r="T33" s="38"/>
+      <c r="U33" s="38"/>
       <c r="V33" s="38"/>
       <c r="W33" s="165"/>
-      <c r="X33" s="133"/>
-      <c r="Y33" s="155"/>
-      <c r="AA33" s="31"/>
-      <c r="AB33" s="32"/>
-      <c r="AC33" s="32"/>
-    </row>
-    <row r="34" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X33" s="165"/>
+      <c r="Y33" s="165"/>
+      <c r="Z33" s="165"/>
+      <c r="AA33" s="165"/>
+      <c r="AB33" s="165"/>
+      <c r="AC33" s="133"/>
+      <c r="AD33" s="155"/>
+      <c r="AF33" s="31"/>
+      <c r="AG33" s="32"/>
+      <c r="AH33" s="32"/>
+    </row>
+    <row r="34" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B34" s="44"/>
       <c r="C34" s="45"/>
       <c r="D34" s="174"/>
@@ -5378,15 +5696,21 @@
       <c r="R34" s="38"/>
       <c r="S34" s="38"/>
       <c r="T34" s="38"/>
+      <c r="U34" s="38"/>
       <c r="V34" s="38"/>
       <c r="W34" s="165"/>
-      <c r="X34" s="133"/>
-      <c r="Y34" s="155"/>
-      <c r="AA34" s="31"/>
-      <c r="AB34" s="32"/>
-      <c r="AC34" s="32"/>
-    </row>
-    <row r="35" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X34" s="165"/>
+      <c r="Y34" s="165"/>
+      <c r="Z34" s="165"/>
+      <c r="AA34" s="165"/>
+      <c r="AB34" s="165"/>
+      <c r="AC34" s="133"/>
+      <c r="AD34" s="155"/>
+      <c r="AF34" s="31"/>
+      <c r="AG34" s="32"/>
+      <c r="AH34" s="32"/>
+    </row>
+    <row r="35" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B35" s="44"/>
       <c r="C35" s="45"/>
       <c r="D35" s="174"/>
@@ -5406,15 +5730,21 @@
       <c r="R35" s="38"/>
       <c r="S35" s="38"/>
       <c r="T35" s="38"/>
+      <c r="U35" s="38"/>
       <c r="V35" s="38"/>
       <c r="W35" s="165"/>
-      <c r="X35" s="133"/>
-      <c r="Y35" s="155"/>
-      <c r="AA35" s="31"/>
-      <c r="AB35" s="32"/>
-      <c r="AC35" s="32"/>
-    </row>
-    <row r="36" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X35" s="165"/>
+      <c r="Y35" s="165"/>
+      <c r="Z35" s="165"/>
+      <c r="AA35" s="165"/>
+      <c r="AB35" s="165"/>
+      <c r="AC35" s="133"/>
+      <c r="AD35" s="155"/>
+      <c r="AF35" s="31"/>
+      <c r="AG35" s="32"/>
+      <c r="AH35" s="32"/>
+    </row>
+    <row r="36" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B36" s="44"/>
       <c r="C36" s="45"/>
       <c r="D36" s="174"/>
@@ -5434,15 +5764,21 @@
       <c r="R36" s="38"/>
       <c r="S36" s="38"/>
       <c r="T36" s="38"/>
+      <c r="U36" s="38"/>
       <c r="V36" s="38"/>
       <c r="W36" s="165"/>
-      <c r="X36" s="133"/>
-      <c r="Y36" s="155"/>
-      <c r="AA36" s="31"/>
-      <c r="AB36" s="32"/>
-      <c r="AC36" s="32"/>
-    </row>
-    <row r="37" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X36" s="165"/>
+      <c r="Y36" s="165"/>
+      <c r="Z36" s="165"/>
+      <c r="AA36" s="165"/>
+      <c r="AB36" s="165"/>
+      <c r="AC36" s="133"/>
+      <c r="AD36" s="155"/>
+      <c r="AF36" s="31"/>
+      <c r="AG36" s="32"/>
+      <c r="AH36" s="32"/>
+    </row>
+    <row r="37" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B37" s="44"/>
       <c r="C37" s="45"/>
       <c r="D37" s="174"/>
@@ -5462,15 +5798,21 @@
       <c r="R37" s="38"/>
       <c r="S37" s="38"/>
       <c r="T37" s="38"/>
+      <c r="U37" s="38"/>
       <c r="V37" s="38"/>
       <c r="W37" s="165"/>
-      <c r="X37" s="133"/>
-      <c r="Y37" s="155"/>
-      <c r="AA37" s="31"/>
-      <c r="AB37" s="32"/>
-      <c r="AC37" s="32"/>
-    </row>
-    <row r="38" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X37" s="165"/>
+      <c r="Y37" s="165"/>
+      <c r="Z37" s="165"/>
+      <c r="AA37" s="165"/>
+      <c r="AB37" s="165"/>
+      <c r="AC37" s="133"/>
+      <c r="AD37" s="155"/>
+      <c r="AF37" s="31"/>
+      <c r="AG37" s="32"/>
+      <c r="AH37" s="32"/>
+    </row>
+    <row r="38" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B38" s="44"/>
       <c r="C38" s="45"/>
       <c r="D38" s="174"/>
@@ -5490,15 +5832,21 @@
       <c r="R38" s="38"/>
       <c r="S38" s="38"/>
       <c r="T38" s="38"/>
+      <c r="U38" s="38"/>
       <c r="V38" s="38"/>
       <c r="W38" s="165"/>
-      <c r="X38" s="133"/>
-      <c r="Y38" s="155"/>
-      <c r="AA38" s="31"/>
-      <c r="AB38" s="32"/>
-      <c r="AC38" s="32"/>
-    </row>
-    <row r="39" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X38" s="165"/>
+      <c r="Y38" s="165"/>
+      <c r="Z38" s="165"/>
+      <c r="AA38" s="165"/>
+      <c r="AB38" s="165"/>
+      <c r="AC38" s="133"/>
+      <c r="AD38" s="155"/>
+      <c r="AF38" s="31"/>
+      <c r="AG38" s="32"/>
+      <c r="AH38" s="32"/>
+    </row>
+    <row r="39" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B39" s="44"/>
       <c r="C39" s="45"/>
       <c r="D39" s="174"/>
@@ -5518,15 +5866,21 @@
       <c r="R39" s="38"/>
       <c r="S39" s="38"/>
       <c r="T39" s="38"/>
+      <c r="U39" s="38"/>
       <c r="V39" s="38"/>
       <c r="W39" s="165"/>
-      <c r="X39" s="133"/>
-      <c r="Y39" s="155"/>
-      <c r="AA39" s="31"/>
-      <c r="AB39" s="32"/>
-      <c r="AC39" s="32"/>
-    </row>
-    <row r="40" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X39" s="165"/>
+      <c r="Y39" s="165"/>
+      <c r="Z39" s="165"/>
+      <c r="AA39" s="165"/>
+      <c r="AB39" s="165"/>
+      <c r="AC39" s="133"/>
+      <c r="AD39" s="155"/>
+      <c r="AF39" s="31"/>
+      <c r="AG39" s="32"/>
+      <c r="AH39" s="32"/>
+    </row>
+    <row r="40" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B40" s="44"/>
       <c r="C40" s="45"/>
       <c r="D40" s="174"/>
@@ -5546,15 +5900,21 @@
       <c r="R40" s="38"/>
       <c r="S40" s="38"/>
       <c r="T40" s="38"/>
+      <c r="U40" s="38"/>
       <c r="V40" s="38"/>
       <c r="W40" s="165"/>
-      <c r="X40" s="133"/>
-      <c r="Y40" s="155"/>
-      <c r="AA40" s="31"/>
-      <c r="AB40" s="32"/>
-      <c r="AC40" s="32"/>
-    </row>
-    <row r="41" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X40" s="165"/>
+      <c r="Y40" s="165"/>
+      <c r="Z40" s="165"/>
+      <c r="AA40" s="165"/>
+      <c r="AB40" s="165"/>
+      <c r="AC40" s="133"/>
+      <c r="AD40" s="155"/>
+      <c r="AF40" s="31"/>
+      <c r="AG40" s="32"/>
+      <c r="AH40" s="32"/>
+    </row>
+    <row r="41" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B41" s="44"/>
       <c r="C41" s="45"/>
       <c r="D41" s="174"/>
@@ -5574,15 +5934,21 @@
       <c r="R41" s="38"/>
       <c r="S41" s="38"/>
       <c r="T41" s="38"/>
+      <c r="U41" s="38"/>
       <c r="V41" s="38"/>
       <c r="W41" s="165"/>
-      <c r="X41" s="133"/>
-      <c r="Y41" s="155"/>
-      <c r="AA41" s="31"/>
-      <c r="AB41" s="32"/>
-      <c r="AC41" s="32"/>
-    </row>
-    <row r="42" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X41" s="165"/>
+      <c r="Y41" s="165"/>
+      <c r="Z41" s="165"/>
+      <c r="AA41" s="165"/>
+      <c r="AB41" s="165"/>
+      <c r="AC41" s="133"/>
+      <c r="AD41" s="155"/>
+      <c r="AF41" s="31"/>
+      <c r="AG41" s="32"/>
+      <c r="AH41" s="32"/>
+    </row>
+    <row r="42" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B42" s="44"/>
       <c r="C42" s="45"/>
       <c r="D42" s="174"/>
@@ -5602,15 +5968,21 @@
       <c r="R42" s="38"/>
       <c r="S42" s="38"/>
       <c r="T42" s="38"/>
+      <c r="U42" s="38"/>
       <c r="V42" s="38"/>
       <c r="W42" s="165"/>
-      <c r="X42" s="133"/>
-      <c r="Y42" s="155"/>
-      <c r="AA42" s="31"/>
-      <c r="AB42" s="32"/>
-      <c r="AC42" s="32"/>
-    </row>
-    <row r="43" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X42" s="165"/>
+      <c r="Y42" s="165"/>
+      <c r="Z42" s="165"/>
+      <c r="AA42" s="165"/>
+      <c r="AB42" s="165"/>
+      <c r="AC42" s="133"/>
+      <c r="AD42" s="155"/>
+      <c r="AF42" s="31"/>
+      <c r="AG42" s="32"/>
+      <c r="AH42" s="32"/>
+    </row>
+    <row r="43" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B43" s="44"/>
       <c r="C43" s="45"/>
       <c r="D43" s="174"/>
@@ -5630,15 +6002,21 @@
       <c r="R43" s="38"/>
       <c r="S43" s="38"/>
       <c r="T43" s="38"/>
+      <c r="U43" s="38"/>
       <c r="V43" s="38"/>
       <c r="W43" s="165"/>
-      <c r="X43" s="133"/>
-      <c r="Y43" s="155"/>
-      <c r="AA43" s="31"/>
-      <c r="AB43" s="32"/>
-      <c r="AC43" s="32"/>
-    </row>
-    <row r="44" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X43" s="165"/>
+      <c r="Y43" s="165"/>
+      <c r="Z43" s="165"/>
+      <c r="AA43" s="165"/>
+      <c r="AB43" s="165"/>
+      <c r="AC43" s="133"/>
+      <c r="AD43" s="155"/>
+      <c r="AF43" s="31"/>
+      <c r="AG43" s="32"/>
+      <c r="AH43" s="32"/>
+    </row>
+    <row r="44" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B44" s="44"/>
       <c r="C44" s="45"/>
       <c r="D44" s="174"/>
@@ -5658,15 +6036,21 @@
       <c r="R44" s="38"/>
       <c r="S44" s="38"/>
       <c r="T44" s="38"/>
+      <c r="U44" s="38"/>
       <c r="V44" s="38"/>
       <c r="W44" s="165"/>
-      <c r="X44" s="133"/>
-      <c r="Y44" s="155"/>
-      <c r="AA44" s="31"/>
-      <c r="AB44" s="32"/>
-      <c r="AC44" s="32"/>
-    </row>
-    <row r="45" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X44" s="165"/>
+      <c r="Y44" s="165"/>
+      <c r="Z44" s="165"/>
+      <c r="AA44" s="165"/>
+      <c r="AB44" s="165"/>
+      <c r="AC44" s="133"/>
+      <c r="AD44" s="155"/>
+      <c r="AF44" s="31"/>
+      <c r="AG44" s="32"/>
+      <c r="AH44" s="32"/>
+    </row>
+    <row r="45" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B45" s="44"/>
       <c r="C45" s="45"/>
       <c r="D45" s="174"/>
@@ -5686,15 +6070,21 @@
       <c r="R45" s="38"/>
       <c r="S45" s="38"/>
       <c r="T45" s="38"/>
+      <c r="U45" s="38"/>
       <c r="V45" s="38"/>
       <c r="W45" s="165"/>
-      <c r="X45" s="133"/>
-      <c r="Y45" s="155"/>
-      <c r="AA45" s="31"/>
-      <c r="AB45" s="32"/>
-      <c r="AC45" s="32"/>
-    </row>
-    <row r="46" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X45" s="165"/>
+      <c r="Y45" s="165"/>
+      <c r="Z45" s="165"/>
+      <c r="AA45" s="165"/>
+      <c r="AB45" s="165"/>
+      <c r="AC45" s="133"/>
+      <c r="AD45" s="155"/>
+      <c r="AF45" s="31"/>
+      <c r="AG45" s="32"/>
+      <c r="AH45" s="32"/>
+    </row>
+    <row r="46" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B46" s="44"/>
       <c r="C46" s="45"/>
       <c r="D46" s="174"/>
@@ -5714,15 +6104,21 @@
       <c r="R46" s="38"/>
       <c r="S46" s="38"/>
       <c r="T46" s="38"/>
+      <c r="U46" s="38"/>
       <c r="V46" s="38"/>
       <c r="W46" s="165"/>
-      <c r="X46" s="133"/>
-      <c r="Y46" s="155"/>
-      <c r="AA46" s="31"/>
-      <c r="AB46" s="32"/>
-      <c r="AC46" s="32"/>
-    </row>
-    <row r="47" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X46" s="165"/>
+      <c r="Y46" s="165"/>
+      <c r="Z46" s="165"/>
+      <c r="AA46" s="165"/>
+      <c r="AB46" s="165"/>
+      <c r="AC46" s="133"/>
+      <c r="AD46" s="155"/>
+      <c r="AF46" s="31"/>
+      <c r="AG46" s="32"/>
+      <c r="AH46" s="32"/>
+    </row>
+    <row r="47" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B47" s="44"/>
       <c r="C47" s="45"/>
       <c r="D47" s="174"/>
@@ -5742,15 +6138,21 @@
       <c r="R47" s="38"/>
       <c r="S47" s="38"/>
       <c r="T47" s="38"/>
+      <c r="U47" s="38"/>
       <c r="V47" s="38"/>
       <c r="W47" s="165"/>
-      <c r="X47" s="133"/>
-      <c r="Y47" s="155"/>
-      <c r="AA47" s="31"/>
-      <c r="AB47" s="32"/>
-      <c r="AC47" s="32"/>
-    </row>
-    <row r="48" spans="2:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X47" s="165"/>
+      <c r="Y47" s="165"/>
+      <c r="Z47" s="165"/>
+      <c r="AA47" s="165"/>
+      <c r="AB47" s="165"/>
+      <c r="AC47" s="133"/>
+      <c r="AD47" s="155"/>
+      <c r="AF47" s="31"/>
+      <c r="AG47" s="32"/>
+      <c r="AH47" s="32"/>
+    </row>
+    <row r="48" spans="2:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B48" s="44"/>
       <c r="C48" s="45"/>
       <c r="D48" s="174"/>
@@ -5770,15 +6172,21 @@
       <c r="R48" s="38"/>
       <c r="S48" s="38"/>
       <c r="T48" s="38"/>
+      <c r="U48" s="38"/>
       <c r="V48" s="38"/>
       <c r="W48" s="165"/>
-      <c r="X48" s="133"/>
-      <c r="Y48" s="155"/>
-      <c r="AA48" s="31"/>
-      <c r="AB48" s="32"/>
-      <c r="AC48" s="32"/>
-    </row>
-    <row r="49" spans="1:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X48" s="165"/>
+      <c r="Y48" s="165"/>
+      <c r="Z48" s="165"/>
+      <c r="AA48" s="165"/>
+      <c r="AB48" s="165"/>
+      <c r="AC48" s="133"/>
+      <c r="AD48" s="155"/>
+      <c r="AF48" s="31"/>
+      <c r="AG48" s="32"/>
+      <c r="AH48" s="32"/>
+    </row>
+    <row r="49" spans="1:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B49" s="44"/>
       <c r="C49" s="45"/>
       <c r="D49" s="174"/>
@@ -5801,13 +6209,18 @@
       <c r="U49" s="38"/>
       <c r="V49" s="38"/>
       <c r="W49" s="165"/>
-      <c r="X49" s="133"/>
-      <c r="Y49" s="155"/>
-      <c r="AA49" s="31"/>
-      <c r="AB49" s="32"/>
-      <c r="AC49" s="32"/>
-    </row>
-    <row r="50" spans="1:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X49" s="165"/>
+      <c r="Y49" s="165"/>
+      <c r="Z49" s="165"/>
+      <c r="AA49" s="165"/>
+      <c r="AB49" s="165"/>
+      <c r="AC49" s="133"/>
+      <c r="AD49" s="155"/>
+      <c r="AF49" s="31"/>
+      <c r="AG49" s="32"/>
+      <c r="AH49" s="32"/>
+    </row>
+    <row r="50" spans="1:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B50" s="44"/>
       <c r="C50" s="45"/>
       <c r="D50" s="174"/>
@@ -5830,13 +6243,18 @@
       <c r="U50" s="38"/>
       <c r="V50" s="38"/>
       <c r="W50" s="165"/>
-      <c r="X50" s="133"/>
-      <c r="Y50" s="129"/>
-      <c r="AA50" s="31"/>
-      <c r="AB50" s="32"/>
-      <c r="AC50" s="32"/>
-    </row>
-    <row r="51" spans="1:29" s="25" customFormat="1" ht="13.8" x14ac:dyDescent="0.3">
+      <c r="X50" s="165"/>
+      <c r="Y50" s="165"/>
+      <c r="Z50" s="165"/>
+      <c r="AA50" s="165"/>
+      <c r="AB50" s="165"/>
+      <c r="AC50" s="133"/>
+      <c r="AD50" s="129"/>
+      <c r="AF50" s="31"/>
+      <c r="AG50" s="32"/>
+      <c r="AH50" s="32"/>
+    </row>
+    <row r="51" spans="1:34" s="25" customFormat="1" ht="13.8" x14ac:dyDescent="0.3">
       <c r="B51" s="50"/>
       <c r="C51" s="51"/>
       <c r="D51" s="175"/>
@@ -5863,15 +6281,20 @@
       <c r="U51" s="57"/>
       <c r="V51" s="57"/>
       <c r="W51" s="166"/>
-      <c r="X51" s="215" t="s">
+      <c r="X51" s="166"/>
+      <c r="Y51" s="166"/>
+      <c r="Z51" s="166"/>
+      <c r="AA51" s="166"/>
+      <c r="AB51" s="166"/>
+      <c r="AC51" s="222" t="s">
         <v>37</v>
       </c>
-      <c r="Y51" s="216"/>
-      <c r="AA51" s="31"/>
-      <c r="AB51" s="32"/>
-      <c r="AC51" s="32"/>
-    </row>
-    <row r="52" spans="1:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="AD51" s="223"/>
+      <c r="AF51" s="31"/>
+      <c r="AG51" s="32"/>
+      <c r="AH51" s="32"/>
+    </row>
+    <row r="52" spans="1:34" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B52" s="58"/>
       <c r="C52" s="59"/>
       <c r="D52" s="172"/>
@@ -5898,13 +6321,18 @@
       <c r="U52" s="63"/>
       <c r="V52" s="63"/>
       <c r="W52" s="147"/>
-      <c r="X52" s="157"/>
-      <c r="Y52" s="158"/>
-      <c r="AA52" s="31"/>
-      <c r="AB52" s="32"/>
-      <c r="AC52" s="32"/>
-    </row>
-    <row r="53" spans="1:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="X52" s="147"/>
+      <c r="Y52" s="147"/>
+      <c r="Z52" s="147"/>
+      <c r="AA52" s="147"/>
+      <c r="AB52" s="147"/>
+      <c r="AC52" s="157"/>
+      <c r="AD52" s="158"/>
+      <c r="AF52" s="31"/>
+      <c r="AG52" s="32"/>
+      <c r="AH52" s="32"/>
+    </row>
+    <row r="53" spans="1:34" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B53" s="58"/>
       <c r="C53" s="59"/>
       <c r="D53" s="172"/>
@@ -5931,13 +6359,18 @@
       <c r="U53" s="63"/>
       <c r="V53" s="63"/>
       <c r="W53" s="147"/>
-      <c r="X53" s="159"/>
-      <c r="Y53" s="158"/>
-      <c r="AA53" s="31"/>
-      <c r="AB53" s="32"/>
-      <c r="AC53" s="32"/>
-    </row>
-    <row r="54" spans="1:29" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="X53" s="147"/>
+      <c r="Y53" s="147"/>
+      <c r="Z53" s="147"/>
+      <c r="AA53" s="147"/>
+      <c r="AB53" s="147"/>
+      <c r="AC53" s="159"/>
+      <c r="AD53" s="158"/>
+      <c r="AF53" s="31"/>
+      <c r="AG53" s="32"/>
+      <c r="AH53" s="32"/>
+    </row>
+    <row r="54" spans="1:34" s="25" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B54" s="26"/>
       <c r="C54" s="33"/>
       <c r="D54" s="173"/>
@@ -5964,13 +6397,18 @@
       <c r="U54" s="65"/>
       <c r="V54" s="65"/>
       <c r="W54" s="66"/>
-      <c r="X54" s="130"/>
-      <c r="Y54" s="160"/>
-      <c r="AA54" s="31"/>
-      <c r="AB54" s="32"/>
-      <c r="AC54" s="32"/>
-    </row>
-    <row r="55" spans="1:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X54" s="66"/>
+      <c r="Y54" s="66"/>
+      <c r="Z54" s="66"/>
+      <c r="AA54" s="66"/>
+      <c r="AB54" s="66"/>
+      <c r="AC54" s="130"/>
+      <c r="AD54" s="160"/>
+      <c r="AF54" s="31"/>
+      <c r="AG54" s="32"/>
+      <c r="AH54" s="32"/>
+    </row>
+    <row r="55" spans="1:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B55" s="26"/>
       <c r="C55" s="33"/>
       <c r="D55" s="173"/>
@@ -5995,13 +6433,18 @@
       <c r="U55" s="65"/>
       <c r="V55" s="65"/>
       <c r="W55" s="66"/>
-      <c r="X55" s="130"/>
-      <c r="Y55" s="155"/>
-      <c r="AA55" s="31"/>
-      <c r="AB55" s="32"/>
-      <c r="AC55" s="32"/>
-    </row>
-    <row r="56" spans="1:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X55" s="66"/>
+      <c r="Y55" s="66"/>
+      <c r="Z55" s="66"/>
+      <c r="AA55" s="66"/>
+      <c r="AB55" s="66"/>
+      <c r="AC55" s="130"/>
+      <c r="AD55" s="155"/>
+      <c r="AF55" s="31"/>
+      <c r="AG55" s="32"/>
+      <c r="AH55" s="32"/>
+    </row>
+    <row r="56" spans="1:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B56" s="26"/>
       <c r="C56" s="33"/>
       <c r="D56" s="173"/>
@@ -6026,13 +6469,18 @@
       <c r="U56" s="65"/>
       <c r="V56" s="65"/>
       <c r="W56" s="66"/>
-      <c r="X56" s="156"/>
-      <c r="Y56" s="129"/>
-      <c r="AA56" s="31"/>
-      <c r="AB56" s="32"/>
-      <c r="AC56" s="32"/>
-    </row>
-    <row r="57" spans="1:29" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="X56" s="66"/>
+      <c r="Y56" s="66"/>
+      <c r="Z56" s="66"/>
+      <c r="AA56" s="66"/>
+      <c r="AB56" s="66"/>
+      <c r="AC56" s="156"/>
+      <c r="AD56" s="129"/>
+      <c r="AF56" s="31"/>
+      <c r="AG56" s="32"/>
+      <c r="AH56" s="32"/>
+    </row>
+    <row r="57" spans="1:34" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B57" s="67"/>
       <c r="C57" s="68"/>
       <c r="D57" s="176"/>
@@ -6055,13 +6503,18 @@
       <c r="U57" s="71"/>
       <c r="V57" s="71"/>
       <c r="W57" s="167"/>
-      <c r="X57" s="72"/>
-      <c r="Y57" s="73"/>
-      <c r="AA57" s="31"/>
-      <c r="AB57" s="32"/>
-      <c r="AC57" s="32"/>
-    </row>
-    <row r="58" spans="1:29" s="85" customFormat="1" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="X57" s="167"/>
+      <c r="Y57" s="167"/>
+      <c r="Z57" s="167"/>
+      <c r="AA57" s="167"/>
+      <c r="AB57" s="167"/>
+      <c r="AC57" s="72"/>
+      <c r="AD57" s="73"/>
+      <c r="AF57" s="31"/>
+      <c r="AG57" s="32"/>
+      <c r="AH57" s="32"/>
+    </row>
+    <row r="58" spans="1:34" s="85" customFormat="1" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="74"/>
       <c r="B58" s="75"/>
       <c r="C58" s="76"/>
@@ -6107,17 +6560,32 @@
       <c r="W58" s="136">
         <v>1</v>
       </c>
-      <c r="X58" s="82"/>
-      <c r="Y58" s="84"/>
-      <c r="AA58" s="86"/>
-      <c r="AB58" s="87"/>
-      <c r="AC58" s="87"/>
-    </row>
-    <row r="59" spans="1:29" s="25" customFormat="1" ht="4.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="X58" s="136">
+        <v>1</v>
+      </c>
+      <c r="Y58" s="136">
+        <v>1</v>
+      </c>
+      <c r="Z58" s="136">
+        <v>1</v>
+      </c>
+      <c r="AA58" s="136">
+        <v>1</v>
+      </c>
+      <c r="AB58" s="136">
+        <v>1</v>
+      </c>
+      <c r="AC58" s="82"/>
+      <c r="AD58" s="84"/>
+      <c r="AF58" s="86"/>
+      <c r="AG58" s="87"/>
+      <c r="AH58" s="87"/>
+    </row>
+    <row r="59" spans="1:34" s="25" customFormat="1" ht="4.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="88"/>
       <c r="C59" s="89"/>
       <c r="D59" s="178"/>
-      <c r="E59" s="188" t="s">
+      <c r="E59" s="224" t="s">
         <v>42</v>
       </c>
       <c r="F59" s="178"/>
@@ -6138,230 +6606,275 @@
       <c r="U59" s="94"/>
       <c r="V59" s="94"/>
       <c r="W59" s="94"/>
-      <c r="X59" s="93"/>
-      <c r="Y59" s="95"/>
-      <c r="Z59" s="2"/>
-      <c r="AA59" s="31"/>
-      <c r="AB59" s="32"/>
-      <c r="AC59" s="32"/>
-    </row>
-    <row r="60" spans="1:29" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="205" t="s">
+      <c r="X59" s="94"/>
+      <c r="Y59" s="94"/>
+      <c r="Z59" s="94"/>
+      <c r="AA59" s="94"/>
+      <c r="AB59" s="94"/>
+      <c r="AC59" s="93"/>
+      <c r="AD59" s="95"/>
+      <c r="AE59" s="2"/>
+      <c r="AF59" s="31"/>
+      <c r="AG59" s="32"/>
+      <c r="AH59" s="32"/>
+    </row>
+    <row r="60" spans="1:34" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B60" s="212" t="s">
         <v>39</v>
       </c>
-      <c r="C60" s="205" t="s">
+      <c r="C60" s="212" t="s">
         <v>40</v>
       </c>
-      <c r="D60" s="186" t="s">
+      <c r="D60" s="215" t="s">
         <v>41</v>
       </c>
-      <c r="E60" s="189"/>
-      <c r="F60" s="186" t="s">
+      <c r="E60" s="225"/>
+      <c r="F60" s="215" t="s">
         <v>43</v>
       </c>
-      <c r="G60" s="186" t="s">
+      <c r="G60" s="215" t="s">
         <v>44</v>
       </c>
-      <c r="H60" s="186" t="s">
+      <c r="H60" s="215" t="s">
         <v>45</v>
       </c>
-      <c r="I60" s="186"/>
+      <c r="I60" s="215"/>
       <c r="J60" s="101"/>
       <c r="K60" s="96"/>
       <c r="L60" s="97"/>
       <c r="M60" s="97"/>
-      <c r="N60" s="208">
+      <c r="N60" s="186">
         <v>46099</v>
       </c>
-      <c r="O60" s="208">
+      <c r="O60" s="186">
         <v>46100</v>
       </c>
-      <c r="P60" s="208">
+      <c r="P60" s="186">
         <v>46101</v>
       </c>
-      <c r="Q60" s="208">
+      <c r="Q60" s="186">
         <v>46102</v>
       </c>
-      <c r="R60" s="208">
+      <c r="R60" s="186">
         <v>46103</v>
       </c>
-      <c r="S60" s="208">
+      <c r="S60" s="186">
         <v>46104</v>
       </c>
-      <c r="T60" s="208">
+      <c r="T60" s="186">
         <v>46105</v>
       </c>
-      <c r="U60" s="208">
-        <v>46106</v>
-      </c>
-      <c r="V60" s="208">
-        <v>46107</v>
-      </c>
-      <c r="W60" s="208">
+      <c r="U60" s="227">
         <v>46108</v>
       </c>
-      <c r="X60" s="212" t="s">
+      <c r="V60" s="227">
+        <v>46109</v>
+      </c>
+      <c r="W60" s="227">
+        <v>46110</v>
+      </c>
+      <c r="X60" s="227">
+        <v>46111</v>
+      </c>
+      <c r="Y60" s="227">
+        <v>46112</v>
+      </c>
+      <c r="Z60" s="227">
+        <v>46113</v>
+      </c>
+      <c r="AA60" s="227">
+        <v>46114</v>
+      </c>
+      <c r="AB60" s="227">
+        <v>46115</v>
+      </c>
+      <c r="AC60" s="219" t="s">
         <v>18</v>
       </c>
-      <c r="Y60" s="224" t="s">
+      <c r="AD60" s="188" t="s">
         <v>19</v>
       </c>
-      <c r="AA60" s="31"/>
-      <c r="AB60" s="32"/>
-      <c r="AC60" s="32"/>
-    </row>
-    <row r="61" spans="1:29" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="206"/>
-      <c r="C61" s="206"/>
-      <c r="D61" s="186"/>
-      <c r="E61" s="189"/>
-      <c r="F61" s="186"/>
-      <c r="G61" s="186"/>
-      <c r="H61" s="186"/>
-      <c r="I61" s="186"/>
+      <c r="AF60" s="31"/>
+      <c r="AG60" s="32"/>
+      <c r="AH60" s="32"/>
+    </row>
+    <row r="61" spans="1:34" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B61" s="213"/>
+      <c r="C61" s="213"/>
+      <c r="D61" s="215"/>
+      <c r="E61" s="225"/>
+      <c r="F61" s="215"/>
+      <c r="G61" s="215"/>
+      <c r="H61" s="215"/>
+      <c r="I61" s="215"/>
       <c r="J61" s="101"/>
       <c r="K61" s="98"/>
       <c r="L61" s="97"/>
       <c r="M61" s="97"/>
-      <c r="N61" s="208"/>
-      <c r="O61" s="208"/>
-      <c r="P61" s="208"/>
-      <c r="Q61" s="208"/>
-      <c r="R61" s="208"/>
-      <c r="S61" s="208"/>
-      <c r="T61" s="208"/>
-      <c r="U61" s="208"/>
-      <c r="V61" s="208"/>
-      <c r="W61" s="208"/>
-      <c r="X61" s="213"/>
-      <c r="Y61" s="225"/>
-      <c r="AA61" s="31"/>
-      <c r="AB61" s="32"/>
-      <c r="AC61" s="32"/>
-    </row>
-    <row r="62" spans="1:29" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B62" s="206"/>
-      <c r="C62" s="206"/>
-      <c r="D62" s="186"/>
-      <c r="E62" s="189"/>
-      <c r="F62" s="186"/>
-      <c r="G62" s="186"/>
-      <c r="H62" s="186"/>
-      <c r="I62" s="186"/>
+      <c r="N61" s="186"/>
+      <c r="O61" s="186"/>
+      <c r="P61" s="186"/>
+      <c r="Q61" s="186"/>
+      <c r="R61" s="186"/>
+      <c r="S61" s="186"/>
+      <c r="T61" s="186"/>
+      <c r="U61" s="227"/>
+      <c r="V61" s="227"/>
+      <c r="W61" s="227"/>
+      <c r="X61" s="227"/>
+      <c r="Y61" s="227"/>
+      <c r="Z61" s="227"/>
+      <c r="AA61" s="227"/>
+      <c r="AB61" s="227"/>
+      <c r="AC61" s="220"/>
+      <c r="AD61" s="189"/>
+      <c r="AF61" s="31"/>
+      <c r="AG61" s="32"/>
+      <c r="AH61" s="32"/>
+    </row>
+    <row r="62" spans="1:34" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B62" s="213"/>
+      <c r="C62" s="213"/>
+      <c r="D62" s="215"/>
+      <c r="E62" s="225"/>
+      <c r="F62" s="215"/>
+      <c r="G62" s="215"/>
+      <c r="H62" s="215"/>
+      <c r="I62" s="215"/>
       <c r="J62" s="101"/>
       <c r="K62" s="98"/>
       <c r="L62" s="97"/>
       <c r="M62" s="97"/>
-      <c r="N62" s="208"/>
-      <c r="O62" s="208"/>
-      <c r="P62" s="208"/>
-      <c r="Q62" s="208"/>
-      <c r="R62" s="208"/>
-      <c r="S62" s="208"/>
-      <c r="T62" s="208"/>
-      <c r="U62" s="208"/>
-      <c r="V62" s="208"/>
-      <c r="W62" s="208"/>
-      <c r="X62" s="213"/>
-      <c r="Y62" s="225"/>
-      <c r="AA62" s="31"/>
-      <c r="AB62" s="32"/>
-      <c r="AC62" s="32"/>
-    </row>
-    <row r="63" spans="1:29" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B63" s="206"/>
-      <c r="C63" s="206"/>
-      <c r="D63" s="186"/>
-      <c r="E63" s="189"/>
-      <c r="F63" s="186"/>
-      <c r="G63" s="186"/>
-      <c r="H63" s="186"/>
-      <c r="I63" s="186"/>
+      <c r="N62" s="186"/>
+      <c r="O62" s="186"/>
+      <c r="P62" s="186"/>
+      <c r="Q62" s="186"/>
+      <c r="R62" s="186"/>
+      <c r="S62" s="186"/>
+      <c r="T62" s="186"/>
+      <c r="U62" s="227"/>
+      <c r="V62" s="227"/>
+      <c r="W62" s="227"/>
+      <c r="X62" s="227"/>
+      <c r="Y62" s="227"/>
+      <c r="Z62" s="227"/>
+      <c r="AA62" s="227"/>
+      <c r="AB62" s="227"/>
+      <c r="AC62" s="220"/>
+      <c r="AD62" s="189"/>
+      <c r="AF62" s="31"/>
+      <c r="AG62" s="32"/>
+      <c r="AH62" s="32"/>
+    </row>
+    <row r="63" spans="1:34" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B63" s="213"/>
+      <c r="C63" s="213"/>
+      <c r="D63" s="215"/>
+      <c r="E63" s="225"/>
+      <c r="F63" s="215"/>
+      <c r="G63" s="215"/>
+      <c r="H63" s="215"/>
+      <c r="I63" s="215"/>
       <c r="J63" s="101"/>
       <c r="K63" s="99"/>
       <c r="L63" s="97"/>
       <c r="M63" s="97"/>
-      <c r="N63" s="208"/>
-      <c r="O63" s="208"/>
-      <c r="P63" s="208"/>
-      <c r="Q63" s="208"/>
-      <c r="R63" s="208"/>
-      <c r="S63" s="208"/>
-      <c r="T63" s="208"/>
-      <c r="U63" s="208"/>
-      <c r="V63" s="208"/>
-      <c r="W63" s="208"/>
-      <c r="X63" s="213"/>
-      <c r="Y63" s="225"/>
-      <c r="AB63" s="32"/>
-      <c r="AC63" s="32"/>
-    </row>
-    <row r="64" spans="1:29" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B64" s="206"/>
-      <c r="C64" s="206"/>
-      <c r="D64" s="186"/>
-      <c r="E64" s="189"/>
-      <c r="F64" s="186"/>
-      <c r="G64" s="186"/>
-      <c r="H64" s="186"/>
-      <c r="I64" s="186"/>
+      <c r="N63" s="186"/>
+      <c r="O63" s="186"/>
+      <c r="P63" s="186"/>
+      <c r="Q63" s="186"/>
+      <c r="R63" s="186"/>
+      <c r="S63" s="186"/>
+      <c r="T63" s="186"/>
+      <c r="U63" s="227"/>
+      <c r="V63" s="227"/>
+      <c r="W63" s="227"/>
+      <c r="X63" s="227"/>
+      <c r="Y63" s="227"/>
+      <c r="Z63" s="227"/>
+      <c r="AA63" s="227"/>
+      <c r="AB63" s="227"/>
+      <c r="AC63" s="220"/>
+      <c r="AD63" s="189"/>
+      <c r="AG63" s="32"/>
+      <c r="AH63" s="32"/>
+    </row>
+    <row r="64" spans="1:34" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B64" s="213"/>
+      <c r="C64" s="213"/>
+      <c r="D64" s="215"/>
+      <c r="E64" s="225"/>
+      <c r="F64" s="215"/>
+      <c r="G64" s="215"/>
+      <c r="H64" s="215"/>
+      <c r="I64" s="215"/>
       <c r="J64" s="101"/>
       <c r="K64" s="96"/>
       <c r="L64" s="97"/>
       <c r="M64" s="97"/>
-      <c r="N64" s="208"/>
-      <c r="O64" s="208"/>
-      <c r="P64" s="208"/>
-      <c r="Q64" s="208"/>
-      <c r="R64" s="208"/>
-      <c r="S64" s="208"/>
-      <c r="T64" s="208"/>
-      <c r="U64" s="208"/>
-      <c r="V64" s="208"/>
-      <c r="W64" s="208"/>
-      <c r="X64" s="213"/>
-      <c r="Y64" s="225"/>
-      <c r="AB64" s="32"/>
-      <c r="AC64" s="32"/>
-    </row>
-    <row r="65" spans="2:29" ht="12.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B65" s="206"/>
-      <c r="C65" s="206"/>
-      <c r="D65" s="186"/>
-      <c r="E65" s="189"/>
-      <c r="F65" s="186"/>
-      <c r="G65" s="186"/>
-      <c r="H65" s="186"/>
-      <c r="I65" s="186"/>
+      <c r="N64" s="186"/>
+      <c r="O64" s="186"/>
+      <c r="P64" s="186"/>
+      <c r="Q64" s="186"/>
+      <c r="R64" s="186"/>
+      <c r="S64" s="186"/>
+      <c r="T64" s="186"/>
+      <c r="U64" s="227"/>
+      <c r="V64" s="227"/>
+      <c r="W64" s="227"/>
+      <c r="X64" s="227"/>
+      <c r="Y64" s="227"/>
+      <c r="Z64" s="227"/>
+      <c r="AA64" s="227"/>
+      <c r="AB64" s="227"/>
+      <c r="AC64" s="220"/>
+      <c r="AD64" s="189"/>
+      <c r="AG64" s="32"/>
+      <c r="AH64" s="32"/>
+    </row>
+    <row r="65" spans="2:34" ht="12.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B65" s="213"/>
+      <c r="C65" s="213"/>
+      <c r="D65" s="215"/>
+      <c r="E65" s="225"/>
+      <c r="F65" s="215"/>
+      <c r="G65" s="215"/>
+      <c r="H65" s="215"/>
+      <c r="I65" s="215"/>
       <c r="J65" s="101"/>
       <c r="K65" s="100"/>
       <c r="L65" s="97"/>
       <c r="M65" s="97"/>
-      <c r="N65" s="209"/>
-      <c r="O65" s="209"/>
-      <c r="P65" s="209"/>
-      <c r="Q65" s="209"/>
-      <c r="R65" s="209"/>
-      <c r="S65" s="209"/>
-      <c r="T65" s="209"/>
-      <c r="U65" s="209"/>
-      <c r="V65" s="209"/>
-      <c r="W65" s="209"/>
-      <c r="X65" s="214"/>
-      <c r="Y65" s="226"/>
-      <c r="AA65" s="23"/>
-      <c r="AB65" s="23"/>
-      <c r="AC65" s="23"/>
-    </row>
-    <row r="66" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="206"/>
-      <c r="C66" s="206"/>
-      <c r="D66" s="186"/>
-      <c r="E66" s="189"/>
-      <c r="F66" s="186"/>
-      <c r="G66" s="186"/>
-      <c r="H66" s="186"/>
-      <c r="I66" s="186"/>
+      <c r="N65" s="187"/>
+      <c r="O65" s="187"/>
+      <c r="P65" s="187"/>
+      <c r="Q65" s="187"/>
+      <c r="R65" s="187"/>
+      <c r="S65" s="187"/>
+      <c r="T65" s="187"/>
+      <c r="U65" s="228"/>
+      <c r="V65" s="228"/>
+      <c r="W65" s="228"/>
+      <c r="X65" s="228"/>
+      <c r="Y65" s="228"/>
+      <c r="Z65" s="228"/>
+      <c r="AA65" s="228"/>
+      <c r="AB65" s="228"/>
+      <c r="AC65" s="221"/>
+      <c r="AD65" s="190"/>
+      <c r="AF65" s="23"/>
+      <c r="AG65" s="23"/>
+      <c r="AH65" s="23"/>
+    </row>
+    <row r="66" spans="2:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B66" s="213"/>
+      <c r="C66" s="213"/>
+      <c r="D66" s="215"/>
+      <c r="E66" s="225"/>
+      <c r="F66" s="215"/>
+      <c r="G66" s="215"/>
+      <c r="H66" s="215"/>
+      <c r="I66" s="215"/>
       <c r="J66" s="101"/>
       <c r="K66" s="100"/>
       <c r="L66" s="100"/>
@@ -6377,22 +6890,27 @@
       <c r="V66" s="103"/>
       <c r="W66" s="103"/>
       <c r="X66" s="103"/>
-      <c r="Y66" s="104"/>
-      <c r="AA66" s="23"/>
-      <c r="AB66" s="217" t="s">
+      <c r="Y66" s="103"/>
+      <c r="Z66" s="103"/>
+      <c r="AA66" s="103"/>
+      <c r="AB66" s="103"/>
+      <c r="AC66" s="103"/>
+      <c r="AD66" s="104"/>
+      <c r="AF66" s="23"/>
+      <c r="AG66" s="191" t="s">
         <v>6</v>
       </c>
-      <c r="AC66" s="217"/>
-    </row>
-    <row r="67" spans="2:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B67" s="206"/>
-      <c r="C67" s="206"/>
-      <c r="D67" s="186"/>
-      <c r="E67" s="189"/>
-      <c r="F67" s="186"/>
-      <c r="G67" s="186"/>
-      <c r="H67" s="186"/>
-      <c r="I67" s="186"/>
+      <c r="AH66" s="191"/>
+    </row>
+    <row r="67" spans="2:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B67" s="213"/>
+      <c r="C67" s="213"/>
+      <c r="D67" s="215"/>
+      <c r="E67" s="225"/>
+      <c r="F67" s="215"/>
+      <c r="G67" s="215"/>
+      <c r="H67" s="215"/>
+      <c r="I67" s="215"/>
       <c r="J67" s="105"/>
       <c r="K67" s="100"/>
       <c r="L67" s="98"/>
@@ -6408,26 +6926,31 @@
       <c r="V67" s="107"/>
       <c r="W67" s="107"/>
       <c r="X67" s="107"/>
-      <c r="Y67" s="108"/>
-      <c r="AA67" s="109" t="s">
+      <c r="Y67" s="107"/>
+      <c r="Z67" s="107"/>
+      <c r="AA67" s="107"/>
+      <c r="AB67" s="107"/>
+      <c r="AC67" s="107"/>
+      <c r="AD67" s="108"/>
+      <c r="AF67" s="109" t="s">
         <v>7</v>
       </c>
-      <c r="AB67" s="110" t="s">
+      <c r="AG67" s="110" t="s">
         <v>8</v>
       </c>
-      <c r="AC67" s="110" t="s">
+      <c r="AH67" s="110" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="68" spans="2:29" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B68" s="206"/>
-      <c r="C68" s="206"/>
-      <c r="D68" s="186"/>
-      <c r="E68" s="189"/>
-      <c r="F68" s="186"/>
-      <c r="G68" s="186"/>
-      <c r="H68" s="186"/>
-      <c r="I68" s="186"/>
+    <row r="68" spans="2:34" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B68" s="213"/>
+      <c r="C68" s="213"/>
+      <c r="D68" s="215"/>
+      <c r="E68" s="225"/>
+      <c r="F68" s="215"/>
+      <c r="G68" s="215"/>
+      <c r="H68" s="215"/>
+      <c r="I68" s="215"/>
       <c r="J68" s="101"/>
       <c r="K68" s="96"/>
       <c r="L68" s="98"/>
@@ -6443,22 +6966,27 @@
       <c r="V68" s="107"/>
       <c r="W68" s="107"/>
       <c r="X68" s="107"/>
-      <c r="Y68" s="108"/>
-      <c r="AA68" s="23" t="s">
+      <c r="Y68" s="107"/>
+      <c r="Z68" s="107"/>
+      <c r="AA68" s="107"/>
+      <c r="AB68" s="107"/>
+      <c r="AC68" s="107"/>
+      <c r="AD68" s="108"/>
+      <c r="AF68" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="AB68" s="148"/>
-      <c r="AC68" s="111"/>
-    </row>
-    <row r="69" spans="2:29" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B69" s="206"/>
-      <c r="C69" s="206"/>
-      <c r="D69" s="186"/>
-      <c r="E69" s="189"/>
-      <c r="F69" s="186"/>
-      <c r="G69" s="186"/>
-      <c r="H69" s="186"/>
-      <c r="I69" s="186"/>
+      <c r="AG68" s="148"/>
+      <c r="AH68" s="111"/>
+    </row>
+    <row r="69" spans="2:34" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B69" s="213"/>
+      <c r="C69" s="213"/>
+      <c r="D69" s="215"/>
+      <c r="E69" s="225"/>
+      <c r="F69" s="215"/>
+      <c r="G69" s="215"/>
+      <c r="H69" s="215"/>
+      <c r="I69" s="215"/>
       <c r="J69" s="101"/>
       <c r="K69" s="96"/>
       <c r="L69" s="98"/>
@@ -6474,22 +7002,27 @@
       <c r="V69" s="107"/>
       <c r="W69" s="107"/>
       <c r="X69" s="107"/>
-      <c r="Y69" s="108"/>
-      <c r="AA69" s="23" t="s">
+      <c r="Y69" s="107"/>
+      <c r="Z69" s="107"/>
+      <c r="AA69" s="107"/>
+      <c r="AB69" s="107"/>
+      <c r="AC69" s="107"/>
+      <c r="AD69" s="108"/>
+      <c r="AF69" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="AB69" s="148"/>
-      <c r="AC69" s="113"/>
-    </row>
-    <row r="70" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B70" s="206"/>
-      <c r="C70" s="206"/>
-      <c r="D70" s="186"/>
-      <c r="E70" s="189"/>
-      <c r="F70" s="186"/>
-      <c r="G70" s="186"/>
-      <c r="H70" s="186"/>
-      <c r="I70" s="186"/>
+      <c r="AG69" s="148"/>
+      <c r="AH69" s="113"/>
+    </row>
+    <row r="70" spans="2:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B70" s="213"/>
+      <c r="C70" s="213"/>
+      <c r="D70" s="215"/>
+      <c r="E70" s="225"/>
+      <c r="F70" s="215"/>
+      <c r="G70" s="215"/>
+      <c r="H70" s="215"/>
+      <c r="I70" s="215"/>
       <c r="J70" s="101"/>
       <c r="K70" s="96"/>
       <c r="L70" s="96"/>
@@ -6505,22 +7038,27 @@
       <c r="V70" s="107"/>
       <c r="W70" s="107"/>
       <c r="X70" s="107"/>
-      <c r="Y70" s="108"/>
-      <c r="AA70" s="23" t="s">
+      <c r="Y70" s="107"/>
+      <c r="Z70" s="107"/>
+      <c r="AA70" s="107"/>
+      <c r="AB70" s="107"/>
+      <c r="AC70" s="107"/>
+      <c r="AD70" s="108"/>
+      <c r="AF70" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="AB70" s="148"/>
-      <c r="AC70" s="111"/>
-    </row>
-    <row r="71" spans="2:29" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B71" s="206"/>
-      <c r="C71" s="206"/>
-      <c r="D71" s="186"/>
-      <c r="E71" s="189"/>
-      <c r="F71" s="186"/>
-      <c r="G71" s="186"/>
-      <c r="H71" s="186"/>
-      <c r="I71" s="186"/>
+      <c r="AG70" s="148"/>
+      <c r="AH70" s="111"/>
+    </row>
+    <row r="71" spans="2:34" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B71" s="213"/>
+      <c r="C71" s="213"/>
+      <c r="D71" s="215"/>
+      <c r="E71" s="225"/>
+      <c r="F71" s="215"/>
+      <c r="G71" s="215"/>
+      <c r="H71" s="215"/>
+      <c r="I71" s="215"/>
       <c r="J71" s="101"/>
       <c r="K71" s="114"/>
       <c r="L71" s="101"/>
@@ -6536,19 +7074,24 @@
       <c r="V71" s="107"/>
       <c r="W71" s="107"/>
       <c r="X71" s="107"/>
-      <c r="Y71" s="108"/>
-      <c r="AA71" s="23"/>
-      <c r="AB71" s="115"/>
-    </row>
-    <row r="72" spans="2:29" ht="15.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B72" s="206"/>
-      <c r="C72" s="206"/>
-      <c r="D72" s="186"/>
-      <c r="E72" s="189"/>
-      <c r="F72" s="186"/>
-      <c r="G72" s="186"/>
-      <c r="H72" s="186"/>
-      <c r="I72" s="186"/>
+      <c r="Y71" s="107"/>
+      <c r="Z71" s="107"/>
+      <c r="AA71" s="107"/>
+      <c r="AB71" s="107"/>
+      <c r="AC71" s="107"/>
+      <c r="AD71" s="108"/>
+      <c r="AF71" s="23"/>
+      <c r="AG71" s="115"/>
+    </row>
+    <row r="72" spans="2:34" ht="15.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B72" s="213"/>
+      <c r="C72" s="213"/>
+      <c r="D72" s="215"/>
+      <c r="E72" s="225"/>
+      <c r="F72" s="215"/>
+      <c r="G72" s="215"/>
+      <c r="H72" s="215"/>
+      <c r="I72" s="215"/>
       <c r="J72" s="117"/>
       <c r="K72" s="116"/>
       <c r="L72" s="117"/>
@@ -6564,123 +7107,148 @@
       <c r="V72" s="119"/>
       <c r="W72" s="119"/>
       <c r="X72" s="119"/>
-      <c r="Y72" s="120"/>
-      <c r="AB72" s="115"/>
-      <c r="AC72" s="115"/>
-    </row>
-    <row r="73" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B73" s="206"/>
-      <c r="C73" s="206"/>
-      <c r="D73" s="186"/>
-      <c r="E73" s="189"/>
-      <c r="F73" s="186"/>
-      <c r="G73" s="186"/>
-      <c r="H73" s="186"/>
-      <c r="I73" s="186"/>
-      <c r="J73" s="218"/>
-      <c r="K73" s="218"/>
-      <c r="L73" s="218"/>
-      <c r="M73" s="218"/>
-      <c r="N73" s="218"/>
-      <c r="O73" s="218"/>
-      <c r="P73" s="218"/>
-      <c r="Q73" s="218"/>
-      <c r="R73" s="218"/>
-      <c r="S73" s="218"/>
-      <c r="T73" s="218"/>
-      <c r="U73" s="218"/>
-      <c r="V73" s="218"/>
-      <c r="W73" s="218"/>
-      <c r="X73" s="218"/>
-      <c r="Y73" s="219"/>
-    </row>
-    <row r="74" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B74" s="206"/>
-      <c r="C74" s="206"/>
-      <c r="D74" s="186"/>
-      <c r="E74" s="189"/>
-      <c r="F74" s="186"/>
-      <c r="G74" s="186"/>
-      <c r="H74" s="186"/>
-      <c r="I74" s="186"/>
-      <c r="J74" s="220"/>
-      <c r="K74" s="220"/>
-      <c r="L74" s="220"/>
-      <c r="M74" s="220"/>
-      <c r="N74" s="220"/>
-      <c r="O74" s="220"/>
-      <c r="P74" s="220"/>
-      <c r="Q74" s="220"/>
-      <c r="R74" s="220"/>
-      <c r="S74" s="220"/>
-      <c r="T74" s="220"/>
-      <c r="U74" s="220"/>
-      <c r="V74" s="220"/>
-      <c r="W74" s="220"/>
-      <c r="X74" s="220"/>
-      <c r="Y74" s="221"/>
-    </row>
-    <row r="75" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B75" s="206"/>
-      <c r="C75" s="206"/>
-      <c r="D75" s="186"/>
-      <c r="E75" s="189"/>
-      <c r="F75" s="186"/>
-      <c r="G75" s="186"/>
-      <c r="H75" s="186"/>
-      <c r="I75" s="186"/>
-      <c r="J75" s="220"/>
-      <c r="K75" s="220"/>
-      <c r="L75" s="220"/>
-      <c r="M75" s="220"/>
-      <c r="N75" s="220"/>
-      <c r="O75" s="220"/>
-      <c r="P75" s="220"/>
-      <c r="Q75" s="220"/>
-      <c r="R75" s="220"/>
-      <c r="S75" s="220"/>
-      <c r="T75" s="220"/>
-      <c r="U75" s="220"/>
-      <c r="V75" s="220"/>
-      <c r="W75" s="220"/>
-      <c r="X75" s="220"/>
-      <c r="Y75" s="221"/>
-    </row>
-    <row r="76" spans="2:29" s="1" customFormat="1" ht="15.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B76" s="207"/>
-      <c r="C76" s="207"/>
-      <c r="D76" s="187"/>
-      <c r="E76" s="190"/>
-      <c r="F76" s="187"/>
-      <c r="G76" s="187"/>
-      <c r="H76" s="187"/>
-      <c r="I76" s="187"/>
-      <c r="J76" s="210"/>
-      <c r="K76" s="210"/>
-      <c r="L76" s="210"/>
-      <c r="M76" s="210"/>
-      <c r="N76" s="210"/>
-      <c r="O76" s="210"/>
-      <c r="P76" s="210"/>
-      <c r="Q76" s="210"/>
-      <c r="R76" s="210"/>
-      <c r="S76" s="210"/>
-      <c r="T76" s="210"/>
-      <c r="U76" s="210"/>
-      <c r="V76" s="210"/>
-      <c r="W76" s="210"/>
-      <c r="X76" s="210"/>
-      <c r="Y76" s="211"/>
-      <c r="AA76" s="23"/>
-      <c r="AB76" s="24"/>
-      <c r="AC76" s="24"/>
-    </row>
-    <row r="77" spans="2:29" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="AA77" s="23"/>
-      <c r="AB77" s="24"/>
-      <c r="AC77" s="24"/>
-    </row>
-    <row r="78" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="Y72" s="119"/>
+      <c r="Z72" s="119"/>
+      <c r="AA72" s="119"/>
+      <c r="AB72" s="119"/>
+      <c r="AC72" s="119"/>
+      <c r="AD72" s="120"/>
+      <c r="AG72" s="115"/>
+      <c r="AH72" s="115"/>
+    </row>
+    <row r="73" spans="2:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B73" s="213"/>
+      <c r="C73" s="213"/>
+      <c r="D73" s="215"/>
+      <c r="E73" s="225"/>
+      <c r="F73" s="215"/>
+      <c r="G73" s="215"/>
+      <c r="H73" s="215"/>
+      <c r="I73" s="215"/>
+      <c r="J73" s="192"/>
+      <c r="K73" s="192"/>
+      <c r="L73" s="192"/>
+      <c r="M73" s="192"/>
+      <c r="N73" s="192"/>
+      <c r="O73" s="192"/>
+      <c r="P73" s="192"/>
+      <c r="Q73" s="192"/>
+      <c r="R73" s="192"/>
+      <c r="S73" s="192"/>
+      <c r="T73" s="192"/>
+      <c r="U73" s="192"/>
+      <c r="V73" s="192"/>
+      <c r="W73" s="192"/>
+      <c r="X73" s="192"/>
+      <c r="Y73" s="192"/>
+      <c r="Z73" s="192"/>
+      <c r="AA73" s="192"/>
+      <c r="AB73" s="192"/>
+      <c r="AC73" s="192"/>
+      <c r="AD73" s="193"/>
+    </row>
+    <row r="74" spans="2:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B74" s="213"/>
+      <c r="C74" s="213"/>
+      <c r="D74" s="215"/>
+      <c r="E74" s="225"/>
+      <c r="F74" s="215"/>
+      <c r="G74" s="215"/>
+      <c r="H74" s="215"/>
+      <c r="I74" s="215"/>
+      <c r="J74" s="194"/>
+      <c r="K74" s="194"/>
+      <c r="L74" s="194"/>
+      <c r="M74" s="194"/>
+      <c r="N74" s="194"/>
+      <c r="O74" s="194"/>
+      <c r="P74" s="194"/>
+      <c r="Q74" s="194"/>
+      <c r="R74" s="194"/>
+      <c r="S74" s="194"/>
+      <c r="T74" s="194"/>
+      <c r="U74" s="194"/>
+      <c r="V74" s="194"/>
+      <c r="W74" s="194"/>
+      <c r="X74" s="194"/>
+      <c r="Y74" s="194"/>
+      <c r="Z74" s="194"/>
+      <c r="AA74" s="194"/>
+      <c r="AB74" s="194"/>
+      <c r="AC74" s="194"/>
+      <c r="AD74" s="195"/>
+    </row>
+    <row r="75" spans="2:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B75" s="213"/>
+      <c r="C75" s="213"/>
+      <c r="D75" s="215"/>
+      <c r="E75" s="225"/>
+      <c r="F75" s="215"/>
+      <c r="G75" s="215"/>
+      <c r="H75" s="215"/>
+      <c r="I75" s="215"/>
+      <c r="J75" s="194"/>
+      <c r="K75" s="194"/>
+      <c r="L75" s="194"/>
+      <c r="M75" s="194"/>
+      <c r="N75" s="194"/>
+      <c r="O75" s="194"/>
+      <c r="P75" s="194"/>
+      <c r="Q75" s="194"/>
+      <c r="R75" s="194"/>
+      <c r="S75" s="194"/>
+      <c r="T75" s="194"/>
+      <c r="U75" s="194"/>
+      <c r="V75" s="194"/>
+      <c r="W75" s="194"/>
+      <c r="X75" s="194"/>
+      <c r="Y75" s="194"/>
+      <c r="Z75" s="194"/>
+      <c r="AA75" s="194"/>
+      <c r="AB75" s="194"/>
+      <c r="AC75" s="194"/>
+      <c r="AD75" s="195"/>
+    </row>
+    <row r="76" spans="2:34" s="1" customFormat="1" ht="15.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B76" s="214"/>
+      <c r="C76" s="214"/>
+      <c r="D76" s="216"/>
+      <c r="E76" s="226"/>
+      <c r="F76" s="216"/>
+      <c r="G76" s="216"/>
+      <c r="H76" s="216"/>
+      <c r="I76" s="216"/>
+      <c r="J76" s="217"/>
+      <c r="K76" s="217"/>
+      <c r="L76" s="217"/>
+      <c r="M76" s="217"/>
+      <c r="N76" s="217"/>
+      <c r="O76" s="217"/>
+      <c r="P76" s="217"/>
+      <c r="Q76" s="217"/>
+      <c r="R76" s="217"/>
+      <c r="S76" s="217"/>
+      <c r="T76" s="217"/>
+      <c r="U76" s="217"/>
+      <c r="V76" s="217"/>
+      <c r="W76" s="217"/>
+      <c r="X76" s="217"/>
+      <c r="Y76" s="217"/>
+      <c r="Z76" s="217"/>
+      <c r="AA76" s="217"/>
+      <c r="AB76" s="217"/>
+      <c r="AC76" s="217"/>
+      <c r="AD76" s="218"/>
+      <c r="AF76" s="23"/>
+      <c r="AG76" s="24"/>
+      <c r="AH76" s="24"/>
+    </row>
+    <row r="77" spans="2:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AF77" s="23"/>
+      <c r="AG77" s="24"/>
+      <c r="AH77" s="24"/>
+    </row>
+    <row r="78" spans="2:34" x14ac:dyDescent="0.25">
       <c r="M78" s="121"/>
       <c r="N78" s="121"/>
       <c r="O78" s="1"/>
@@ -6700,17 +7268,22 @@
       <c r="U78" s="131" t="s">
         <v>15</v>
       </c>
-      <c r="V78" s="222" t="s">
+      <c r="V78" s="196" t="s">
         <v>23</v>
       </c>
-      <c r="W78" s="223"/>
-      <c r="Y78" s="123"/>
-      <c r="Z78" s="123"/>
-      <c r="AA78" s="123"/>
-      <c r="AB78" s="123"/>
-      <c r="AC78" s="123"/>
-    </row>
-    <row r="79" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="W78" s="197"/>
+      <c r="X78" s="197"/>
+      <c r="Y78" s="197"/>
+      <c r="Z78" s="197"/>
+      <c r="AA78" s="197"/>
+      <c r="AB78" s="197"/>
+      <c r="AD78" s="123"/>
+      <c r="AE78" s="123"/>
+      <c r="AF78" s="123"/>
+      <c r="AG78" s="123"/>
+      <c r="AH78" s="123"/>
+    </row>
+    <row r="79" spans="2:34" x14ac:dyDescent="0.25">
       <c r="M79" s="121"/>
       <c r="N79" s="121"/>
       <c r="O79" s="4" t="s">
@@ -6732,17 +7305,22 @@
       <c r="U79" s="138" t="s">
         <v>16</v>
       </c>
-      <c r="V79" s="222" t="s">
+      <c r="V79" s="196" t="s">
         <v>24</v>
       </c>
-      <c r="W79" s="223"/>
-      <c r="Y79" s="125"/>
-      <c r="Z79" s="125"/>
-      <c r="AA79" s="125"/>
-      <c r="AB79" s="125"/>
-      <c r="AC79" s="125"/>
-    </row>
-    <row r="80" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="W79" s="197"/>
+      <c r="X79" s="197"/>
+      <c r="Y79" s="197"/>
+      <c r="Z79" s="197"/>
+      <c r="AA79" s="197"/>
+      <c r="AB79" s="197"/>
+      <c r="AD79" s="125"/>
+      <c r="AE79" s="125"/>
+      <c r="AF79" s="125"/>
+      <c r="AG79" s="125"/>
+      <c r="AH79" s="125"/>
+    </row>
+    <row r="80" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B80" s="1"/>
       <c r="C80" s="1"/>
       <c r="D80" s="1"/>
@@ -6765,17 +7343,22 @@
       <c r="U80" s="146" t="s">
         <v>17</v>
       </c>
-      <c r="V80" s="222" t="s">
+      <c r="V80" s="196" t="s">
         <v>25</v>
       </c>
-      <c r="W80" s="223"/>
-      <c r="Y80" s="121"/>
-      <c r="Z80" s="121"/>
-      <c r="AA80" s="121"/>
-      <c r="AB80" s="121"/>
-      <c r="AC80" s="121"/>
-    </row>
-    <row r="81" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="W80" s="197"/>
+      <c r="X80" s="197"/>
+      <c r="Y80" s="197"/>
+      <c r="Z80" s="197"/>
+      <c r="AA80" s="197"/>
+      <c r="AB80" s="197"/>
+      <c r="AD80" s="121"/>
+      <c r="AE80" s="121"/>
+      <c r="AF80" s="121"/>
+      <c r="AG80" s="121"/>
+      <c r="AH80" s="121"/>
+    </row>
+    <row r="81" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B81" s="1"/>
       <c r="C81" s="1"/>
       <c r="D81" s="1"/>
@@ -6804,149 +7387,170 @@
       <c r="AA81" s="1"/>
       <c r="AB81" s="1"/>
       <c r="AC81" s="1"/>
-    </row>
-    <row r="82" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="AD81" s="1"/>
+      <c r="AE81" s="1"/>
+      <c r="AF81" s="1"/>
+      <c r="AG81" s="1"/>
+      <c r="AH81" s="1"/>
+    </row>
+    <row r="82" spans="2:34" x14ac:dyDescent="0.25">
       <c r="P82" s="151"/>
       <c r="Q82" s="154" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="83" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:34" x14ac:dyDescent="0.25">
       <c r="P83" s="152"/>
       <c r="Q83" s="154" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="84" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:34" x14ac:dyDescent="0.25">
       <c r="P84" s="153"/>
       <c r="Q84" s="154" t="s">
         <v>29</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="33">
-    <mergeCell ref="S60:S65"/>
-    <mergeCell ref="T60:T65"/>
-    <mergeCell ref="U60:U65"/>
-    <mergeCell ref="V60:V65"/>
-    <mergeCell ref="Y60:Y65"/>
-    <mergeCell ref="AB66:AC66"/>
-    <mergeCell ref="J73:Y73"/>
-    <mergeCell ref="J74:Y74"/>
-    <mergeCell ref="V80:W80"/>
-    <mergeCell ref="J75:Y75"/>
-    <mergeCell ref="V79:W79"/>
-    <mergeCell ref="V78:W78"/>
-    <mergeCell ref="J3:Y4"/>
+  <mergeCells count="38">
+    <mergeCell ref="H60:H76"/>
+    <mergeCell ref="E59:E76"/>
+    <mergeCell ref="G60:G76"/>
+    <mergeCell ref="F60:F76"/>
+    <mergeCell ref="D60:D76"/>
+    <mergeCell ref="J3:AD4"/>
     <mergeCell ref="B5:I5"/>
-    <mergeCell ref="N5:W5"/>
-    <mergeCell ref="X5:Y5"/>
+    <mergeCell ref="N5:AB5"/>
+    <mergeCell ref="AC5:AD5"/>
     <mergeCell ref="B60:B76"/>
     <mergeCell ref="C60:C76"/>
     <mergeCell ref="I60:I76"/>
     <mergeCell ref="N60:N65"/>
     <mergeCell ref="O60:O65"/>
     <mergeCell ref="P60:P65"/>
-    <mergeCell ref="J76:Y76"/>
+    <mergeCell ref="J76:AD76"/>
     <mergeCell ref="W60:W65"/>
-    <mergeCell ref="X60:X65"/>
-    <mergeCell ref="X51:Y51"/>
+    <mergeCell ref="AC60:AC65"/>
+    <mergeCell ref="AC51:AD51"/>
     <mergeCell ref="Q60:Q65"/>
     <mergeCell ref="R60:R65"/>
-    <mergeCell ref="H60:H76"/>
-    <mergeCell ref="E59:E76"/>
-    <mergeCell ref="G60:G76"/>
-    <mergeCell ref="F60:F76"/>
-    <mergeCell ref="D60:D76"/>
+    <mergeCell ref="AG66:AH66"/>
+    <mergeCell ref="J73:AD73"/>
+    <mergeCell ref="J74:AD74"/>
+    <mergeCell ref="V80:AB80"/>
+    <mergeCell ref="J75:AD75"/>
+    <mergeCell ref="V79:AB79"/>
+    <mergeCell ref="V78:AB78"/>
+    <mergeCell ref="S60:S65"/>
+    <mergeCell ref="T60:T65"/>
+    <mergeCell ref="U60:U65"/>
+    <mergeCell ref="V60:V65"/>
+    <mergeCell ref="AD60:AD65"/>
+    <mergeCell ref="X60:X65"/>
+    <mergeCell ref="Y60:Y65"/>
+    <mergeCell ref="Z60:Z65"/>
+    <mergeCell ref="AA60:AA65"/>
+    <mergeCell ref="AB60:AB65"/>
   </mergeCells>
   <phoneticPr fontId="26" type="noConversion"/>
   <conditionalFormatting sqref="B59:D59 F59:I59">
-    <cfRule type="cellIs" dxfId="22" priority="58" stopIfTrue="1" operator="notEqual">
+    <cfRule type="cellIs" dxfId="25" priority="61" stopIfTrue="1" operator="notEqual">
       <formula>""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M79:N79 Y79:AC79">
-    <cfRule type="cellIs" dxfId="21" priority="62" stopIfTrue="1" operator="equal">
+  <conditionalFormatting sqref="M79:N79 AD79:AH79">
+    <cfRule type="cellIs" dxfId="24" priority="65" stopIfTrue="1" operator="equal">
       <formula>"G"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="63" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="66" stopIfTrue="1" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="64" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="67" stopIfTrue="1" operator="equal">
       <formula>"R"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N49:W58">
-    <cfRule type="cellIs" dxfId="18" priority="12" stopIfTrue="1" operator="equal">
+  <conditionalFormatting sqref="N49:AB58">
+    <cfRule type="cellIs" dxfId="21" priority="15" stopIfTrue="1" operator="equal">
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N49:W59">
-    <cfRule type="cellIs" dxfId="17" priority="10" stopIfTrue="1" operator="equal">
+  <conditionalFormatting sqref="N49:AB59">
+    <cfRule type="cellIs" dxfId="20" priority="13" stopIfTrue="1" operator="equal">
       <formula>"S"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="11" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="14" stopIfTrue="1" operator="equal">
       <formula>"C"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N59:W59">
-    <cfRule type="cellIs" dxfId="15" priority="61" stopIfTrue="1" operator="equal">
+  <conditionalFormatting sqref="N59:AB59">
+    <cfRule type="cellIs" dxfId="18" priority="64" stopIfTrue="1" operator="equal">
       <formula>"L"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O6:W7 T8:W13 N8:R15 U14:W15 N20:Q27 N16:W19">
-    <cfRule type="cellIs" dxfId="14" priority="49" stopIfTrue="1" operator="equal">
+  <conditionalFormatting sqref="O6:AB7 T8:AB13 N8:R15 U14:AB15 N16:AB19 N20:Q27">
+    <cfRule type="cellIs" dxfId="17" priority="52" stopIfTrue="1" operator="equal">
       <formula>"S"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="50" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="53" stopIfTrue="1" operator="equal">
       <formula>"C"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="51" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="54" stopIfTrue="1" operator="equal">
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R20:U25 W20:W48 S26:U27 N28:U28 N29:T48 V29:V48">
-    <cfRule type="cellIs" dxfId="11" priority="52" stopIfTrue="1" operator="equal">
+  <conditionalFormatting sqref="R20:U25 AB20:AB48 S26:U27 N28:U28 N29:T48 V28:AA48">
+    <cfRule type="cellIs" dxfId="14" priority="55" stopIfTrue="1" operator="equal">
       <formula>"S"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="53" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="56" stopIfTrue="1" operator="equal">
       <formula>"C"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="54" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="57" stopIfTrue="1" operator="equal">
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R79:W79">
-    <cfRule type="cellIs" dxfId="8" priority="25" stopIfTrue="1" operator="equal">
+  <conditionalFormatting sqref="R79:AB79">
+    <cfRule type="cellIs" dxfId="11" priority="28" stopIfTrue="1" operator="equal">
       <formula>"G"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="26" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="29" stopIfTrue="1" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="27" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="30" stopIfTrue="1" operator="equal">
       <formula>"R"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V20:V27">
-    <cfRule type="cellIs" dxfId="5" priority="1" stopIfTrue="1" operator="equal">
+  <conditionalFormatting sqref="V20:AA27">
+    <cfRule type="cellIs" dxfId="8" priority="4" stopIfTrue="1" operator="equal">
       <formula>"S"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="5" stopIfTrue="1" operator="equal">
       <formula>"C"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="6" stopIfTrue="1" operator="equal">
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X59:Y59">
-    <cfRule type="cellIs" dxfId="2" priority="55" stopIfTrue="1" operator="equal">
+  <conditionalFormatting sqref="AC59:AD59">
+    <cfRule type="cellIs" dxfId="5" priority="58" stopIfTrue="1" operator="equal">
       <formula>"A"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="56" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="59" stopIfTrue="1" operator="equal">
       <formula>"B"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="57" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="60" stopIfTrue="1" operator="equal">
       <formula>"C"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U29:U48">
+    <cfRule type="cellIs" dxfId="2" priority="1" stopIfTrue="1" operator="equal">
+      <formula>"S"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" stopIfTrue="1" operator="equal">
+      <formula>"C"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="3" stopIfTrue="1" operator="equal">
+      <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.5" right="0.5" top="0.65" bottom="0.35" header="0.4" footer="0.2"/>

</xml_diff>

<commit_message>
UC CRUD Company, Dashboard admin, update fix bug
</commit_message>
<xml_diff>
--- a/document/02_c_LAB301x_VN_v0.01_OPPM.xlsx
+++ b/document/02_c_LAB301x_VN_v0.01_OPPM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thanh\Downloads\FU\LAB\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FC2F255-4FA4-4393-A6FD-ECD4F8F52FBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0633200-05EF-440F-AEFC-654AE057DD2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2159,6 +2159,80 @@
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="66" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="65" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="56" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="56" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="49" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="169" fontId="5" fillId="0" borderId="56" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
       <protection locked="0"/>
@@ -2167,6 +2241,69 @@
       <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="59" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="60" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="73" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="74" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="49" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="71" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="72" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="63" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
       <protection locked="0"/>
@@ -2176,143 +2313,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="51" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="63" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="56" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="56" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="49" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="66" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="65" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="59" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="60" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="49" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="71" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="72" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="73" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="74" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -2328,36 +2328,6 @@
     <cellStyle name="Normal_Project Matrix Collection II" xfId="2" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
   </cellStyles>
   <dxfs count="26">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="mediumGray">
-          <fgColor indexed="10"/>
-          <bgColor indexed="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="mediumGray">
-          <fgColor indexed="42"/>
-          <bgColor indexed="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="mediumGray">
-          <fgColor indexed="43"/>
-          <bgColor indexed="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="mediumGray">
@@ -2536,6 +2506,36 @@
       <fill>
         <patternFill patternType="mediumGray">
           <fgColor indexed="10"/>
+          <bgColor indexed="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="mediumGray">
+          <fgColor indexed="10"/>
+          <bgColor indexed="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="mediumGray">
+          <fgColor indexed="42"/>
+          <bgColor indexed="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="mediumGray">
+          <fgColor indexed="43"/>
           <bgColor indexed="9"/>
         </patternFill>
       </fill>
@@ -3015,7 +3015,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:noFill/>
             </a14:hiddenFill>
           </a:ext>
@@ -3069,7 +3069,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:noFill/>
             </a14:hiddenFill>
           </a:ext>
@@ -3425,14 +3425,14 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="3175">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="3175">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -3491,7 +3491,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:noFill/>
             </a14:hiddenFill>
           </a:ext>
@@ -3545,7 +3545,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:noFill/>
             </a14:hiddenFill>
           </a:ext>
@@ -3599,7 +3599,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:noFill/>
             </a14:hiddenFill>
           </a:ext>
@@ -4339,29 +4339,29 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
       <c r="I3" s="17"/>
-      <c r="J3" s="198" t="s">
+      <c r="J3" s="191" t="s">
         <v>38</v>
       </c>
-      <c r="K3" s="199"/>
-      <c r="L3" s="199"/>
-      <c r="M3" s="199"/>
-      <c r="N3" s="199"/>
-      <c r="O3" s="199"/>
-      <c r="P3" s="199"/>
-      <c r="Q3" s="199"/>
-      <c r="R3" s="199"/>
-      <c r="S3" s="199"/>
-      <c r="T3" s="199"/>
-      <c r="U3" s="199"/>
-      <c r="V3" s="199"/>
-      <c r="W3" s="199"/>
-      <c r="X3" s="199"/>
-      <c r="Y3" s="199"/>
-      <c r="Z3" s="199"/>
-      <c r="AA3" s="199"/>
-      <c r="AB3" s="199"/>
-      <c r="AC3" s="199"/>
-      <c r="AD3" s="200"/>
+      <c r="K3" s="192"/>
+      <c r="L3" s="192"/>
+      <c r="M3" s="192"/>
+      <c r="N3" s="192"/>
+      <c r="O3" s="192"/>
+      <c r="P3" s="192"/>
+      <c r="Q3" s="192"/>
+      <c r="R3" s="192"/>
+      <c r="S3" s="192"/>
+      <c r="T3" s="192"/>
+      <c r="U3" s="192"/>
+      <c r="V3" s="192"/>
+      <c r="W3" s="192"/>
+      <c r="X3" s="192"/>
+      <c r="Y3" s="192"/>
+      <c r="Z3" s="192"/>
+      <c r="AA3" s="192"/>
+      <c r="AB3" s="192"/>
+      <c r="AC3" s="192"/>
+      <c r="AD3" s="193"/>
       <c r="AF3" s="13"/>
       <c r="AG3" s="14"/>
       <c r="AH3" s="14"/>
@@ -4375,69 +4375,69 @@
       <c r="G4" s="20"/>
       <c r="H4" s="20"/>
       <c r="I4" s="20"/>
-      <c r="J4" s="201"/>
-      <c r="K4" s="202"/>
-      <c r="L4" s="202"/>
-      <c r="M4" s="202"/>
-      <c r="N4" s="202"/>
-      <c r="O4" s="202"/>
-      <c r="P4" s="202"/>
-      <c r="Q4" s="202"/>
-      <c r="R4" s="202"/>
-      <c r="S4" s="202"/>
-      <c r="T4" s="202"/>
-      <c r="U4" s="202"/>
-      <c r="V4" s="202"/>
-      <c r="W4" s="202"/>
-      <c r="X4" s="202"/>
-      <c r="Y4" s="202"/>
-      <c r="Z4" s="202"/>
-      <c r="AA4" s="202"/>
-      <c r="AB4" s="202"/>
-      <c r="AC4" s="202"/>
-      <c r="AD4" s="203"/>
+      <c r="J4" s="194"/>
+      <c r="K4" s="195"/>
+      <c r="L4" s="195"/>
+      <c r="M4" s="195"/>
+      <c r="N4" s="195"/>
+      <c r="O4" s="195"/>
+      <c r="P4" s="195"/>
+      <c r="Q4" s="195"/>
+      <c r="R4" s="195"/>
+      <c r="S4" s="195"/>
+      <c r="T4" s="195"/>
+      <c r="U4" s="195"/>
+      <c r="V4" s="195"/>
+      <c r="W4" s="195"/>
+      <c r="X4" s="195"/>
+      <c r="Y4" s="195"/>
+      <c r="Z4" s="195"/>
+      <c r="AA4" s="195"/>
+      <c r="AB4" s="195"/>
+      <c r="AC4" s="195"/>
+      <c r="AD4" s="196"/>
       <c r="AF4" s="21"/>
       <c r="AG4" s="22"/>
       <c r="AH4" s="22"/>
     </row>
     <row r="5" spans="1:34" s="1" customFormat="1" ht="26.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="204" t="s">
+      <c r="B5" s="197" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="205"/>
-      <c r="D5" s="205"/>
-      <c r="E5" s="205"/>
-      <c r="F5" s="205"/>
-      <c r="G5" s="205"/>
-      <c r="H5" s="205"/>
-      <c r="I5" s="206"/>
+      <c r="C5" s="198"/>
+      <c r="D5" s="198"/>
+      <c r="E5" s="198"/>
+      <c r="F5" s="198"/>
+      <c r="G5" s="198"/>
+      <c r="H5" s="198"/>
+      <c r="I5" s="199"/>
       <c r="J5" s="168"/>
       <c r="K5" s="169" t="s">
         <v>1</v>
       </c>
       <c r="L5" s="170"/>
       <c r="M5" s="170"/>
-      <c r="N5" s="207" t="s">
+      <c r="N5" s="200" t="s">
         <v>2</v>
       </c>
-      <c r="O5" s="208"/>
-      <c r="P5" s="208"/>
-      <c r="Q5" s="208"/>
-      <c r="R5" s="208"/>
-      <c r="S5" s="208"/>
-      <c r="T5" s="208"/>
-      <c r="U5" s="208"/>
-      <c r="V5" s="208"/>
-      <c r="W5" s="209"/>
-      <c r="X5" s="209"/>
-      <c r="Y5" s="209"/>
-      <c r="Z5" s="209"/>
-      <c r="AA5" s="209"/>
-      <c r="AB5" s="209"/>
-      <c r="AC5" s="210" t="s">
+      <c r="O5" s="201"/>
+      <c r="P5" s="201"/>
+      <c r="Q5" s="201"/>
+      <c r="R5" s="201"/>
+      <c r="S5" s="201"/>
+      <c r="T5" s="201"/>
+      <c r="U5" s="201"/>
+      <c r="V5" s="201"/>
+      <c r="W5" s="202"/>
+      <c r="X5" s="202"/>
+      <c r="Y5" s="202"/>
+      <c r="Z5" s="202"/>
+      <c r="AA5" s="202"/>
+      <c r="AB5" s="202"/>
+      <c r="AC5" s="203" t="s">
         <v>3</v>
       </c>
-      <c r="AD5" s="211"/>
+      <c r="AD5" s="204"/>
       <c r="AF5" s="23"/>
       <c r="AG5" s="24"/>
       <c r="AH5" s="24"/>
@@ -5164,7 +5164,7 @@
       <c r="T21" s="37"/>
       <c r="U21" s="37"/>
       <c r="V21" s="37" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="W21" s="39"/>
       <c r="X21" s="39"/>
@@ -5210,7 +5210,7 @@
       <c r="T22" s="37"/>
       <c r="U22" s="37"/>
       <c r="V22" s="37" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="W22" s="39"/>
       <c r="X22" s="39"/>
@@ -5255,10 +5255,10 @@
       <c r="S23" s="37"/>
       <c r="T23" s="37"/>
       <c r="U23" s="37"/>
-      <c r="V23" s="37"/>
-      <c r="W23" s="39" t="s">
-        <v>11</v>
-      </c>
+      <c r="V23" s="37" t="s">
+        <v>10</v>
+      </c>
+      <c r="W23" s="39"/>
       <c r="X23" s="39"/>
       <c r="Y23" s="39"/>
       <c r="Z23" s="39"/>
@@ -6286,10 +6286,10 @@
       <c r="Z51" s="166"/>
       <c r="AA51" s="166"/>
       <c r="AB51" s="166"/>
-      <c r="AC51" s="222" t="s">
+      <c r="AC51" s="217" t="s">
         <v>37</v>
       </c>
-      <c r="AD51" s="223"/>
+      <c r="AD51" s="218"/>
       <c r="AF51" s="31"/>
       <c r="AG51" s="32"/>
       <c r="AH51" s="32"/>
@@ -6585,7 +6585,7 @@
       <c r="B59" s="88"/>
       <c r="C59" s="89"/>
       <c r="D59" s="178"/>
-      <c r="E59" s="224" t="s">
+      <c r="E59" s="188" t="s">
         <v>42</v>
       </c>
       <c r="F59" s="178"/>
@@ -6619,79 +6619,79 @@
       <c r="AH59" s="32"/>
     </row>
     <row r="60" spans="1:34" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="212" t="s">
+      <c r="B60" s="205" t="s">
         <v>39</v>
       </c>
-      <c r="C60" s="212" t="s">
+      <c r="C60" s="205" t="s">
         <v>40</v>
       </c>
-      <c r="D60" s="215" t="s">
+      <c r="D60" s="186" t="s">
         <v>41</v>
       </c>
-      <c r="E60" s="225"/>
-      <c r="F60" s="215" t="s">
+      <c r="E60" s="189"/>
+      <c r="F60" s="186" t="s">
         <v>43</v>
       </c>
-      <c r="G60" s="215" t="s">
+      <c r="G60" s="186" t="s">
         <v>44</v>
       </c>
-      <c r="H60" s="215" t="s">
+      <c r="H60" s="186" t="s">
         <v>45</v>
       </c>
-      <c r="I60" s="215"/>
+      <c r="I60" s="186"/>
       <c r="J60" s="101"/>
       <c r="K60" s="96"/>
       <c r="L60" s="97"/>
       <c r="M60" s="97"/>
-      <c r="N60" s="186">
+      <c r="N60" s="208">
         <v>46099</v>
       </c>
-      <c r="O60" s="186">
+      <c r="O60" s="208">
         <v>46100</v>
       </c>
-      <c r="P60" s="186">
+      <c r="P60" s="208">
         <v>46101</v>
       </c>
-      <c r="Q60" s="186">
+      <c r="Q60" s="208">
         <v>46102</v>
       </c>
-      <c r="R60" s="186">
+      <c r="R60" s="208">
         <v>46103</v>
       </c>
-      <c r="S60" s="186">
+      <c r="S60" s="208">
         <v>46104</v>
       </c>
-      <c r="T60" s="186">
+      <c r="T60" s="208">
         <v>46105</v>
       </c>
-      <c r="U60" s="227">
+      <c r="U60" s="212">
         <v>46108</v>
       </c>
-      <c r="V60" s="227">
+      <c r="V60" s="212">
         <v>46109</v>
       </c>
-      <c r="W60" s="227">
-        <v>46110</v>
-      </c>
-      <c r="X60" s="227">
-        <v>46111</v>
-      </c>
-      <c r="Y60" s="227">
+      <c r="W60" s="212">
         <v>46112</v>
       </c>
-      <c r="Z60" s="227">
+      <c r="X60" s="212">
         <v>46113</v>
       </c>
-      <c r="AA60" s="227">
+      <c r="Y60" s="212">
         <v>46114</v>
       </c>
-      <c r="AB60" s="227">
+      <c r="Z60" s="212">
         <v>46115</v>
       </c>
-      <c r="AC60" s="219" t="s">
+      <c r="AA60" s="212">
+        <v>46116</v>
+      </c>
+      <c r="AB60" s="212">
+        <v>46117</v>
+      </c>
+      <c r="AC60" s="214" t="s">
         <v>18</v>
       </c>
-      <c r="AD60" s="188" t="s">
+      <c r="AD60" s="226" t="s">
         <v>19</v>
       </c>
       <c r="AF60" s="31"/>
@@ -6699,182 +6699,182 @@
       <c r="AH60" s="32"/>
     </row>
     <row r="61" spans="1:34" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="213"/>
-      <c r="C61" s="213"/>
-      <c r="D61" s="215"/>
-      <c r="E61" s="225"/>
-      <c r="F61" s="215"/>
-      <c r="G61" s="215"/>
-      <c r="H61" s="215"/>
-      <c r="I61" s="215"/>
+      <c r="B61" s="206"/>
+      <c r="C61" s="206"/>
+      <c r="D61" s="186"/>
+      <c r="E61" s="189"/>
+      <c r="F61" s="186"/>
+      <c r="G61" s="186"/>
+      <c r="H61" s="186"/>
+      <c r="I61" s="186"/>
       <c r="J61" s="101"/>
       <c r="K61" s="98"/>
       <c r="L61" s="97"/>
       <c r="M61" s="97"/>
-      <c r="N61" s="186"/>
-      <c r="O61" s="186"/>
-      <c r="P61" s="186"/>
-      <c r="Q61" s="186"/>
-      <c r="R61" s="186"/>
-      <c r="S61" s="186"/>
-      <c r="T61" s="186"/>
-      <c r="U61" s="227"/>
-      <c r="V61" s="227"/>
-      <c r="W61" s="227"/>
-      <c r="X61" s="227"/>
-      <c r="Y61" s="227"/>
-      <c r="Z61" s="227"/>
-      <c r="AA61" s="227"/>
-      <c r="AB61" s="227"/>
-      <c r="AC61" s="220"/>
-      <c r="AD61" s="189"/>
+      <c r="N61" s="208"/>
+      <c r="O61" s="208"/>
+      <c r="P61" s="208"/>
+      <c r="Q61" s="208"/>
+      <c r="R61" s="208"/>
+      <c r="S61" s="208"/>
+      <c r="T61" s="208"/>
+      <c r="U61" s="212"/>
+      <c r="V61" s="212"/>
+      <c r="W61" s="212"/>
+      <c r="X61" s="212"/>
+      <c r="Y61" s="212"/>
+      <c r="Z61" s="212"/>
+      <c r="AA61" s="212"/>
+      <c r="AB61" s="212"/>
+      <c r="AC61" s="215"/>
+      <c r="AD61" s="227"/>
       <c r="AF61" s="31"/>
       <c r="AG61" s="32"/>
       <c r="AH61" s="32"/>
     </row>
     <row r="62" spans="1:34" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B62" s="213"/>
-      <c r="C62" s="213"/>
-      <c r="D62" s="215"/>
-      <c r="E62" s="225"/>
-      <c r="F62" s="215"/>
-      <c r="G62" s="215"/>
-      <c r="H62" s="215"/>
-      <c r="I62" s="215"/>
+      <c r="B62" s="206"/>
+      <c r="C62" s="206"/>
+      <c r="D62" s="186"/>
+      <c r="E62" s="189"/>
+      <c r="F62" s="186"/>
+      <c r="G62" s="186"/>
+      <c r="H62" s="186"/>
+      <c r="I62" s="186"/>
       <c r="J62" s="101"/>
       <c r="K62" s="98"/>
       <c r="L62" s="97"/>
       <c r="M62" s="97"/>
-      <c r="N62" s="186"/>
-      <c r="O62" s="186"/>
-      <c r="P62" s="186"/>
-      <c r="Q62" s="186"/>
-      <c r="R62" s="186"/>
-      <c r="S62" s="186"/>
-      <c r="T62" s="186"/>
-      <c r="U62" s="227"/>
-      <c r="V62" s="227"/>
-      <c r="W62" s="227"/>
-      <c r="X62" s="227"/>
-      <c r="Y62" s="227"/>
-      <c r="Z62" s="227"/>
-      <c r="AA62" s="227"/>
-      <c r="AB62" s="227"/>
-      <c r="AC62" s="220"/>
-      <c r="AD62" s="189"/>
+      <c r="N62" s="208"/>
+      <c r="O62" s="208"/>
+      <c r="P62" s="208"/>
+      <c r="Q62" s="208"/>
+      <c r="R62" s="208"/>
+      <c r="S62" s="208"/>
+      <c r="T62" s="208"/>
+      <c r="U62" s="212"/>
+      <c r="V62" s="212"/>
+      <c r="W62" s="212"/>
+      <c r="X62" s="212"/>
+      <c r="Y62" s="212"/>
+      <c r="Z62" s="212"/>
+      <c r="AA62" s="212"/>
+      <c r="AB62" s="212"/>
+      <c r="AC62" s="215"/>
+      <c r="AD62" s="227"/>
       <c r="AF62" s="31"/>
       <c r="AG62" s="32"/>
       <c r="AH62" s="32"/>
     </row>
     <row r="63" spans="1:34" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B63" s="213"/>
-      <c r="C63" s="213"/>
-      <c r="D63" s="215"/>
-      <c r="E63" s="225"/>
-      <c r="F63" s="215"/>
-      <c r="G63" s="215"/>
-      <c r="H63" s="215"/>
-      <c r="I63" s="215"/>
+      <c r="B63" s="206"/>
+      <c r="C63" s="206"/>
+      <c r="D63" s="186"/>
+      <c r="E63" s="189"/>
+      <c r="F63" s="186"/>
+      <c r="G63" s="186"/>
+      <c r="H63" s="186"/>
+      <c r="I63" s="186"/>
       <c r="J63" s="101"/>
       <c r="K63" s="99"/>
       <c r="L63" s="97"/>
       <c r="M63" s="97"/>
-      <c r="N63" s="186"/>
-      <c r="O63" s="186"/>
-      <c r="P63" s="186"/>
-      <c r="Q63" s="186"/>
-      <c r="R63" s="186"/>
-      <c r="S63" s="186"/>
-      <c r="T63" s="186"/>
-      <c r="U63" s="227"/>
-      <c r="V63" s="227"/>
-      <c r="W63" s="227"/>
-      <c r="X63" s="227"/>
-      <c r="Y63" s="227"/>
-      <c r="Z63" s="227"/>
-      <c r="AA63" s="227"/>
-      <c r="AB63" s="227"/>
-      <c r="AC63" s="220"/>
-      <c r="AD63" s="189"/>
+      <c r="N63" s="208"/>
+      <c r="O63" s="208"/>
+      <c r="P63" s="208"/>
+      <c r="Q63" s="208"/>
+      <c r="R63" s="208"/>
+      <c r="S63" s="208"/>
+      <c r="T63" s="208"/>
+      <c r="U63" s="212"/>
+      <c r="V63" s="212"/>
+      <c r="W63" s="212"/>
+      <c r="X63" s="212"/>
+      <c r="Y63" s="212"/>
+      <c r="Z63" s="212"/>
+      <c r="AA63" s="212"/>
+      <c r="AB63" s="212"/>
+      <c r="AC63" s="215"/>
+      <c r="AD63" s="227"/>
       <c r="AG63" s="32"/>
       <c r="AH63" s="32"/>
     </row>
     <row r="64" spans="1:34" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B64" s="213"/>
-      <c r="C64" s="213"/>
-      <c r="D64" s="215"/>
-      <c r="E64" s="225"/>
-      <c r="F64" s="215"/>
-      <c r="G64" s="215"/>
-      <c r="H64" s="215"/>
-      <c r="I64" s="215"/>
+      <c r="B64" s="206"/>
+      <c r="C64" s="206"/>
+      <c r="D64" s="186"/>
+      <c r="E64" s="189"/>
+      <c r="F64" s="186"/>
+      <c r="G64" s="186"/>
+      <c r="H64" s="186"/>
+      <c r="I64" s="186"/>
       <c r="J64" s="101"/>
       <c r="K64" s="96"/>
       <c r="L64" s="97"/>
       <c r="M64" s="97"/>
-      <c r="N64" s="186"/>
-      <c r="O64" s="186"/>
-      <c r="P64" s="186"/>
-      <c r="Q64" s="186"/>
-      <c r="R64" s="186"/>
-      <c r="S64" s="186"/>
-      <c r="T64" s="186"/>
-      <c r="U64" s="227"/>
-      <c r="V64" s="227"/>
-      <c r="W64" s="227"/>
-      <c r="X64" s="227"/>
-      <c r="Y64" s="227"/>
-      <c r="Z64" s="227"/>
-      <c r="AA64" s="227"/>
-      <c r="AB64" s="227"/>
-      <c r="AC64" s="220"/>
-      <c r="AD64" s="189"/>
+      <c r="N64" s="208"/>
+      <c r="O64" s="208"/>
+      <c r="P64" s="208"/>
+      <c r="Q64" s="208"/>
+      <c r="R64" s="208"/>
+      <c r="S64" s="208"/>
+      <c r="T64" s="208"/>
+      <c r="U64" s="212"/>
+      <c r="V64" s="212"/>
+      <c r="W64" s="212"/>
+      <c r="X64" s="212"/>
+      <c r="Y64" s="212"/>
+      <c r="Z64" s="212"/>
+      <c r="AA64" s="212"/>
+      <c r="AB64" s="212"/>
+      <c r="AC64" s="215"/>
+      <c r="AD64" s="227"/>
       <c r="AG64" s="32"/>
       <c r="AH64" s="32"/>
     </row>
     <row r="65" spans="2:34" ht="12.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B65" s="213"/>
-      <c r="C65" s="213"/>
-      <c r="D65" s="215"/>
-      <c r="E65" s="225"/>
-      <c r="F65" s="215"/>
-      <c r="G65" s="215"/>
-      <c r="H65" s="215"/>
-      <c r="I65" s="215"/>
+      <c r="B65" s="206"/>
+      <c r="C65" s="206"/>
+      <c r="D65" s="186"/>
+      <c r="E65" s="189"/>
+      <c r="F65" s="186"/>
+      <c r="G65" s="186"/>
+      <c r="H65" s="186"/>
+      <c r="I65" s="186"/>
       <c r="J65" s="101"/>
       <c r="K65" s="100"/>
       <c r="L65" s="97"/>
       <c r="M65" s="97"/>
-      <c r="N65" s="187"/>
-      <c r="O65" s="187"/>
-      <c r="P65" s="187"/>
-      <c r="Q65" s="187"/>
-      <c r="R65" s="187"/>
-      <c r="S65" s="187"/>
-      <c r="T65" s="187"/>
-      <c r="U65" s="228"/>
-      <c r="V65" s="228"/>
-      <c r="W65" s="228"/>
-      <c r="X65" s="228"/>
-      <c r="Y65" s="228"/>
-      <c r="Z65" s="228"/>
-      <c r="AA65" s="228"/>
-      <c r="AB65" s="228"/>
-      <c r="AC65" s="221"/>
-      <c r="AD65" s="190"/>
+      <c r="N65" s="209"/>
+      <c r="O65" s="209"/>
+      <c r="P65" s="209"/>
+      <c r="Q65" s="209"/>
+      <c r="R65" s="209"/>
+      <c r="S65" s="209"/>
+      <c r="T65" s="209"/>
+      <c r="U65" s="213"/>
+      <c r="V65" s="213"/>
+      <c r="W65" s="213"/>
+      <c r="X65" s="213"/>
+      <c r="Y65" s="213"/>
+      <c r="Z65" s="213"/>
+      <c r="AA65" s="213"/>
+      <c r="AB65" s="213"/>
+      <c r="AC65" s="216"/>
+      <c r="AD65" s="228"/>
       <c r="AF65" s="23"/>
       <c r="AG65" s="23"/>
       <c r="AH65" s="23"/>
     </row>
     <row r="66" spans="2:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="213"/>
-      <c r="C66" s="213"/>
-      <c r="D66" s="215"/>
-      <c r="E66" s="225"/>
-      <c r="F66" s="215"/>
-      <c r="G66" s="215"/>
-      <c r="H66" s="215"/>
-      <c r="I66" s="215"/>
+      <c r="B66" s="206"/>
+      <c r="C66" s="206"/>
+      <c r="D66" s="186"/>
+      <c r="E66" s="189"/>
+      <c r="F66" s="186"/>
+      <c r="G66" s="186"/>
+      <c r="H66" s="186"/>
+      <c r="I66" s="186"/>
       <c r="J66" s="101"/>
       <c r="K66" s="100"/>
       <c r="L66" s="100"/>
@@ -6897,20 +6897,20 @@
       <c r="AC66" s="103"/>
       <c r="AD66" s="104"/>
       <c r="AF66" s="23"/>
-      <c r="AG66" s="191" t="s">
+      <c r="AG66" s="219" t="s">
         <v>6</v>
       </c>
-      <c r="AH66" s="191"/>
+      <c r="AH66" s="219"/>
     </row>
     <row r="67" spans="2:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B67" s="213"/>
-      <c r="C67" s="213"/>
-      <c r="D67" s="215"/>
-      <c r="E67" s="225"/>
-      <c r="F67" s="215"/>
-      <c r="G67" s="215"/>
-      <c r="H67" s="215"/>
-      <c r="I67" s="215"/>
+      <c r="B67" s="206"/>
+      <c r="C67" s="206"/>
+      <c r="D67" s="186"/>
+      <c r="E67" s="189"/>
+      <c r="F67" s="186"/>
+      <c r="G67" s="186"/>
+      <c r="H67" s="186"/>
+      <c r="I67" s="186"/>
       <c r="J67" s="105"/>
       <c r="K67" s="100"/>
       <c r="L67" s="98"/>
@@ -6943,14 +6943,14 @@
       </c>
     </row>
     <row r="68" spans="2:34" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B68" s="213"/>
-      <c r="C68" s="213"/>
-      <c r="D68" s="215"/>
-      <c r="E68" s="225"/>
-      <c r="F68" s="215"/>
-      <c r="G68" s="215"/>
-      <c r="H68" s="215"/>
-      <c r="I68" s="215"/>
+      <c r="B68" s="206"/>
+      <c r="C68" s="206"/>
+      <c r="D68" s="186"/>
+      <c r="E68" s="189"/>
+      <c r="F68" s="186"/>
+      <c r="G68" s="186"/>
+      <c r="H68" s="186"/>
+      <c r="I68" s="186"/>
       <c r="J68" s="101"/>
       <c r="K68" s="96"/>
       <c r="L68" s="98"/>
@@ -6979,14 +6979,14 @@
       <c r="AH68" s="111"/>
     </row>
     <row r="69" spans="2:34" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B69" s="213"/>
-      <c r="C69" s="213"/>
-      <c r="D69" s="215"/>
-      <c r="E69" s="225"/>
-      <c r="F69" s="215"/>
-      <c r="G69" s="215"/>
-      <c r="H69" s="215"/>
-      <c r="I69" s="215"/>
+      <c r="B69" s="206"/>
+      <c r="C69" s="206"/>
+      <c r="D69" s="186"/>
+      <c r="E69" s="189"/>
+      <c r="F69" s="186"/>
+      <c r="G69" s="186"/>
+      <c r="H69" s="186"/>
+      <c r="I69" s="186"/>
       <c r="J69" s="101"/>
       <c r="K69" s="96"/>
       <c r="L69" s="98"/>
@@ -7015,14 +7015,14 @@
       <c r="AH69" s="113"/>
     </row>
     <row r="70" spans="2:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B70" s="213"/>
-      <c r="C70" s="213"/>
-      <c r="D70" s="215"/>
-      <c r="E70" s="225"/>
-      <c r="F70" s="215"/>
-      <c r="G70" s="215"/>
-      <c r="H70" s="215"/>
-      <c r="I70" s="215"/>
+      <c r="B70" s="206"/>
+      <c r="C70" s="206"/>
+      <c r="D70" s="186"/>
+      <c r="E70" s="189"/>
+      <c r="F70" s="186"/>
+      <c r="G70" s="186"/>
+      <c r="H70" s="186"/>
+      <c r="I70" s="186"/>
       <c r="J70" s="101"/>
       <c r="K70" s="96"/>
       <c r="L70" s="96"/>
@@ -7051,14 +7051,14 @@
       <c r="AH70" s="111"/>
     </row>
     <row r="71" spans="2:34" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B71" s="213"/>
-      <c r="C71" s="213"/>
-      <c r="D71" s="215"/>
-      <c r="E71" s="225"/>
-      <c r="F71" s="215"/>
-      <c r="G71" s="215"/>
-      <c r="H71" s="215"/>
-      <c r="I71" s="215"/>
+      <c r="B71" s="206"/>
+      <c r="C71" s="206"/>
+      <c r="D71" s="186"/>
+      <c r="E71" s="189"/>
+      <c r="F71" s="186"/>
+      <c r="G71" s="186"/>
+      <c r="H71" s="186"/>
+      <c r="I71" s="186"/>
       <c r="J71" s="101"/>
       <c r="K71" s="114"/>
       <c r="L71" s="101"/>
@@ -7084,14 +7084,14 @@
       <c r="AG71" s="115"/>
     </row>
     <row r="72" spans="2:34" ht="15.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B72" s="213"/>
-      <c r="C72" s="213"/>
-      <c r="D72" s="215"/>
-      <c r="E72" s="225"/>
-      <c r="F72" s="215"/>
-      <c r="G72" s="215"/>
-      <c r="H72" s="215"/>
-      <c r="I72" s="215"/>
+      <c r="B72" s="206"/>
+      <c r="C72" s="206"/>
+      <c r="D72" s="186"/>
+      <c r="E72" s="189"/>
+      <c r="F72" s="186"/>
+      <c r="G72" s="186"/>
+      <c r="H72" s="186"/>
+      <c r="I72" s="186"/>
       <c r="J72" s="117"/>
       <c r="K72" s="116"/>
       <c r="L72" s="117"/>
@@ -7117,128 +7117,128 @@
       <c r="AH72" s="115"/>
     </row>
     <row r="73" spans="2:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B73" s="213"/>
-      <c r="C73" s="213"/>
-      <c r="D73" s="215"/>
-      <c r="E73" s="225"/>
-      <c r="F73" s="215"/>
-      <c r="G73" s="215"/>
-      <c r="H73" s="215"/>
-      <c r="I73" s="215"/>
-      <c r="J73" s="192"/>
-      <c r="K73" s="192"/>
-      <c r="L73" s="192"/>
-      <c r="M73" s="192"/>
-      <c r="N73" s="192"/>
-      <c r="O73" s="192"/>
-      <c r="P73" s="192"/>
-      <c r="Q73" s="192"/>
-      <c r="R73" s="192"/>
-      <c r="S73" s="192"/>
-      <c r="T73" s="192"/>
-      <c r="U73" s="192"/>
-      <c r="V73" s="192"/>
-      <c r="W73" s="192"/>
-      <c r="X73" s="192"/>
-      <c r="Y73" s="192"/>
-      <c r="Z73" s="192"/>
-      <c r="AA73" s="192"/>
-      <c r="AB73" s="192"/>
-      <c r="AC73" s="192"/>
-      <c r="AD73" s="193"/>
+      <c r="B73" s="206"/>
+      <c r="C73" s="206"/>
+      <c r="D73" s="186"/>
+      <c r="E73" s="189"/>
+      <c r="F73" s="186"/>
+      <c r="G73" s="186"/>
+      <c r="H73" s="186"/>
+      <c r="I73" s="186"/>
+      <c r="J73" s="220"/>
+      <c r="K73" s="220"/>
+      <c r="L73" s="220"/>
+      <c r="M73" s="220"/>
+      <c r="N73" s="220"/>
+      <c r="O73" s="220"/>
+      <c r="P73" s="220"/>
+      <c r="Q73" s="220"/>
+      <c r="R73" s="220"/>
+      <c r="S73" s="220"/>
+      <c r="T73" s="220"/>
+      <c r="U73" s="220"/>
+      <c r="V73" s="220"/>
+      <c r="W73" s="220"/>
+      <c r="X73" s="220"/>
+      <c r="Y73" s="220"/>
+      <c r="Z73" s="220"/>
+      <c r="AA73" s="220"/>
+      <c r="AB73" s="220"/>
+      <c r="AC73" s="220"/>
+      <c r="AD73" s="221"/>
     </row>
     <row r="74" spans="2:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B74" s="213"/>
-      <c r="C74" s="213"/>
-      <c r="D74" s="215"/>
-      <c r="E74" s="225"/>
-      <c r="F74" s="215"/>
-      <c r="G74" s="215"/>
-      <c r="H74" s="215"/>
-      <c r="I74" s="215"/>
-      <c r="J74" s="194"/>
-      <c r="K74" s="194"/>
-      <c r="L74" s="194"/>
-      <c r="M74" s="194"/>
-      <c r="N74" s="194"/>
-      <c r="O74" s="194"/>
-      <c r="P74" s="194"/>
-      <c r="Q74" s="194"/>
-      <c r="R74" s="194"/>
-      <c r="S74" s="194"/>
-      <c r="T74" s="194"/>
-      <c r="U74" s="194"/>
-      <c r="V74" s="194"/>
-      <c r="W74" s="194"/>
-      <c r="X74" s="194"/>
-      <c r="Y74" s="194"/>
-      <c r="Z74" s="194"/>
-      <c r="AA74" s="194"/>
-      <c r="AB74" s="194"/>
-      <c r="AC74" s="194"/>
-      <c r="AD74" s="195"/>
+      <c r="B74" s="206"/>
+      <c r="C74" s="206"/>
+      <c r="D74" s="186"/>
+      <c r="E74" s="189"/>
+      <c r="F74" s="186"/>
+      <c r="G74" s="186"/>
+      <c r="H74" s="186"/>
+      <c r="I74" s="186"/>
+      <c r="J74" s="222"/>
+      <c r="K74" s="222"/>
+      <c r="L74" s="222"/>
+      <c r="M74" s="222"/>
+      <c r="N74" s="222"/>
+      <c r="O74" s="222"/>
+      <c r="P74" s="222"/>
+      <c r="Q74" s="222"/>
+      <c r="R74" s="222"/>
+      <c r="S74" s="222"/>
+      <c r="T74" s="222"/>
+      <c r="U74" s="222"/>
+      <c r="V74" s="222"/>
+      <c r="W74" s="222"/>
+      <c r="X74" s="222"/>
+      <c r="Y74" s="222"/>
+      <c r="Z74" s="222"/>
+      <c r="AA74" s="222"/>
+      <c r="AB74" s="222"/>
+      <c r="AC74" s="222"/>
+      <c r="AD74" s="223"/>
     </row>
     <row r="75" spans="2:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B75" s="213"/>
-      <c r="C75" s="213"/>
-      <c r="D75" s="215"/>
-      <c r="E75" s="225"/>
-      <c r="F75" s="215"/>
-      <c r="G75" s="215"/>
-      <c r="H75" s="215"/>
-      <c r="I75" s="215"/>
-      <c r="J75" s="194"/>
-      <c r="K75" s="194"/>
-      <c r="L75" s="194"/>
-      <c r="M75" s="194"/>
-      <c r="N75" s="194"/>
-      <c r="O75" s="194"/>
-      <c r="P75" s="194"/>
-      <c r="Q75" s="194"/>
-      <c r="R75" s="194"/>
-      <c r="S75" s="194"/>
-      <c r="T75" s="194"/>
-      <c r="U75" s="194"/>
-      <c r="V75" s="194"/>
-      <c r="W75" s="194"/>
-      <c r="X75" s="194"/>
-      <c r="Y75" s="194"/>
-      <c r="Z75" s="194"/>
-      <c r="AA75" s="194"/>
-      <c r="AB75" s="194"/>
-      <c r="AC75" s="194"/>
-      <c r="AD75" s="195"/>
+      <c r="B75" s="206"/>
+      <c r="C75" s="206"/>
+      <c r="D75" s="186"/>
+      <c r="E75" s="189"/>
+      <c r="F75" s="186"/>
+      <c r="G75" s="186"/>
+      <c r="H75" s="186"/>
+      <c r="I75" s="186"/>
+      <c r="J75" s="222"/>
+      <c r="K75" s="222"/>
+      <c r="L75" s="222"/>
+      <c r="M75" s="222"/>
+      <c r="N75" s="222"/>
+      <c r="O75" s="222"/>
+      <c r="P75" s="222"/>
+      <c r="Q75" s="222"/>
+      <c r="R75" s="222"/>
+      <c r="S75" s="222"/>
+      <c r="T75" s="222"/>
+      <c r="U75" s="222"/>
+      <c r="V75" s="222"/>
+      <c r="W75" s="222"/>
+      <c r="X75" s="222"/>
+      <c r="Y75" s="222"/>
+      <c r="Z75" s="222"/>
+      <c r="AA75" s="222"/>
+      <c r="AB75" s="222"/>
+      <c r="AC75" s="222"/>
+      <c r="AD75" s="223"/>
     </row>
     <row r="76" spans="2:34" s="1" customFormat="1" ht="15.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B76" s="214"/>
-      <c r="C76" s="214"/>
-      <c r="D76" s="216"/>
-      <c r="E76" s="226"/>
-      <c r="F76" s="216"/>
-      <c r="G76" s="216"/>
-      <c r="H76" s="216"/>
-      <c r="I76" s="216"/>
-      <c r="J76" s="217"/>
-      <c r="K76" s="217"/>
-      <c r="L76" s="217"/>
-      <c r="M76" s="217"/>
-      <c r="N76" s="217"/>
-      <c r="O76" s="217"/>
-      <c r="P76" s="217"/>
-      <c r="Q76" s="217"/>
-      <c r="R76" s="217"/>
-      <c r="S76" s="217"/>
-      <c r="T76" s="217"/>
-      <c r="U76" s="217"/>
-      <c r="V76" s="217"/>
-      <c r="W76" s="217"/>
-      <c r="X76" s="217"/>
-      <c r="Y76" s="217"/>
-      <c r="Z76" s="217"/>
-      <c r="AA76" s="217"/>
-      <c r="AB76" s="217"/>
-      <c r="AC76" s="217"/>
-      <c r="AD76" s="218"/>
+      <c r="B76" s="207"/>
+      <c r="C76" s="207"/>
+      <c r="D76" s="187"/>
+      <c r="E76" s="190"/>
+      <c r="F76" s="187"/>
+      <c r="G76" s="187"/>
+      <c r="H76" s="187"/>
+      <c r="I76" s="187"/>
+      <c r="J76" s="210"/>
+      <c r="K76" s="210"/>
+      <c r="L76" s="210"/>
+      <c r="M76" s="210"/>
+      <c r="N76" s="210"/>
+      <c r="O76" s="210"/>
+      <c r="P76" s="210"/>
+      <c r="Q76" s="210"/>
+      <c r="R76" s="210"/>
+      <c r="S76" s="210"/>
+      <c r="T76" s="210"/>
+      <c r="U76" s="210"/>
+      <c r="V76" s="210"/>
+      <c r="W76" s="210"/>
+      <c r="X76" s="210"/>
+      <c r="Y76" s="210"/>
+      <c r="Z76" s="210"/>
+      <c r="AA76" s="210"/>
+      <c r="AB76" s="210"/>
+      <c r="AC76" s="210"/>
+      <c r="AD76" s="211"/>
       <c r="AF76" s="23"/>
       <c r="AG76" s="24"/>
       <c r="AH76" s="24"/>
@@ -7268,15 +7268,15 @@
       <c r="U78" s="131" t="s">
         <v>15</v>
       </c>
-      <c r="V78" s="196" t="s">
+      <c r="V78" s="224" t="s">
         <v>23</v>
       </c>
-      <c r="W78" s="197"/>
-      <c r="X78" s="197"/>
-      <c r="Y78" s="197"/>
-      <c r="Z78" s="197"/>
-      <c r="AA78" s="197"/>
-      <c r="AB78" s="197"/>
+      <c r="W78" s="225"/>
+      <c r="X78" s="225"/>
+      <c r="Y78" s="225"/>
+      <c r="Z78" s="225"/>
+      <c r="AA78" s="225"/>
+      <c r="AB78" s="225"/>
       <c r="AD78" s="123"/>
       <c r="AE78" s="123"/>
       <c r="AF78" s="123"/>
@@ -7305,15 +7305,15 @@
       <c r="U79" s="138" t="s">
         <v>16</v>
       </c>
-      <c r="V79" s="196" t="s">
+      <c r="V79" s="224" t="s">
         <v>24</v>
       </c>
-      <c r="W79" s="197"/>
-      <c r="X79" s="197"/>
-      <c r="Y79" s="197"/>
-      <c r="Z79" s="197"/>
-      <c r="AA79" s="197"/>
-      <c r="AB79" s="197"/>
+      <c r="W79" s="225"/>
+      <c r="X79" s="225"/>
+      <c r="Y79" s="225"/>
+      <c r="Z79" s="225"/>
+      <c r="AA79" s="225"/>
+      <c r="AB79" s="225"/>
       <c r="AD79" s="125"/>
       <c r="AE79" s="125"/>
       <c r="AF79" s="125"/>
@@ -7343,15 +7343,15 @@
       <c r="U80" s="146" t="s">
         <v>17</v>
       </c>
-      <c r="V80" s="196" t="s">
+      <c r="V80" s="224" t="s">
         <v>25</v>
       </c>
-      <c r="W80" s="197"/>
-      <c r="X80" s="197"/>
-      <c r="Y80" s="197"/>
-      <c r="Z80" s="197"/>
-      <c r="AA80" s="197"/>
-      <c r="AB80" s="197"/>
+      <c r="W80" s="225"/>
+      <c r="X80" s="225"/>
+      <c r="Y80" s="225"/>
+      <c r="Z80" s="225"/>
+      <c r="AA80" s="225"/>
+      <c r="AB80" s="225"/>
       <c r="AD80" s="121"/>
       <c r="AE80" s="121"/>
       <c r="AF80" s="121"/>
@@ -7413,11 +7413,23 @@
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="H60:H76"/>
-    <mergeCell ref="E59:E76"/>
-    <mergeCell ref="G60:G76"/>
-    <mergeCell ref="F60:F76"/>
-    <mergeCell ref="D60:D76"/>
+    <mergeCell ref="S60:S65"/>
+    <mergeCell ref="T60:T65"/>
+    <mergeCell ref="U60:U65"/>
+    <mergeCell ref="V60:V65"/>
+    <mergeCell ref="AD60:AD65"/>
+    <mergeCell ref="X60:X65"/>
+    <mergeCell ref="Y60:Y65"/>
+    <mergeCell ref="Z60:Z65"/>
+    <mergeCell ref="AA60:AA65"/>
+    <mergeCell ref="AB60:AB65"/>
+    <mergeCell ref="AG66:AH66"/>
+    <mergeCell ref="J73:AD73"/>
+    <mergeCell ref="J74:AD74"/>
+    <mergeCell ref="V80:AB80"/>
+    <mergeCell ref="J75:AD75"/>
+    <mergeCell ref="V79:AB79"/>
+    <mergeCell ref="V78:AB78"/>
     <mergeCell ref="J3:AD4"/>
     <mergeCell ref="B5:I5"/>
     <mergeCell ref="N5:AB5"/>
@@ -7434,23 +7446,11 @@
     <mergeCell ref="AC51:AD51"/>
     <mergeCell ref="Q60:Q65"/>
     <mergeCell ref="R60:R65"/>
-    <mergeCell ref="AG66:AH66"/>
-    <mergeCell ref="J73:AD73"/>
-    <mergeCell ref="J74:AD74"/>
-    <mergeCell ref="V80:AB80"/>
-    <mergeCell ref="J75:AD75"/>
-    <mergeCell ref="V79:AB79"/>
-    <mergeCell ref="V78:AB78"/>
-    <mergeCell ref="S60:S65"/>
-    <mergeCell ref="T60:T65"/>
-    <mergeCell ref="U60:U65"/>
-    <mergeCell ref="V60:V65"/>
-    <mergeCell ref="AD60:AD65"/>
-    <mergeCell ref="X60:X65"/>
-    <mergeCell ref="Y60:Y65"/>
-    <mergeCell ref="Z60:Z65"/>
-    <mergeCell ref="AA60:AA65"/>
-    <mergeCell ref="AB60:AB65"/>
+    <mergeCell ref="H60:H76"/>
+    <mergeCell ref="E59:E76"/>
+    <mergeCell ref="G60:G76"/>
+    <mergeCell ref="F60:F76"/>
+    <mergeCell ref="D60:D76"/>
   </mergeCells>
   <phoneticPr fontId="26" type="noConversion"/>
   <conditionalFormatting sqref="B59:D59 F59:I59">
@@ -7469,88 +7469,88 @@
       <formula>"R"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="N28:U48">
+    <cfRule type="cellIs" dxfId="21" priority="1" stopIfTrue="1" operator="equal">
+      <formula>"S"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="20" priority="2" stopIfTrue="1" operator="equal">
+      <formula>"C"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="19" priority="3" stopIfTrue="1" operator="equal">
+      <formula>"D"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="N49:AB58">
-    <cfRule type="cellIs" dxfId="21" priority="15" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="15" stopIfTrue="1" operator="equal">
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N49:AB59">
-    <cfRule type="cellIs" dxfId="20" priority="13" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="13" stopIfTrue="1" operator="equal">
       <formula>"S"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="14" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="14" stopIfTrue="1" operator="equal">
       <formula>"C"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N59:AB59">
-    <cfRule type="cellIs" dxfId="18" priority="64" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="64" stopIfTrue="1" operator="equal">
       <formula>"L"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O6:AB7 T8:AB13 N8:R15 U14:AB15 N16:AB19 N20:Q27">
-    <cfRule type="cellIs" dxfId="17" priority="52" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="52" stopIfTrue="1" operator="equal">
       <formula>"S"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="53" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="53" stopIfTrue="1" operator="equal">
       <formula>"C"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="54" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="54" stopIfTrue="1" operator="equal">
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R20:U25 AB20:AB48 S26:U27 N28:U28 N29:T48 V28:AA48">
-    <cfRule type="cellIs" dxfId="14" priority="55" stopIfTrue="1" operator="equal">
+  <conditionalFormatting sqref="R20:U25 S26:U27">
+    <cfRule type="cellIs" dxfId="11" priority="55" stopIfTrue="1" operator="equal">
       <formula>"S"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="56" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="56" stopIfTrue="1" operator="equal">
       <formula>"C"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="57" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="57" stopIfTrue="1" operator="equal">
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R79:AB79">
-    <cfRule type="cellIs" dxfId="11" priority="28" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="28" stopIfTrue="1" operator="equal">
       <formula>"G"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="29" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="29" stopIfTrue="1" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="30" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="30" stopIfTrue="1" operator="equal">
       <formula>"R"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V20:AA27">
-    <cfRule type="cellIs" dxfId="8" priority="4" stopIfTrue="1" operator="equal">
+  <conditionalFormatting sqref="V20:AB48">
+    <cfRule type="cellIs" dxfId="5" priority="4" stopIfTrue="1" operator="equal">
       <formula>"S"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="5" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="5" stopIfTrue="1" operator="equal">
       <formula>"C"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="6" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="6" stopIfTrue="1" operator="equal">
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC59:AD59">
-    <cfRule type="cellIs" dxfId="5" priority="58" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="58" stopIfTrue="1" operator="equal">
       <formula>"A"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="59" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="59" stopIfTrue="1" operator="equal">
       <formula>"B"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="60" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="60" stopIfTrue="1" operator="equal">
       <formula>"C"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U29:U48">
-    <cfRule type="cellIs" dxfId="2" priority="1" stopIfTrue="1" operator="equal">
-      <formula>"S"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" stopIfTrue="1" operator="equal">
-      <formula>"C"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" stopIfTrue="1" operator="equal">
-      <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.5" right="0.5" top="0.65" bottom="0.35" header="0.4" footer="0.2"/>

</xml_diff>

<commit_message>
clean code - update fix later
</commit_message>
<xml_diff>
--- a/document/02_c_LAB301x_VN_v0.01_OPPM.xlsx
+++ b/document/02_c_LAB301x_VN_v0.01_OPPM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thanh\Downloads\FU\LAB\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C191D11-FCC0-4848-929F-87D0A0AA21DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DD3B23A-CF5C-45A4-AF52-73BF6F9423E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="192">
   <si>
     <t>Sub-Objectives</t>
   </si>
@@ -698,6 +698,9 @@
   </si>
   <si>
     <t>STT</t>
+  </si>
+  <si>
+    <t>fixed</t>
   </si>
 </sst>
 </file>
@@ -917,7 +920,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -996,6 +999,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="84">
     <border>
@@ -2075,7 +2084,7 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="267">
+  <cellXfs count="271">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyProtection="1"/>
@@ -2787,9 +2796,6 @@
     <xf numFmtId="0" fontId="30" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="81" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="83" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -2802,6 +2808,21 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="81" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="81" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="66" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90"/>
       <protection locked="0"/>
@@ -2979,8 +3000,8 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="83" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="81" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -5007,30 +5028,30 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
       <c r="I3" s="17"/>
-      <c r="J3" s="222" t="s">
+      <c r="J3" s="226" t="s">
         <v>38</v>
       </c>
-      <c r="K3" s="223"/>
-      <c r="L3" s="223"/>
-      <c r="M3" s="223"/>
-      <c r="N3" s="223"/>
-      <c r="O3" s="223"/>
-      <c r="P3" s="223"/>
-      <c r="Q3" s="223"/>
-      <c r="R3" s="223"/>
-      <c r="S3" s="223"/>
-      <c r="T3" s="223"/>
-      <c r="U3" s="223"/>
-      <c r="V3" s="223"/>
-      <c r="W3" s="223"/>
-      <c r="X3" s="223"/>
-      <c r="Y3" s="223"/>
-      <c r="Z3" s="223"/>
-      <c r="AA3" s="223"/>
-      <c r="AB3" s="223"/>
-      <c r="AC3" s="223"/>
-      <c r="AD3" s="223"/>
-      <c r="AE3" s="224"/>
+      <c r="K3" s="227"/>
+      <c r="L3" s="227"/>
+      <c r="M3" s="227"/>
+      <c r="N3" s="227"/>
+      <c r="O3" s="227"/>
+      <c r="P3" s="227"/>
+      <c r="Q3" s="227"/>
+      <c r="R3" s="227"/>
+      <c r="S3" s="227"/>
+      <c r="T3" s="227"/>
+      <c r="U3" s="227"/>
+      <c r="V3" s="227"/>
+      <c r="W3" s="227"/>
+      <c r="X3" s="227"/>
+      <c r="Y3" s="227"/>
+      <c r="Z3" s="227"/>
+      <c r="AA3" s="227"/>
+      <c r="AB3" s="227"/>
+      <c r="AC3" s="227"/>
+      <c r="AD3" s="227"/>
+      <c r="AE3" s="228"/>
       <c r="AG3" s="13"/>
       <c r="AH3" s="14"/>
       <c r="AI3" s="14"/>
@@ -5044,73 +5065,73 @@
       <c r="G4" s="20"/>
       <c r="H4" s="20"/>
       <c r="I4" s="20"/>
-      <c r="J4" s="225"/>
-      <c r="K4" s="226"/>
-      <c r="L4" s="226"/>
-      <c r="M4" s="226"/>
-      <c r="N4" s="226"/>
-      <c r="O4" s="226"/>
-      <c r="P4" s="226"/>
-      <c r="Q4" s="226"/>
-      <c r="R4" s="226"/>
-      <c r="S4" s="226"/>
-      <c r="T4" s="226"/>
-      <c r="U4" s="226"/>
-      <c r="V4" s="226"/>
-      <c r="W4" s="226"/>
-      <c r="X4" s="226"/>
-      <c r="Y4" s="226"/>
-      <c r="Z4" s="226"/>
-      <c r="AA4" s="226"/>
-      <c r="AB4" s="226"/>
-      <c r="AC4" s="226"/>
-      <c r="AD4" s="226"/>
-      <c r="AE4" s="227"/>
+      <c r="J4" s="229"/>
+      <c r="K4" s="230"/>
+      <c r="L4" s="230"/>
+      <c r="M4" s="230"/>
+      <c r="N4" s="230"/>
+      <c r="O4" s="230"/>
+      <c r="P4" s="230"/>
+      <c r="Q4" s="230"/>
+      <c r="R4" s="230"/>
+      <c r="S4" s="230"/>
+      <c r="T4" s="230"/>
+      <c r="U4" s="230"/>
+      <c r="V4" s="230"/>
+      <c r="W4" s="230"/>
+      <c r="X4" s="230"/>
+      <c r="Y4" s="230"/>
+      <c r="Z4" s="230"/>
+      <c r="AA4" s="230"/>
+      <c r="AB4" s="230"/>
+      <c r="AC4" s="230"/>
+      <c r="AD4" s="230"/>
+      <c r="AE4" s="231"/>
       <c r="AG4" s="21"/>
       <c r="AH4" s="22"/>
       <c r="AI4" s="22"/>
     </row>
     <row r="5" spans="1:35" s="1" customFormat="1" ht="26.4" customHeight="1" thickBot="1">
-      <c r="B5" s="228" t="s">
+      <c r="B5" s="232" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="229"/>
-      <c r="D5" s="229"/>
-      <c r="E5" s="229"/>
-      <c r="F5" s="229"/>
-      <c r="G5" s="229"/>
-      <c r="H5" s="229"/>
-      <c r="I5" s="230"/>
+      <c r="C5" s="233"/>
+      <c r="D5" s="233"/>
+      <c r="E5" s="233"/>
+      <c r="F5" s="233"/>
+      <c r="G5" s="233"/>
+      <c r="H5" s="233"/>
+      <c r="I5" s="234"/>
       <c r="J5" s="168"/>
       <c r="K5" s="169" t="s">
         <v>1</v>
       </c>
       <c r="L5" s="170"/>
       <c r="M5" s="170"/>
-      <c r="N5" s="231" t="s">
+      <c r="N5" s="235" t="s">
         <v>2</v>
       </c>
-      <c r="O5" s="232"/>
-      <c r="P5" s="232"/>
-      <c r="Q5" s="232"/>
-      <c r="R5" s="232"/>
-      <c r="S5" s="232"/>
-      <c r="T5" s="232"/>
-      <c r="U5" s="232"/>
-      <c r="V5" s="232"/>
-      <c r="W5" s="233"/>
-      <c r="X5" s="233"/>
-      <c r="Y5" s="233"/>
-      <c r="Z5" s="233"/>
-      <c r="AA5" s="233"/>
-      <c r="AB5" s="233"/>
+      <c r="O5" s="236"/>
+      <c r="P5" s="236"/>
+      <c r="Q5" s="236"/>
+      <c r="R5" s="236"/>
+      <c r="S5" s="236"/>
+      <c r="T5" s="236"/>
+      <c r="U5" s="236"/>
+      <c r="V5" s="236"/>
+      <c r="W5" s="237"/>
+      <c r="X5" s="237"/>
+      <c r="Y5" s="237"/>
+      <c r="Z5" s="237"/>
+      <c r="AA5" s="237"/>
+      <c r="AB5" s="237"/>
       <c r="AC5" s="170" t="s">
         <v>120</v>
       </c>
-      <c r="AD5" s="234" t="s">
+      <c r="AD5" s="238" t="s">
         <v>3</v>
       </c>
-      <c r="AE5" s="235"/>
+      <c r="AE5" s="239"/>
       <c r="AG5" s="23"/>
       <c r="AH5" s="24"/>
       <c r="AI5" s="24"/>
@@ -7009,10 +7030,10 @@
       <c r="AA51" s="166"/>
       <c r="AB51" s="166"/>
       <c r="AC51" s="200"/>
-      <c r="AD51" s="248" t="s">
+      <c r="AD51" s="252" t="s">
         <v>37</v>
       </c>
-      <c r="AE51" s="249"/>
+      <c r="AE51" s="253"/>
       <c r="AG51" s="31"/>
       <c r="AH51" s="32"/>
       <c r="AI51" s="32"/>
@@ -7315,7 +7336,7 @@
       <c r="B59" s="88"/>
       <c r="C59" s="89"/>
       <c r="D59" s="178"/>
-      <c r="E59" s="219" t="s">
+      <c r="E59" s="223" t="s">
         <v>42</v>
       </c>
       <c r="F59" s="178"/>
@@ -7350,80 +7371,80 @@
       <c r="AI59" s="32"/>
     </row>
     <row r="60" spans="1:35" ht="12.75" customHeight="1">
-      <c r="B60" s="236" t="s">
+      <c r="B60" s="240" t="s">
         <v>39</v>
       </c>
-      <c r="C60" s="236" t="s">
+      <c r="C60" s="240" t="s">
         <v>40</v>
       </c>
-      <c r="D60" s="217" t="s">
+      <c r="D60" s="221" t="s">
         <v>41</v>
       </c>
-      <c r="E60" s="220"/>
-      <c r="F60" s="217" t="s">
+      <c r="E60" s="224"/>
+      <c r="F60" s="221" t="s">
         <v>43</v>
       </c>
-      <c r="G60" s="217" t="s">
+      <c r="G60" s="221" t="s">
         <v>44</v>
       </c>
-      <c r="H60" s="217" t="s">
+      <c r="H60" s="221" t="s">
         <v>45</v>
       </c>
-      <c r="I60" s="217"/>
+      <c r="I60" s="221"/>
       <c r="J60" s="101"/>
       <c r="K60" s="96"/>
       <c r="L60" s="97"/>
       <c r="M60" s="97"/>
-      <c r="N60" s="239">
+      <c r="N60" s="243">
         <v>46099</v>
       </c>
-      <c r="O60" s="239">
+      <c r="O60" s="243">
         <v>46100</v>
       </c>
-      <c r="P60" s="239">
+      <c r="P60" s="243">
         <v>46101</v>
       </c>
-      <c r="Q60" s="239">
+      <c r="Q60" s="243">
         <v>46102</v>
       </c>
-      <c r="R60" s="239">
+      <c r="R60" s="243">
         <v>46103</v>
       </c>
-      <c r="S60" s="239">
+      <c r="S60" s="243">
         <v>46104</v>
       </c>
-      <c r="T60" s="239">
+      <c r="T60" s="243">
         <v>46105</v>
       </c>
-      <c r="U60" s="243">
+      <c r="U60" s="247">
         <v>46108</v>
       </c>
-      <c r="V60" s="243">
+      <c r="V60" s="247">
         <v>46109</v>
       </c>
-      <c r="W60" s="243">
+      <c r="W60" s="247">
         <v>46112</v>
       </c>
-      <c r="X60" s="243">
+      <c r="X60" s="247">
         <v>46113</v>
       </c>
-      <c r="Y60" s="243">
+      <c r="Y60" s="247">
         <v>46114</v>
       </c>
-      <c r="Z60" s="243">
+      <c r="Z60" s="247">
         <v>46115</v>
       </c>
-      <c r="AA60" s="243">
+      <c r="AA60" s="247">
         <v>46116</v>
       </c>
-      <c r="AB60" s="260">
+      <c r="AB60" s="264">
         <v>46117</v>
       </c>
       <c r="AC60" s="192"/>
-      <c r="AD60" s="245" t="s">
+      <c r="AD60" s="249" t="s">
         <v>18</v>
       </c>
-      <c r="AE60" s="257" t="s">
+      <c r="AE60" s="261" t="s">
         <v>19</v>
       </c>
       <c r="AG60" s="31"/>
@@ -7431,187 +7452,187 @@
       <c r="AI60" s="32"/>
     </row>
     <row r="61" spans="1:35" ht="12.75" customHeight="1">
-      <c r="B61" s="237"/>
-      <c r="C61" s="237"/>
-      <c r="D61" s="217"/>
-      <c r="E61" s="220"/>
-      <c r="F61" s="217"/>
-      <c r="G61" s="217"/>
-      <c r="H61" s="217"/>
-      <c r="I61" s="217"/>
+      <c r="B61" s="241"/>
+      <c r="C61" s="241"/>
+      <c r="D61" s="221"/>
+      <c r="E61" s="224"/>
+      <c r="F61" s="221"/>
+      <c r="G61" s="221"/>
+      <c r="H61" s="221"/>
+      <c r="I61" s="221"/>
       <c r="J61" s="101"/>
       <c r="K61" s="98"/>
       <c r="L61" s="97"/>
       <c r="M61" s="97"/>
-      <c r="N61" s="239"/>
-      <c r="O61" s="239"/>
-      <c r="P61" s="239"/>
-      <c r="Q61" s="239"/>
-      <c r="R61" s="239"/>
-      <c r="S61" s="239"/>
-      <c r="T61" s="239"/>
-      <c r="U61" s="243"/>
-      <c r="V61" s="243"/>
-      <c r="W61" s="243"/>
-      <c r="X61" s="243"/>
-      <c r="Y61" s="243"/>
-      <c r="Z61" s="243"/>
-      <c r="AA61" s="243"/>
-      <c r="AB61" s="260"/>
+      <c r="N61" s="243"/>
+      <c r="O61" s="243"/>
+      <c r="P61" s="243"/>
+      <c r="Q61" s="243"/>
+      <c r="R61" s="243"/>
+      <c r="S61" s="243"/>
+      <c r="T61" s="243"/>
+      <c r="U61" s="247"/>
+      <c r="V61" s="247"/>
+      <c r="W61" s="247"/>
+      <c r="X61" s="247"/>
+      <c r="Y61" s="247"/>
+      <c r="Z61" s="247"/>
+      <c r="AA61" s="247"/>
+      <c r="AB61" s="264"/>
       <c r="AC61" s="192"/>
-      <c r="AD61" s="246"/>
-      <c r="AE61" s="258"/>
+      <c r="AD61" s="250"/>
+      <c r="AE61" s="262"/>
       <c r="AG61" s="31"/>
       <c r="AH61" s="32"/>
       <c r="AI61" s="32"/>
     </row>
     <row r="62" spans="1:35" ht="12.75" customHeight="1">
-      <c r="B62" s="237"/>
-      <c r="C62" s="237"/>
-      <c r="D62" s="217"/>
-      <c r="E62" s="220"/>
-      <c r="F62" s="217"/>
-      <c r="G62" s="217"/>
-      <c r="H62" s="217"/>
-      <c r="I62" s="217"/>
+      <c r="B62" s="241"/>
+      <c r="C62" s="241"/>
+      <c r="D62" s="221"/>
+      <c r="E62" s="224"/>
+      <c r="F62" s="221"/>
+      <c r="G62" s="221"/>
+      <c r="H62" s="221"/>
+      <c r="I62" s="221"/>
       <c r="J62" s="101"/>
       <c r="K62" s="98"/>
       <c r="L62" s="97"/>
       <c r="M62" s="97"/>
-      <c r="N62" s="239"/>
-      <c r="O62" s="239"/>
-      <c r="P62" s="239"/>
-      <c r="Q62" s="239"/>
-      <c r="R62" s="239"/>
-      <c r="S62" s="239"/>
-      <c r="T62" s="239"/>
-      <c r="U62" s="243"/>
-      <c r="V62" s="243"/>
-      <c r="W62" s="243"/>
-      <c r="X62" s="243"/>
-      <c r="Y62" s="243"/>
-      <c r="Z62" s="243"/>
-      <c r="AA62" s="243"/>
-      <c r="AB62" s="260"/>
+      <c r="N62" s="243"/>
+      <c r="O62" s="243"/>
+      <c r="P62" s="243"/>
+      <c r="Q62" s="243"/>
+      <c r="R62" s="243"/>
+      <c r="S62" s="243"/>
+      <c r="T62" s="243"/>
+      <c r="U62" s="247"/>
+      <c r="V62" s="247"/>
+      <c r="W62" s="247"/>
+      <c r="X62" s="247"/>
+      <c r="Y62" s="247"/>
+      <c r="Z62" s="247"/>
+      <c r="AA62" s="247"/>
+      <c r="AB62" s="264"/>
       <c r="AC62" s="192"/>
-      <c r="AD62" s="246"/>
-      <c r="AE62" s="258"/>
+      <c r="AD62" s="250"/>
+      <c r="AE62" s="262"/>
       <c r="AG62" s="31"/>
       <c r="AH62" s="32"/>
       <c r="AI62" s="32"/>
     </row>
     <row r="63" spans="1:35" ht="12.75" customHeight="1">
-      <c r="B63" s="237"/>
-      <c r="C63" s="237"/>
-      <c r="D63" s="217"/>
-      <c r="E63" s="220"/>
-      <c r="F63" s="217"/>
-      <c r="G63" s="217"/>
-      <c r="H63" s="217"/>
-      <c r="I63" s="217"/>
+      <c r="B63" s="241"/>
+      <c r="C63" s="241"/>
+      <c r="D63" s="221"/>
+      <c r="E63" s="224"/>
+      <c r="F63" s="221"/>
+      <c r="G63" s="221"/>
+      <c r="H63" s="221"/>
+      <c r="I63" s="221"/>
       <c r="J63" s="101"/>
       <c r="K63" s="99"/>
       <c r="L63" s="97"/>
       <c r="M63" s="97"/>
-      <c r="N63" s="239"/>
-      <c r="O63" s="239"/>
-      <c r="P63" s="239"/>
-      <c r="Q63" s="239"/>
-      <c r="R63" s="239"/>
-      <c r="S63" s="239"/>
-      <c r="T63" s="239"/>
-      <c r="U63" s="243"/>
-      <c r="V63" s="243"/>
-      <c r="W63" s="243"/>
-      <c r="X63" s="243"/>
-      <c r="Y63" s="243"/>
-      <c r="Z63" s="243"/>
-      <c r="AA63" s="243"/>
-      <c r="AB63" s="260"/>
+      <c r="N63" s="243"/>
+      <c r="O63" s="243"/>
+      <c r="P63" s="243"/>
+      <c r="Q63" s="243"/>
+      <c r="R63" s="243"/>
+      <c r="S63" s="243"/>
+      <c r="T63" s="243"/>
+      <c r="U63" s="247"/>
+      <c r="V63" s="247"/>
+      <c r="W63" s="247"/>
+      <c r="X63" s="247"/>
+      <c r="Y63" s="247"/>
+      <c r="Z63" s="247"/>
+      <c r="AA63" s="247"/>
+      <c r="AB63" s="264"/>
       <c r="AC63" s="192"/>
-      <c r="AD63" s="246"/>
-      <c r="AE63" s="258"/>
+      <c r="AD63" s="250"/>
+      <c r="AE63" s="262"/>
       <c r="AH63" s="32"/>
       <c r="AI63" s="32"/>
     </row>
     <row r="64" spans="1:35" ht="12.75" customHeight="1">
-      <c r="B64" s="237"/>
-      <c r="C64" s="237"/>
-      <c r="D64" s="217"/>
-      <c r="E64" s="220"/>
-      <c r="F64" s="217"/>
-      <c r="G64" s="217"/>
-      <c r="H64" s="217"/>
-      <c r="I64" s="217"/>
+      <c r="B64" s="241"/>
+      <c r="C64" s="241"/>
+      <c r="D64" s="221"/>
+      <c r="E64" s="224"/>
+      <c r="F64" s="221"/>
+      <c r="G64" s="221"/>
+      <c r="H64" s="221"/>
+      <c r="I64" s="221"/>
       <c r="J64" s="101"/>
       <c r="K64" s="96"/>
       <c r="L64" s="97"/>
       <c r="M64" s="97"/>
-      <c r="N64" s="239"/>
-      <c r="O64" s="239"/>
-      <c r="P64" s="239"/>
-      <c r="Q64" s="239"/>
-      <c r="R64" s="239"/>
-      <c r="S64" s="239"/>
-      <c r="T64" s="239"/>
-      <c r="U64" s="243"/>
-      <c r="V64" s="243"/>
-      <c r="W64" s="243"/>
-      <c r="X64" s="243"/>
-      <c r="Y64" s="243"/>
-      <c r="Z64" s="243"/>
-      <c r="AA64" s="243"/>
-      <c r="AB64" s="260"/>
+      <c r="N64" s="243"/>
+      <c r="O64" s="243"/>
+      <c r="P64" s="243"/>
+      <c r="Q64" s="243"/>
+      <c r="R64" s="243"/>
+      <c r="S64" s="243"/>
+      <c r="T64" s="243"/>
+      <c r="U64" s="247"/>
+      <c r="V64" s="247"/>
+      <c r="W64" s="247"/>
+      <c r="X64" s="247"/>
+      <c r="Y64" s="247"/>
+      <c r="Z64" s="247"/>
+      <c r="AA64" s="247"/>
+      <c r="AB64" s="264"/>
       <c r="AC64" s="192"/>
-      <c r="AD64" s="246"/>
-      <c r="AE64" s="258"/>
+      <c r="AD64" s="250"/>
+      <c r="AE64" s="262"/>
       <c r="AH64" s="32"/>
       <c r="AI64" s="32"/>
     </row>
     <row r="65" spans="2:35" ht="12.6" customHeight="1" thickBot="1">
-      <c r="B65" s="237"/>
-      <c r="C65" s="237"/>
-      <c r="D65" s="217"/>
-      <c r="E65" s="220"/>
-      <c r="F65" s="217"/>
-      <c r="G65" s="217"/>
-      <c r="H65" s="217"/>
-      <c r="I65" s="217"/>
+      <c r="B65" s="241"/>
+      <c r="C65" s="241"/>
+      <c r="D65" s="221"/>
+      <c r="E65" s="224"/>
+      <c r="F65" s="221"/>
+      <c r="G65" s="221"/>
+      <c r="H65" s="221"/>
+      <c r="I65" s="221"/>
       <c r="J65" s="101"/>
       <c r="K65" s="100"/>
       <c r="L65" s="97"/>
       <c r="M65" s="97"/>
-      <c r="N65" s="240"/>
-      <c r="O65" s="240"/>
-      <c r="P65" s="240"/>
-      <c r="Q65" s="240"/>
-      <c r="R65" s="240"/>
-      <c r="S65" s="240"/>
-      <c r="T65" s="240"/>
-      <c r="U65" s="244"/>
-      <c r="V65" s="244"/>
-      <c r="W65" s="244"/>
-      <c r="X65" s="244"/>
-      <c r="Y65" s="244"/>
-      <c r="Z65" s="244"/>
-      <c r="AA65" s="244"/>
-      <c r="AB65" s="261"/>
+      <c r="N65" s="244"/>
+      <c r="O65" s="244"/>
+      <c r="P65" s="244"/>
+      <c r="Q65" s="244"/>
+      <c r="R65" s="244"/>
+      <c r="S65" s="244"/>
+      <c r="T65" s="244"/>
+      <c r="U65" s="248"/>
+      <c r="V65" s="248"/>
+      <c r="W65" s="248"/>
+      <c r="X65" s="248"/>
+      <c r="Y65" s="248"/>
+      <c r="Z65" s="248"/>
+      <c r="AA65" s="248"/>
+      <c r="AB65" s="265"/>
       <c r="AC65" s="193"/>
-      <c r="AD65" s="247"/>
-      <c r="AE65" s="259"/>
+      <c r="AD65" s="251"/>
+      <c r="AE65" s="263"/>
       <c r="AG65" s="23"/>
       <c r="AH65" s="23"/>
       <c r="AI65" s="23"/>
     </row>
     <row r="66" spans="2:35" ht="15" customHeight="1">
-      <c r="B66" s="237"/>
-      <c r="C66" s="237"/>
-      <c r="D66" s="217"/>
-      <c r="E66" s="220"/>
-      <c r="F66" s="217"/>
-      <c r="G66" s="217"/>
-      <c r="H66" s="217"/>
-      <c r="I66" s="217"/>
+      <c r="B66" s="241"/>
+      <c r="C66" s="241"/>
+      <c r="D66" s="221"/>
+      <c r="E66" s="224"/>
+      <c r="F66" s="221"/>
+      <c r="G66" s="221"/>
+      <c r="H66" s="221"/>
+      <c r="I66" s="221"/>
       <c r="J66" s="101"/>
       <c r="K66" s="100"/>
       <c r="L66" s="100"/>
@@ -7635,20 +7656,20 @@
       <c r="AD66" s="103"/>
       <c r="AE66" s="104"/>
       <c r="AG66" s="23"/>
-      <c r="AH66" s="250" t="s">
+      <c r="AH66" s="254" t="s">
         <v>6</v>
       </c>
-      <c r="AI66" s="250"/>
+      <c r="AI66" s="254"/>
     </row>
     <row r="67" spans="2:35" ht="15.75" customHeight="1">
-      <c r="B67" s="237"/>
-      <c r="C67" s="237"/>
-      <c r="D67" s="217"/>
-      <c r="E67" s="220"/>
-      <c r="F67" s="217"/>
-      <c r="G67" s="217"/>
-      <c r="H67" s="217"/>
-      <c r="I67" s="217"/>
+      <c r="B67" s="241"/>
+      <c r="C67" s="241"/>
+      <c r="D67" s="221"/>
+      <c r="E67" s="224"/>
+      <c r="F67" s="221"/>
+      <c r="G67" s="221"/>
+      <c r="H67" s="221"/>
+      <c r="I67" s="221"/>
       <c r="J67" s="105"/>
       <c r="K67" s="100"/>
       <c r="L67" s="98"/>
@@ -7682,14 +7703,14 @@
       </c>
     </row>
     <row r="68" spans="2:35" ht="12.75" customHeight="1">
-      <c r="B68" s="237"/>
-      <c r="C68" s="237"/>
-      <c r="D68" s="217"/>
-      <c r="E68" s="220"/>
-      <c r="F68" s="217"/>
-      <c r="G68" s="217"/>
-      <c r="H68" s="217"/>
-      <c r="I68" s="217"/>
+      <c r="B68" s="241"/>
+      <c r="C68" s="241"/>
+      <c r="D68" s="221"/>
+      <c r="E68" s="224"/>
+      <c r="F68" s="221"/>
+      <c r="G68" s="221"/>
+      <c r="H68" s="221"/>
+      <c r="I68" s="221"/>
       <c r="J68" s="101"/>
       <c r="K68" s="96"/>
       <c r="L68" s="98"/>
@@ -7719,14 +7740,14 @@
       <c r="AI68" s="111"/>
     </row>
     <row r="69" spans="2:35" ht="15.6">
-      <c r="B69" s="237"/>
-      <c r="C69" s="237"/>
-      <c r="D69" s="217"/>
-      <c r="E69" s="220"/>
-      <c r="F69" s="217"/>
-      <c r="G69" s="217"/>
-      <c r="H69" s="217"/>
-      <c r="I69" s="217"/>
+      <c r="B69" s="241"/>
+      <c r="C69" s="241"/>
+      <c r="D69" s="221"/>
+      <c r="E69" s="224"/>
+      <c r="F69" s="221"/>
+      <c r="G69" s="221"/>
+      <c r="H69" s="221"/>
+      <c r="I69" s="221"/>
       <c r="J69" s="101"/>
       <c r="K69" s="96"/>
       <c r="L69" s="98"/>
@@ -7756,14 +7777,14 @@
       <c r="AI69" s="113"/>
     </row>
     <row r="70" spans="2:35" ht="15" customHeight="1">
-      <c r="B70" s="237"/>
-      <c r="C70" s="237"/>
-      <c r="D70" s="217"/>
-      <c r="E70" s="220"/>
-      <c r="F70" s="217"/>
-      <c r="G70" s="217"/>
-      <c r="H70" s="217"/>
-      <c r="I70" s="217"/>
+      <c r="B70" s="241"/>
+      <c r="C70" s="241"/>
+      <c r="D70" s="221"/>
+      <c r="E70" s="224"/>
+      <c r="F70" s="221"/>
+      <c r="G70" s="221"/>
+      <c r="H70" s="221"/>
+      <c r="I70" s="221"/>
       <c r="J70" s="101"/>
       <c r="K70" s="96"/>
       <c r="L70" s="96"/>
@@ -7793,14 +7814,14 @@
       <c r="AI70" s="111"/>
     </row>
     <row r="71" spans="2:35" ht="15.6">
-      <c r="B71" s="237"/>
-      <c r="C71" s="237"/>
-      <c r="D71" s="217"/>
-      <c r="E71" s="220"/>
-      <c r="F71" s="217"/>
-      <c r="G71" s="217"/>
-      <c r="H71" s="217"/>
-      <c r="I71" s="217"/>
+      <c r="B71" s="241"/>
+      <c r="C71" s="241"/>
+      <c r="D71" s="221"/>
+      <c r="E71" s="224"/>
+      <c r="F71" s="221"/>
+      <c r="G71" s="221"/>
+      <c r="H71" s="221"/>
+      <c r="I71" s="221"/>
       <c r="J71" s="101"/>
       <c r="K71" s="114"/>
       <c r="L71" s="101"/>
@@ -7827,14 +7848,14 @@
       <c r="AH71" s="115"/>
     </row>
     <row r="72" spans="2:35" ht="15.45" customHeight="1" thickBot="1">
-      <c r="B72" s="237"/>
-      <c r="C72" s="237"/>
-      <c r="D72" s="217"/>
-      <c r="E72" s="220"/>
-      <c r="F72" s="217"/>
-      <c r="G72" s="217"/>
-      <c r="H72" s="217"/>
-      <c r="I72" s="217"/>
+      <c r="B72" s="241"/>
+      <c r="C72" s="241"/>
+      <c r="D72" s="221"/>
+      <c r="E72" s="224"/>
+      <c r="F72" s="221"/>
+      <c r="G72" s="221"/>
+      <c r="H72" s="221"/>
+      <c r="I72" s="221"/>
       <c r="J72" s="117"/>
       <c r="K72" s="116"/>
       <c r="L72" s="117"/>
@@ -7861,132 +7882,132 @@
       <c r="AI72" s="115"/>
     </row>
     <row r="73" spans="2:35" ht="15" customHeight="1">
-      <c r="B73" s="237"/>
-      <c r="C73" s="237"/>
-      <c r="D73" s="217"/>
-      <c r="E73" s="220"/>
-      <c r="F73" s="217"/>
-      <c r="G73" s="217"/>
-      <c r="H73" s="217"/>
-      <c r="I73" s="217"/>
-      <c r="J73" s="251"/>
-      <c r="K73" s="251"/>
-      <c r="L73" s="251"/>
-      <c r="M73" s="251"/>
-      <c r="N73" s="251"/>
-      <c r="O73" s="251"/>
-      <c r="P73" s="251"/>
-      <c r="Q73" s="251"/>
-      <c r="R73" s="251"/>
-      <c r="S73" s="251"/>
-      <c r="T73" s="251"/>
-      <c r="U73" s="251"/>
-      <c r="V73" s="251"/>
-      <c r="W73" s="251"/>
-      <c r="X73" s="251"/>
-      <c r="Y73" s="251"/>
-      <c r="Z73" s="251"/>
-      <c r="AA73" s="251"/>
-      <c r="AB73" s="251"/>
-      <c r="AC73" s="251"/>
-      <c r="AD73" s="251"/>
-      <c r="AE73" s="252"/>
+      <c r="B73" s="241"/>
+      <c r="C73" s="241"/>
+      <c r="D73" s="221"/>
+      <c r="E73" s="224"/>
+      <c r="F73" s="221"/>
+      <c r="G73" s="221"/>
+      <c r="H73" s="221"/>
+      <c r="I73" s="221"/>
+      <c r="J73" s="255"/>
+      <c r="K73" s="255"/>
+      <c r="L73" s="255"/>
+      <c r="M73" s="255"/>
+      <c r="N73" s="255"/>
+      <c r="O73" s="255"/>
+      <c r="P73" s="255"/>
+      <c r="Q73" s="255"/>
+      <c r="R73" s="255"/>
+      <c r="S73" s="255"/>
+      <c r="T73" s="255"/>
+      <c r="U73" s="255"/>
+      <c r="V73" s="255"/>
+      <c r="W73" s="255"/>
+      <c r="X73" s="255"/>
+      <c r="Y73" s="255"/>
+      <c r="Z73" s="255"/>
+      <c r="AA73" s="255"/>
+      <c r="AB73" s="255"/>
+      <c r="AC73" s="255"/>
+      <c r="AD73" s="255"/>
+      <c r="AE73" s="256"/>
     </row>
     <row r="74" spans="2:35" ht="15" customHeight="1">
-      <c r="B74" s="237"/>
-      <c r="C74" s="237"/>
-      <c r="D74" s="217"/>
-      <c r="E74" s="220"/>
-      <c r="F74" s="217"/>
-      <c r="G74" s="217"/>
-      <c r="H74" s="217"/>
-      <c r="I74" s="217"/>
-      <c r="J74" s="253"/>
-      <c r="K74" s="253"/>
-      <c r="L74" s="253"/>
-      <c r="M74" s="253"/>
-      <c r="N74" s="253"/>
-      <c r="O74" s="253"/>
-      <c r="P74" s="253"/>
-      <c r="Q74" s="253"/>
-      <c r="R74" s="253"/>
-      <c r="S74" s="253"/>
-      <c r="T74" s="253"/>
-      <c r="U74" s="253"/>
-      <c r="V74" s="253"/>
-      <c r="W74" s="253"/>
-      <c r="X74" s="253"/>
-      <c r="Y74" s="253"/>
-      <c r="Z74" s="253"/>
-      <c r="AA74" s="253"/>
-      <c r="AB74" s="253"/>
-      <c r="AC74" s="253"/>
-      <c r="AD74" s="253"/>
-      <c r="AE74" s="254"/>
+      <c r="B74" s="241"/>
+      <c r="C74" s="241"/>
+      <c r="D74" s="221"/>
+      <c r="E74" s="224"/>
+      <c r="F74" s="221"/>
+      <c r="G74" s="221"/>
+      <c r="H74" s="221"/>
+      <c r="I74" s="221"/>
+      <c r="J74" s="257"/>
+      <c r="K74" s="257"/>
+      <c r="L74" s="257"/>
+      <c r="M74" s="257"/>
+      <c r="N74" s="257"/>
+      <c r="O74" s="257"/>
+      <c r="P74" s="257"/>
+      <c r="Q74" s="257"/>
+      <c r="R74" s="257"/>
+      <c r="S74" s="257"/>
+      <c r="T74" s="257"/>
+      <c r="U74" s="257"/>
+      <c r="V74" s="257"/>
+      <c r="W74" s="257"/>
+      <c r="X74" s="257"/>
+      <c r="Y74" s="257"/>
+      <c r="Z74" s="257"/>
+      <c r="AA74" s="257"/>
+      <c r="AB74" s="257"/>
+      <c r="AC74" s="257"/>
+      <c r="AD74" s="257"/>
+      <c r="AE74" s="258"/>
     </row>
     <row r="75" spans="2:35" ht="15" customHeight="1">
-      <c r="B75" s="237"/>
-      <c r="C75" s="237"/>
-      <c r="D75" s="217"/>
-      <c r="E75" s="220"/>
-      <c r="F75" s="217"/>
-      <c r="G75" s="217"/>
-      <c r="H75" s="217"/>
-      <c r="I75" s="217"/>
-      <c r="J75" s="253"/>
-      <c r="K75" s="253"/>
-      <c r="L75" s="253"/>
-      <c r="M75" s="253"/>
-      <c r="N75" s="253"/>
-      <c r="O75" s="253"/>
-      <c r="P75" s="253"/>
-      <c r="Q75" s="253"/>
-      <c r="R75" s="253"/>
-      <c r="S75" s="253"/>
-      <c r="T75" s="253"/>
-      <c r="U75" s="253"/>
-      <c r="V75" s="253"/>
-      <c r="W75" s="253"/>
-      <c r="X75" s="253"/>
-      <c r="Y75" s="253"/>
-      <c r="Z75" s="253"/>
-      <c r="AA75" s="253"/>
-      <c r="AB75" s="253"/>
-      <c r="AC75" s="253"/>
-      <c r="AD75" s="253"/>
-      <c r="AE75" s="254"/>
+      <c r="B75" s="241"/>
+      <c r="C75" s="241"/>
+      <c r="D75" s="221"/>
+      <c r="E75" s="224"/>
+      <c r="F75" s="221"/>
+      <c r="G75" s="221"/>
+      <c r="H75" s="221"/>
+      <c r="I75" s="221"/>
+      <c r="J75" s="257"/>
+      <c r="K75" s="257"/>
+      <c r="L75" s="257"/>
+      <c r="M75" s="257"/>
+      <c r="N75" s="257"/>
+      <c r="O75" s="257"/>
+      <c r="P75" s="257"/>
+      <c r="Q75" s="257"/>
+      <c r="R75" s="257"/>
+      <c r="S75" s="257"/>
+      <c r="T75" s="257"/>
+      <c r="U75" s="257"/>
+      <c r="V75" s="257"/>
+      <c r="W75" s="257"/>
+      <c r="X75" s="257"/>
+      <c r="Y75" s="257"/>
+      <c r="Z75" s="257"/>
+      <c r="AA75" s="257"/>
+      <c r="AB75" s="257"/>
+      <c r="AC75" s="257"/>
+      <c r="AD75" s="257"/>
+      <c r="AE75" s="258"/>
     </row>
     <row r="76" spans="2:35" s="1" customFormat="1" ht="15.45" customHeight="1" thickBot="1">
-      <c r="B76" s="238"/>
-      <c r="C76" s="238"/>
-      <c r="D76" s="218"/>
-      <c r="E76" s="221"/>
-      <c r="F76" s="218"/>
-      <c r="G76" s="218"/>
-      <c r="H76" s="218"/>
-      <c r="I76" s="218"/>
-      <c r="J76" s="241"/>
-      <c r="K76" s="241"/>
-      <c r="L76" s="241"/>
-      <c r="M76" s="241"/>
-      <c r="N76" s="241"/>
-      <c r="O76" s="241"/>
-      <c r="P76" s="241"/>
-      <c r="Q76" s="241"/>
-      <c r="R76" s="241"/>
-      <c r="S76" s="241"/>
-      <c r="T76" s="241"/>
-      <c r="U76" s="241"/>
-      <c r="V76" s="241"/>
-      <c r="W76" s="241"/>
-      <c r="X76" s="241"/>
-      <c r="Y76" s="241"/>
-      <c r="Z76" s="241"/>
-      <c r="AA76" s="241"/>
-      <c r="AB76" s="241"/>
-      <c r="AC76" s="241"/>
-      <c r="AD76" s="241"/>
-      <c r="AE76" s="242"/>
+      <c r="B76" s="242"/>
+      <c r="C76" s="242"/>
+      <c r="D76" s="222"/>
+      <c r="E76" s="225"/>
+      <c r="F76" s="222"/>
+      <c r="G76" s="222"/>
+      <c r="H76" s="222"/>
+      <c r="I76" s="222"/>
+      <c r="J76" s="245"/>
+      <c r="K76" s="245"/>
+      <c r="L76" s="245"/>
+      <c r="M76" s="245"/>
+      <c r="N76" s="245"/>
+      <c r="O76" s="245"/>
+      <c r="P76" s="245"/>
+      <c r="Q76" s="245"/>
+      <c r="R76" s="245"/>
+      <c r="S76" s="245"/>
+      <c r="T76" s="245"/>
+      <c r="U76" s="245"/>
+      <c r="V76" s="245"/>
+      <c r="W76" s="245"/>
+      <c r="X76" s="245"/>
+      <c r="Y76" s="245"/>
+      <c r="Z76" s="245"/>
+      <c r="AA76" s="245"/>
+      <c r="AB76" s="245"/>
+      <c r="AC76" s="245"/>
+      <c r="AD76" s="245"/>
+      <c r="AE76" s="246"/>
       <c r="AG76" s="23"/>
       <c r="AH76" s="24"/>
       <c r="AI76" s="24"/>
@@ -8016,15 +8037,15 @@
       <c r="U78" s="131" t="s">
         <v>15</v>
       </c>
-      <c r="V78" s="255" t="s">
+      <c r="V78" s="259" t="s">
         <v>23</v>
       </c>
-      <c r="W78" s="256"/>
-      <c r="X78" s="256"/>
-      <c r="Y78" s="256"/>
-      <c r="Z78" s="256"/>
-      <c r="AA78" s="256"/>
-      <c r="AB78" s="256"/>
+      <c r="W78" s="260"/>
+      <c r="X78" s="260"/>
+      <c r="Y78" s="260"/>
+      <c r="Z78" s="260"/>
+      <c r="AA78" s="260"/>
+      <c r="AB78" s="260"/>
       <c r="AC78" s="194"/>
       <c r="AE78" s="123"/>
       <c r="AF78" s="123"/>
@@ -8054,15 +8075,15 @@
       <c r="U79" s="138" t="s">
         <v>16</v>
       </c>
-      <c r="V79" s="255" t="s">
+      <c r="V79" s="259" t="s">
         <v>24</v>
       </c>
-      <c r="W79" s="256"/>
-      <c r="X79" s="256"/>
-      <c r="Y79" s="256"/>
-      <c r="Z79" s="256"/>
-      <c r="AA79" s="256"/>
-      <c r="AB79" s="256"/>
+      <c r="W79" s="260"/>
+      <c r="X79" s="260"/>
+      <c r="Y79" s="260"/>
+      <c r="Z79" s="260"/>
+      <c r="AA79" s="260"/>
+      <c r="AB79" s="260"/>
       <c r="AC79" s="194"/>
       <c r="AE79" s="125"/>
       <c r="AF79" s="125"/>
@@ -8093,15 +8114,15 @@
       <c r="U80" s="146" t="s">
         <v>17</v>
       </c>
-      <c r="V80" s="255" t="s">
+      <c r="V80" s="259" t="s">
         <v>25</v>
       </c>
-      <c r="W80" s="256"/>
-      <c r="X80" s="256"/>
-      <c r="Y80" s="256"/>
-      <c r="Z80" s="256"/>
-      <c r="AA80" s="256"/>
-      <c r="AB80" s="256"/>
+      <c r="W80" s="260"/>
+      <c r="X80" s="260"/>
+      <c r="Y80" s="260"/>
+      <c r="Z80" s="260"/>
+      <c r="AA80" s="260"/>
+      <c r="AB80" s="260"/>
       <c r="AC80" s="194"/>
       <c r="AE80" s="121"/>
       <c r="AF80" s="121"/>
@@ -8328,7 +8349,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:6">
-      <c r="A2" s="266" t="s">
+      <c r="A2" s="217" t="s">
         <v>190</v>
       </c>
       <c r="B2" s="211" t="s">
@@ -8347,29 +8368,29 @@
         <v>124</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
-      <c r="A3" s="266">
+    <row r="3" spans="1:6" s="220" customFormat="1">
+      <c r="A3" s="218">
         <v>1</v>
       </c>
-      <c r="B3" s="262" t="s">
+      <c r="B3" s="266" t="s">
         <v>157</v>
       </c>
-      <c r="C3" s="208"/>
-      <c r="D3" s="209" t="s">
+      <c r="C3" s="219"/>
+      <c r="D3" s="219" t="s">
         <v>148</v>
       </c>
-      <c r="E3" s="208"/>
-      <c r="F3" s="208" t="s">
+      <c r="E3" s="219"/>
+      <c r="F3" s="219" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="31.2">
-      <c r="A4" s="266">
+      <c r="A4" s="216">
         <v>2</v>
       </c>
-      <c r="B4" s="263"/>
+      <c r="B4" s="267"/>
       <c r="C4" s="208"/>
-      <c r="D4" s="212" t="s">
+      <c r="D4" s="270" t="s">
         <v>149</v>
       </c>
       <c r="E4" s="208"/>
@@ -8378,7 +8399,7 @@
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="266">
+      <c r="A5" s="216">
         <v>3</v>
       </c>
       <c r="B5" s="210" t="s">
@@ -8396,7 +8417,7 @@
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="266">
+      <c r="A6" s="216">
         <v>4</v>
       </c>
       <c r="B6" s="210" t="s">
@@ -8414,10 +8435,10 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="31.2">
-      <c r="A7" s="266">
+      <c r="A7" s="216">
         <v>5</v>
       </c>
-      <c r="B7" s="262" t="s">
+      <c r="B7" s="266" t="s">
         <v>144</v>
       </c>
       <c r="C7" s="208" t="s">
@@ -8434,10 +8455,10 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="31.2">
-      <c r="A8" s="266">
+      <c r="A8" s="216">
         <v>6</v>
       </c>
-      <c r="B8" s="263"/>
+      <c r="B8" s="267"/>
       <c r="C8" s="208" t="s">
         <v>150</v>
       </c>
@@ -8448,10 +8469,10 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="31.2">
-      <c r="A9" s="266">
+      <c r="A9" s="216">
         <v>7</v>
       </c>
-      <c r="B9" s="262" t="s">
+      <c r="B9" s="266" t="s">
         <v>145</v>
       </c>
       <c r="C9" s="208" t="s">
@@ -8468,10 +8489,10 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="31.2">
-      <c r="A10" s="266">
+      <c r="A10" s="216">
         <v>8</v>
       </c>
-      <c r="B10" s="263"/>
+      <c r="B10" s="267"/>
       <c r="C10" s="208" t="s">
         <v>141</v>
       </c>
@@ -8482,10 +8503,10 @@
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="266">
+      <c r="A11" s="216">
         <v>9</v>
       </c>
-      <c r="B11" s="262" t="s">
+      <c r="B11" s="266" t="s">
         <v>143</v>
       </c>
       <c r="C11" s="208"/>
@@ -8498,10 +8519,10 @@
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="266">
+      <c r="A12" s="216">
         <v>10</v>
       </c>
-      <c r="B12" s="263"/>
+      <c r="B12" s="267"/>
       <c r="C12" s="208"/>
       <c r="D12" s="209" t="s">
         <v>128</v>
@@ -8511,27 +8532,27 @@
         <v>126</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
-      <c r="A13" s="266">
+    <row r="13" spans="1:6" s="220" customFormat="1">
+      <c r="A13" s="218">
         <v>11</v>
       </c>
-      <c r="B13" s="262" t="s">
+      <c r="B13" s="266" t="s">
         <v>131</v>
       </c>
-      <c r="C13" s="208"/>
-      <c r="D13" s="208" t="s">
+      <c r="C13" s="219"/>
+      <c r="D13" s="219" t="s">
         <v>132</v>
       </c>
-      <c r="E13" s="208"/>
-      <c r="F13" s="208" t="s">
-        <v>126</v>
+      <c r="E13" s="219"/>
+      <c r="F13" s="219" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="266">
+      <c r="A14" s="216">
         <v>12</v>
       </c>
-      <c r="B14" s="263"/>
+      <c r="B14" s="267"/>
       <c r="C14" s="208"/>
       <c r="D14" s="209" t="s">
         <v>133</v>
@@ -8542,7 +8563,7 @@
       </c>
     </row>
     <row r="15" spans="1:6" ht="31.2">
-      <c r="A15" s="266">
+      <c r="A15" s="216">
         <v>13</v>
       </c>
       <c r="B15" s="210" t="s">
@@ -8560,7 +8581,7 @@
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="266">
+      <c r="A16" s="216">
         <v>14</v>
       </c>
       <c r="B16" s="210" t="s">
@@ -8576,10 +8597,10 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="31.2">
-      <c r="A17" s="266">
+      <c r="A17" s="216">
         <v>15</v>
       </c>
-      <c r="B17" s="262" t="s">
+      <c r="B17" s="266" t="s">
         <v>151</v>
       </c>
       <c r="C17" s="208" t="s">
@@ -8594,10 +8615,10 @@
       </c>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="266">
+      <c r="A18" s="216">
         <v>16</v>
       </c>
-      <c r="B18" s="263"/>
+      <c r="B18" s="267"/>
       <c r="C18" s="208"/>
       <c r="D18" s="208" t="s">
         <v>154</v>
@@ -8608,10 +8629,10 @@
       </c>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="266">
+      <c r="A19" s="216">
         <v>17</v>
       </c>
-      <c r="B19" s="262" t="s">
+      <c r="B19" s="266" t="s">
         <v>161</v>
       </c>
       <c r="C19" s="208" t="s">
@@ -8626,10 +8647,10 @@
       </c>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="266">
+      <c r="A20" s="216">
         <v>18</v>
       </c>
-      <c r="B20" s="263"/>
+      <c r="B20" s="267"/>
       <c r="C20" s="208"/>
       <c r="D20" s="208" t="s">
         <v>164</v>
@@ -8640,7 +8661,7 @@
       </c>
     </row>
     <row r="21" spans="1:6" ht="31.2">
-      <c r="A21" s="266">
+      <c r="A21" s="216">
         <v>19</v>
       </c>
       <c r="B21" s="210" t="s">
@@ -8656,7 +8677,7 @@
       </c>
     </row>
     <row r="22" spans="1:6" ht="31.2">
-      <c r="A22" s="266">
+      <c r="A22" s="216">
         <v>20</v>
       </c>
       <c r="B22" s="210" t="s">
@@ -8674,7 +8695,7 @@
       </c>
     </row>
     <row r="23" spans="1:6" ht="31.2">
-      <c r="A23" s="266">
+      <c r="A23" s="216">
         <v>21</v>
       </c>
       <c r="B23" s="210"/>
@@ -8688,7 +8709,7 @@
       </c>
     </row>
     <row r="24" spans="1:6" ht="31.2">
-      <c r="A24" s="266">
+      <c r="A24" s="216">
         <v>22</v>
       </c>
       <c r="B24" s="210" t="s">
@@ -8706,7 +8727,7 @@
       </c>
     </row>
     <row r="25" spans="1:6" ht="31.2">
-      <c r="A25" s="266">
+      <c r="A25" s="216">
         <v>23</v>
       </c>
       <c r="B25" s="210" t="s">
@@ -8721,27 +8742,27 @@
         <v>126</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
-      <c r="A26" s="266">
+    <row r="26" spans="1:6" s="220" customFormat="1">
+      <c r="A26" s="218">
         <v>24</v>
       </c>
-      <c r="B26" s="262" t="s">
+      <c r="B26" s="266" t="s">
         <v>129</v>
       </c>
-      <c r="C26" s="208"/>
-      <c r="D26" s="209" t="s">
+      <c r="C26" s="219"/>
+      <c r="D26" s="219" t="s">
         <v>130</v>
       </c>
-      <c r="E26" s="208"/>
-      <c r="F26" s="208" t="s">
+      <c r="E26" s="219"/>
+      <c r="F26" s="219" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="266">
+      <c r="A27" s="216">
         <v>25</v>
       </c>
-      <c r="B27" s="263"/>
+      <c r="B27" s="267"/>
       <c r="C27" s="208"/>
       <c r="D27" s="209" t="s">
         <v>127</v>
@@ -8752,10 +8773,10 @@
       </c>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="266">
+      <c r="A28" s="216">
         <v>26</v>
       </c>
-      <c r="B28" s="264" t="s">
+      <c r="B28" s="268" t="s">
         <v>184</v>
       </c>
       <c r="C28" s="208"/>
@@ -8768,10 +8789,10 @@
       </c>
     </row>
     <row r="29" spans="1:6">
-      <c r="A29" s="266">
+      <c r="A29" s="216">
         <v>27</v>
       </c>
-      <c r="B29" s="265"/>
+      <c r="B29" s="269"/>
       <c r="C29" s="208"/>
       <c r="D29" s="208" t="s">
         <v>186</v>
@@ -8782,10 +8803,10 @@
       </c>
     </row>
     <row r="30" spans="1:6" ht="31.2">
-      <c r="A30" s="266">
+      <c r="A30" s="216">
         <v>28</v>
       </c>
-      <c r="B30" s="216" t="s">
+      <c r="B30" s="215" t="s">
         <v>187</v>
       </c>
       <c r="C30" s="208"/>
@@ -8798,11 +8819,11 @@
       </c>
     </row>
     <row r="31" spans="1:6">
-      <c r="B31" s="213"/>
-      <c r="C31" s="215"/>
-      <c r="D31" s="214"/>
-      <c r="E31" s="214"/>
-      <c r="F31" s="214"/>
+      <c r="B31" s="212"/>
+      <c r="C31" s="214"/>
+      <c r="D31" s="213"/>
+      <c r="E31" s="213"/>
+      <c r="F31" s="213"/>
     </row>
     <row r="32" spans="1:6">
       <c r="B32" s="208" t="s">

</xml_diff>